<commit_message>
Document onboarding agent rules
</commit_message>
<xml_diff>
--- a/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
+++ b/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Target Fields'!$A$1:$S$151</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Template Fields'!$A$1:$H$180</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Evidence'!$A$1:$D$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$J$234</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$J$232</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Output Objects'!$A$1:$E$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Missing Important Fields'!$A$1:$E$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'SAP Investigation Log'!$A$1:$E$10</definedName>
@@ -244,8 +244,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:J234" headerRowCount="1">
-  <autoFilter ref="A1:J234"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:J232" headerRowCount="1">
+  <autoFilter ref="A1:J232"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Field"/>
     <tableColumn id="2" name="Object"/>
@@ -17045,36 +17045,32 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="4" t="inlineStr">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>WarehouseStockOnHand</t>
         </is>
       </c>
-      <c r="B63" s="4" t="inlineStr">
+      <c r="B63" s="5" t="inlineStr">
         <is>
           <t>inventoryType</t>
         </is>
       </c>
-      <c r="C63" s="4" t="inlineStr">
+      <c r="C63" s="5" t="inlineStr">
         <is>
           <t>Enum&lt;String&gt;</t>
         </is>
       </c>
-      <c r="D63" s="4" t="inlineStr"/>
-      <c r="E63" s="4" t="inlineStr">
-        <is>
-          <t>Not available in checked source</t>
-        </is>
-      </c>
-      <c r="F63" s="4" t="inlineStr"/>
-      <c r="G63" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H63" s="4" t="inlineStr">
-        <is>
-          <t>Left blank. SAP OITW live stock metrics do not identify Planning V2 good/bad inventory type; do not infer from warehouse names.</t>
+      <c r="D63" s="5" t="inlineStr"/>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Out of v1 scope</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr"/>
+      <c r="G63" s="5" t="inlineStr"/>
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>Not needed for CoCre8 MVP; no confirmed good/bad inventory type source in SAP stock metrics.</t>
         </is>
       </c>
     </row>
@@ -17193,70 +17189,70 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="4" t="inlineStr">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>WarehouseStockOnHand</t>
         </is>
       </c>
-      <c r="B67" s="4" t="inlineStr">
+      <c r="B67" s="5" t="inlineStr">
         <is>
           <t>quantityOutbound</t>
         </is>
       </c>
-      <c r="C67" s="4" t="inlineStr">
+      <c r="C67" s="5" t="inlineStr">
         <is>
           <t>Double</t>
         </is>
       </c>
-      <c r="D67" s="4" t="inlineStr"/>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>Not available in checked source</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr"/>
-      <c r="G67" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H67" s="4" t="inlineStr">
-        <is>
-          <t>Left blank. SAP OITW has IsCommited, which is already mapped to quantityAllocated; no separate outbound quantity was found in the live stock metrics.</t>
+      <c r="D67" s="5" t="inlineStr"/>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>Out of v1 scope</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr"/>
+      <c r="G67" s="5" t="inlineStr"/>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>Not needed for CoCre8 MVP; CoCre8 issues stock directly and no separate outbound stock source was found.</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="4" t="inlineStr">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>WarehouseStockOnHand</t>
         </is>
       </c>
-      <c r="B68" s="4" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>uniqueId</t>
         </is>
       </c>
-      <c r="C68" s="4" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
         <is>
           <t>Integer</t>
         </is>
       </c>
-      <c r="D68" s="4" t="inlineStr"/>
-      <c r="E68" s="4" t="inlineStr">
-        <is>
-          <t>Investigate source</t>
-        </is>
-      </c>
-      <c r="F68" s="4" t="inlineStr"/>
-      <c r="G68" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H68" s="4" t="inlineStr">
-        <is>
-          <t>Left blank. Template expects an integer technical id, but no confirmed source/key rule has been provided.</t>
+      <c r="D68" s="2" t="inlineStr"/>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Derived stable integer from MinStock-style RowKey part|SPLMaster|warehouse</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -20327,40 +20323,36 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="2" t="inlineStr">
+      <c r="A158" s="3" t="inlineStr">
         <is>
           <t>PurchaseOrders</t>
         </is>
       </c>
-      <c r="B158" s="2" t="inlineStr">
+      <c r="B158" s="3" t="inlineStr">
         <is>
           <t>demandStatus</t>
         </is>
       </c>
-      <c r="C158" s="2" t="inlineStr">
+      <c r="C158" s="3" t="inlineStr">
         <is>
           <t>Enum&lt;String&gt;</t>
         </is>
       </c>
-      <c r="D158" s="2" t="inlineStr"/>
-      <c r="E158" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="F158" s="2" t="inlineStr">
-        <is>
-          <t>CoCre8 HelpDesk issue tracker:ReplenishStatus when exact PO plus exact part/SPL Master evidence exists</t>
-        </is>
-      </c>
-      <c r="G158" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H158" s="2" t="inlineStr">
-        <is>
-          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
+      <c r="D158" s="3" t="inlineStr"/>
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t>Review required</t>
+        </is>
+      </c>
+      <c r="F158" s="3" t="inlineStr"/>
+      <c r="G158" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H158" s="3" t="inlineStr">
+        <is>
+          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.DocNum and part/SPL Master evidence also matches; current export needs reconciliation.</t>
         </is>
       </c>
     </row>
@@ -21447,7 +21439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J234"/>
+  <dimension ref="A1:J232"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -28625,12 +28617,12 @@
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>inventoryType</t>
+          <t>personId</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
         <is>
-          <t>WarehouseStockOnHand</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C150" s="4" t="inlineStr">
@@ -28641,12 +28633,12 @@
       <c r="D150" s="4" t="inlineStr"/>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>Not available in checked source</t>
+          <t>Investigate SAP first</t>
         </is>
       </c>
       <c r="F150" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseStockOnHand.inventoryType?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.personId?</t>
         </is>
       </c>
       <c r="G150" s="4" t="inlineStr">
@@ -28658,19 +28650,19 @@
       <c r="I150" s="4" t="inlineStr"/>
       <c r="J150" s="4" t="inlineStr">
         <is>
-          <t>Left blank. SAP OITW live stock metrics do not identify Planning V2 good/bad inventory type; do not infer from warehouse names.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>quantityOutbound</t>
+          <t>role</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>WarehouseStockOnHand</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
@@ -28681,12 +28673,12 @@
       <c r="D151" s="4" t="inlineStr"/>
       <c r="E151" s="4" t="inlineStr">
         <is>
-          <t>Not available in checked source</t>
+          <t>Investigate SAP first</t>
         </is>
       </c>
       <c r="F151" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseStockOnHand.quantityOutbound?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.role?</t>
         </is>
       </c>
       <c r="G151" s="4" t="inlineStr">
@@ -28698,19 +28690,19 @@
       <c r="I151" s="4" t="inlineStr"/>
       <c r="J151" s="4" t="inlineStr">
         <is>
-          <t>Left blank. SAP OITW has IsCommited, which is already mapped to quantityAllocated; no separate outbound quantity was found in the live stock metrics.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>uniqueId</t>
+          <t>addressId</t>
         </is>
       </c>
       <c r="B152" s="4" t="inlineStr">
         <is>
-          <t>WarehouseStockOnHand</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C152" s="4" t="inlineStr">
@@ -28721,12 +28713,12 @@
       <c r="D152" s="4" t="inlineStr"/>
       <c r="E152" s="4" t="inlineStr">
         <is>
-          <t>Investigate source</t>
+          <t>Investigate SAP first</t>
         </is>
       </c>
       <c r="F152" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseStockOnHand.uniqueId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.addressId?</t>
         </is>
       </c>
       <c r="G152" s="4" t="inlineStr">
@@ -28738,14 +28730,14 @@
       <c r="I152" s="4" t="inlineStr"/>
       <c r="J152" s="4" t="inlineStr">
         <is>
-          <t>Left blank. Template expects an integer technical id, but no confirmed source/key rule has been provided.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>personId</t>
+          <t>nodeId</t>
         </is>
       </c>
       <c r="B153" s="4" t="inlineStr">
@@ -28766,7 +28758,7 @@
       </c>
       <c r="F153" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.personId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.nodeId?</t>
         </is>
       </c>
       <c r="G153" s="4" t="inlineStr">
@@ -28785,7 +28777,7 @@
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>firstName</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
@@ -28806,7 +28798,7 @@
       </c>
       <c r="F154" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.role?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.firstName?</t>
         </is>
       </c>
       <c r="G154" s="4" t="inlineStr">
@@ -28825,7 +28817,7 @@
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>addressId</t>
+          <t>middleName</t>
         </is>
       </c>
       <c r="B155" s="4" t="inlineStr">
@@ -28846,7 +28838,7 @@
       </c>
       <c r="F155" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.addressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.middleName?</t>
         </is>
       </c>
       <c r="G155" s="4" t="inlineStr">
@@ -28865,7 +28857,7 @@
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>nodeId</t>
+          <t>surname</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
@@ -28886,7 +28878,7 @@
       </c>
       <c r="F156" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.nodeId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.surname?</t>
         </is>
       </c>
       <c r="G156" s="4" t="inlineStr">
@@ -28905,7 +28897,7 @@
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>firstName</t>
+          <t>isActive</t>
         </is>
       </c>
       <c r="B157" s="4" t="inlineStr">
@@ -28926,7 +28918,7 @@
       </c>
       <c r="F157" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.firstName?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.isActive?</t>
         </is>
       </c>
       <c r="G157" s="4" t="inlineStr">
@@ -28945,7 +28937,7 @@
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>middleName</t>
+          <t>telephoneNumber</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
@@ -28966,7 +28958,7 @@
       </c>
       <c r="F158" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.middleName?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.telephoneNumber?</t>
         </is>
       </c>
       <c r="G158" s="4" t="inlineStr">
@@ -28985,12 +28977,12 @@
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>surname</t>
+          <t>customerCompanyCode</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C159" s="4" t="inlineStr">
@@ -29006,7 +28998,7 @@
       </c>
       <c r="F159" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.surname?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.customerCompanyCode?</t>
         </is>
       </c>
       <c r="G159" s="4" t="inlineStr">
@@ -29025,12 +29017,12 @@
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>isActive</t>
+          <t>orderType</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C160" s="4" t="inlineStr">
@@ -29046,7 +29038,7 @@
       </c>
       <c r="F160" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.isActive?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderType?</t>
         </is>
       </c>
       <c r="G160" s="4" t="inlineStr">
@@ -29065,12 +29057,12 @@
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>telephoneNumber</t>
+          <t>orderStatus</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C161" s="4" t="inlineStr">
@@ -29086,7 +29078,7 @@
       </c>
       <c r="F161" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.telephoneNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStatus?</t>
         </is>
       </c>
       <c r="G161" s="4" t="inlineStr">
@@ -29105,7 +29097,7 @@
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>customerCompanyCode</t>
+          <t>orderStartDatetime</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
@@ -29126,7 +29118,7 @@
       </c>
       <c r="F162" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.customerCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStartDatetime?</t>
         </is>
       </c>
       <c r="G162" s="4" t="inlineStr">
@@ -29145,7 +29137,7 @@
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>orderType</t>
+          <t>requestTicketDateTime</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
@@ -29166,7 +29158,7 @@
       </c>
       <c r="F163" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderType?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.requestTicketDateTime?</t>
         </is>
       </c>
       <c r="G163" s="4" t="inlineStr">
@@ -29185,7 +29177,7 @@
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>orderStatus</t>
+          <t>siteCompanyCode</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
@@ -29206,7 +29198,7 @@
       </c>
       <c r="F164" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.siteCompanyCode?</t>
         </is>
       </c>
       <c r="G164" s="4" t="inlineStr">
@@ -29225,7 +29217,7 @@
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t>orderStartDatetime</t>
+          <t>assignedPersonCode</t>
         </is>
       </c>
       <c r="B165" s="4" t="inlineStr">
@@ -29246,7 +29238,7 @@
       </c>
       <c r="F165" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStartDatetime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.assignedPersonCode?</t>
         </is>
       </c>
       <c r="G165" s="4" t="inlineStr">
@@ -29265,7 +29257,7 @@
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>requestTicketDateTime</t>
+          <t>resolvedDateTime</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
@@ -29286,7 +29278,7 @@
       </c>
       <c r="F166" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.requestTicketDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.resolvedDateTime?</t>
         </is>
       </c>
       <c r="G166" s="4" t="inlineStr">
@@ -29305,7 +29297,7 @@
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>siteCompanyCode</t>
+          <t>serialNumber</t>
         </is>
       </c>
       <c r="B167" s="4" t="inlineStr">
@@ -29326,7 +29318,7 @@
       </c>
       <c r="F167" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.siteCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.serialNumber?</t>
         </is>
       </c>
       <c r="G167" s="4" t="inlineStr">
@@ -29345,7 +29337,7 @@
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>assignedPersonCode</t>
+          <t>relCompanyId</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
@@ -29366,7 +29358,7 @@
       </c>
       <c r="F168" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.assignedPersonCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.relCompanyId?</t>
         </is>
       </c>
       <c r="G168" s="4" t="inlineStr">
@@ -29385,7 +29377,7 @@
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>resolvedDateTime</t>
+          <t>deviceSerialNumber</t>
         </is>
       </c>
       <c r="B169" s="4" t="inlineStr">
@@ -29406,7 +29398,7 @@
       </c>
       <c r="F169" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.resolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.deviceSerialNumber?</t>
         </is>
       </c>
       <c r="G169" s="4" t="inlineStr">
@@ -29425,12 +29417,12 @@
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>serialNumber</t>
+          <t>orderNumber</t>
         </is>
       </c>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C170" s="4" t="inlineStr">
@@ -29446,7 +29438,7 @@
       </c>
       <c r="F170" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.serialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.orderNumber?</t>
         </is>
       </c>
       <c r="G170" s="4" t="inlineStr">
@@ -29465,12 +29457,12 @@
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>relCompanyId</t>
+          <t>location</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
@@ -29486,7 +29478,7 @@
       </c>
       <c r="F171" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.relCompanyId?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.location?</t>
         </is>
       </c>
       <c r="G171" s="4" t="inlineStr">
@@ -29505,12 +29497,12 @@
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>deviceSerialNumber</t>
+          <t>eta</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C172" s="4" t="inlineStr">
@@ -29526,7 +29518,7 @@
       </c>
       <c r="F172" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.deviceSerialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.eta?</t>
         </is>
       </c>
       <c r="G172" s="4" t="inlineStr">
@@ -29545,7 +29537,7 @@
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>orderNumber</t>
+          <t>actualEta</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
@@ -29566,7 +29558,7 @@
       </c>
       <c r="F173" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.orderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualEta?</t>
         </is>
       </c>
       <c r="G173" s="4" t="inlineStr">
@@ -29585,7 +29577,7 @@
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>actualResolveDateTime</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
@@ -29606,7 +29598,7 @@
       </c>
       <c r="F174" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.location?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualResolveDateTime?</t>
         </is>
       </c>
       <c r="G174" s="4" t="inlineStr">
@@ -29625,7 +29617,7 @@
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>eta</t>
+          <t>recallDateTime</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
@@ -29646,7 +29638,7 @@
       </c>
       <c r="F175" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.eta?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.recallDateTime?</t>
         </is>
       </c>
       <c r="G175" s="4" t="inlineStr">
@@ -29665,7 +29657,7 @@
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>actualEta</t>
+          <t>actualRecallDateTime</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
@@ -29686,7 +29678,7 @@
       </c>
       <c r="F176" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualEta?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualRecallDateTime?</t>
         </is>
       </c>
       <c r="G176" s="4" t="inlineStr">
@@ -29705,7 +29697,7 @@
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>actualResolveDateTime</t>
+          <t>slaEtaClock</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
@@ -29726,7 +29718,7 @@
       </c>
       <c r="F177" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualResolveDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaClock?</t>
         </is>
       </c>
       <c r="G177" s="4" t="inlineStr">
@@ -29745,7 +29737,7 @@
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>recallDateTime</t>
+          <t>slaResolveClock</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
@@ -29766,7 +29758,7 @@
       </c>
       <c r="F178" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.recallDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveClock?</t>
         </is>
       </c>
       <c r="G178" s="4" t="inlineStr">
@@ -29785,7 +29777,7 @@
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>actualRecallDateTime</t>
+          <t>slaFailureCode</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
@@ -29806,7 +29798,7 @@
       </c>
       <c r="F179" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualRecallDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaFailureCode?</t>
         </is>
       </c>
       <c r="G179" s="4" t="inlineStr">
@@ -29825,7 +29817,7 @@
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>slaEtaClock</t>
+          <t>slaEtaHit</t>
         </is>
       </c>
       <c r="B180" s="4" t="inlineStr">
@@ -29846,7 +29838,7 @@
       </c>
       <c r="F180" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaClock?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaHit?</t>
         </is>
       </c>
       <c r="G180" s="4" t="inlineStr">
@@ -29865,7 +29857,7 @@
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>slaResolveClock</t>
+          <t>slaResolvedDateTime</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
@@ -29886,7 +29878,7 @@
       </c>
       <c r="F181" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveClock?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolvedDateTime?</t>
         </is>
       </c>
       <c r="G181" s="4" t="inlineStr">
@@ -29905,12 +29897,12 @@
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>slaFailureCode</t>
+          <t>orderNumber</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C182" s="4" t="inlineStr">
@@ -29926,7 +29918,7 @@
       </c>
       <c r="F182" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaFailureCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderNumber?</t>
         </is>
       </c>
       <c r="G182" s="4" t="inlineStr">
@@ -29945,12 +29937,12 @@
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>slaEtaHit</t>
+          <t>requestId</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C183" s="4" t="inlineStr">
@@ -29966,7 +29958,7 @@
       </c>
       <c r="F183" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaHit?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.requestId?</t>
         </is>
       </c>
       <c r="G183" s="4" t="inlineStr">
@@ -29985,12 +29977,12 @@
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>slaResolvedDateTime</t>
+          <t>customerCompanyCode</t>
         </is>
       </c>
       <c r="B184" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C184" s="4" t="inlineStr">
@@ -30006,7 +29998,7 @@
       </c>
       <c r="F184" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.customerCompanyCode?</t>
         </is>
       </c>
       <c r="G184" s="4" t="inlineStr">
@@ -30025,7 +30017,7 @@
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>orderNumber</t>
+          <t>orderStatus</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
@@ -30046,7 +30038,7 @@
       </c>
       <c r="F185" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStatus?</t>
         </is>
       </c>
       <c r="G185" s="4" t="inlineStr">
@@ -30065,7 +30057,7 @@
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>requestId</t>
+          <t>orderStartDatetime</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
@@ -30086,7 +30078,7 @@
       </c>
       <c r="F186" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.requestId?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStartDatetime?</t>
         </is>
       </c>
       <c r="G186" s="4" t="inlineStr">
@@ -30105,7 +30097,7 @@
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>customerCompanyCode</t>
+          <t>siteCompanyCode</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
@@ -30126,7 +30118,7 @@
       </c>
       <c r="F187" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.customerCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.siteCompanyCode?</t>
         </is>
       </c>
       <c r="G187" s="4" t="inlineStr">
@@ -30145,7 +30137,7 @@
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>orderStatus</t>
+          <t>repairType</t>
         </is>
       </c>
       <c r="B188" s="4" t="inlineStr">
@@ -30166,7 +30158,7 @@
       </c>
       <c r="F188" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairType?</t>
         </is>
       </c>
       <c r="G188" s="4" t="inlineStr">
@@ -30185,7 +30177,7 @@
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>orderStartDatetime</t>
+          <t>partsOrderDateTime</t>
         </is>
       </c>
       <c r="B189" s="4" t="inlineStr">
@@ -30206,7 +30198,7 @@
       </c>
       <c r="F189" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStartDatetime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsOrderDateTime?</t>
         </is>
       </c>
       <c r="G189" s="4" t="inlineStr">
@@ -30225,7 +30217,7 @@
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>siteCompanyCode</t>
+          <t>partsReceivedDateTime</t>
         </is>
       </c>
       <c r="B190" s="4" t="inlineStr">
@@ -30246,7 +30238,7 @@
       </c>
       <c r="F190" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.siteCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsReceivedDateTime?</t>
         </is>
       </c>
       <c r="G190" s="4" t="inlineStr">
@@ -30265,7 +30257,7 @@
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>repairType</t>
+          <t>repairCode</t>
         </is>
       </c>
       <c r="B191" s="4" t="inlineStr">
@@ -30286,7 +30278,7 @@
       </c>
       <c r="F191" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairType?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCode?</t>
         </is>
       </c>
       <c r="G191" s="4" t="inlineStr">
@@ -30305,7 +30297,7 @@
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>partsOrderDateTime</t>
+          <t>repairCompany</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
@@ -30326,7 +30318,7 @@
       </c>
       <c r="F192" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsOrderDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCompany?</t>
         </is>
       </c>
       <c r="G192" s="4" t="inlineStr">
@@ -30345,7 +30337,7 @@
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>partsReceivedDateTime</t>
+          <t>raStatus</t>
         </is>
       </c>
       <c r="B193" s="4" t="inlineStr">
@@ -30366,7 +30358,7 @@
       </c>
       <c r="F193" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsReceivedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.raStatus?</t>
         </is>
       </c>
       <c r="G193" s="4" t="inlineStr">
@@ -30385,7 +30377,7 @@
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>repairCode</t>
+          <t>Warehouse</t>
         </is>
       </c>
       <c r="B194" s="4" t="inlineStr">
@@ -30406,7 +30398,7 @@
       </c>
       <c r="F194" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.Warehouse?</t>
         </is>
       </c>
       <c r="G194" s="4" t="inlineStr">
@@ -30425,7 +30417,7 @@
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>repairCompany</t>
+          <t>assignedPerson</t>
         </is>
       </c>
       <c r="B195" s="4" t="inlineStr">
@@ -30446,7 +30438,7 @@
       </c>
       <c r="F195" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCompany?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.assignedPerson?</t>
         </is>
       </c>
       <c r="G195" s="4" t="inlineStr">
@@ -30465,7 +30457,7 @@
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>raStatus</t>
+          <t>orderedPartId</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
@@ -30486,7 +30478,7 @@
       </c>
       <c r="F196" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.raStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderedPartId?</t>
         </is>
       </c>
       <c r="G196" s="4" t="inlineStr">
@@ -30505,7 +30497,7 @@
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>Warehouse</t>
+          <t>actualPartId</t>
         </is>
       </c>
       <c r="B197" s="4" t="inlineStr">
@@ -30526,7 +30518,7 @@
       </c>
       <c r="F197" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.Warehouse?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.actualPartId?</t>
         </is>
       </c>
       <c r="G197" s="4" t="inlineStr">
@@ -30545,7 +30537,7 @@
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>assignedPerson</t>
+          <t>resolvedDateTime</t>
         </is>
       </c>
       <c r="B198" s="4" t="inlineStr">
@@ -30566,7 +30558,7 @@
       </c>
       <c r="F198" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.assignedPerson?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.resolvedDateTime?</t>
         </is>
       </c>
       <c r="G198" s="4" t="inlineStr">
@@ -30585,7 +30577,7 @@
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>orderedPartId</t>
+          <t>serialNumber</t>
         </is>
       </c>
       <c r="B199" s="4" t="inlineStr">
@@ -30606,7 +30598,7 @@
       </c>
       <c r="F199" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderedPartId?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.serialNumber?</t>
         </is>
       </c>
       <c r="G199" s="4" t="inlineStr">
@@ -30625,7 +30617,7 @@
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>actualPartId</t>
+          <t>quantityUsed</t>
         </is>
       </c>
       <c r="B200" s="4" t="inlineStr">
@@ -30646,7 +30638,7 @@
       </c>
       <c r="F200" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.actualPartId?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.quantityUsed?</t>
         </is>
       </c>
       <c r="G200" s="4" t="inlineStr">
@@ -30665,7 +30657,7 @@
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t>resolvedDateTime</t>
+          <t>relCompanyId</t>
         </is>
       </c>
       <c r="B201" s="4" t="inlineStr">
@@ -30686,7 +30678,7 @@
       </c>
       <c r="F201" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.resolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.relCompanyId?</t>
         </is>
       </c>
       <c r="G201" s="4" t="inlineStr">
@@ -30705,7 +30697,7 @@
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>serialNumber</t>
+          <t>partsUsedDateTime</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
@@ -30726,7 +30718,7 @@
       </c>
       <c r="F202" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.serialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsUsedDateTime?</t>
         </is>
       </c>
       <c r="G202" s="4" t="inlineStr">
@@ -30745,7 +30737,7 @@
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>quantityUsed</t>
+          <t>deviceSerialNumber</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
@@ -30766,7 +30758,7 @@
       </c>
       <c r="F203" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.quantityUsed?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.deviceSerialNumber?</t>
         </is>
       </c>
       <c r="G203" s="4" t="inlineStr">
@@ -30785,12 +30777,12 @@
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>relCompanyId</t>
+          <t>partCode</t>
         </is>
       </c>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>PartCost</t>
         </is>
       </c>
       <c r="C204" s="4" t="inlineStr">
@@ -30806,7 +30798,7 @@
       </c>
       <c r="F204" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.relCompanyId?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.partCode?</t>
         </is>
       </c>
       <c r="G204" s="4" t="inlineStr">
@@ -30825,12 +30817,12 @@
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>partsUsedDateTime</t>
+          <t>cost</t>
         </is>
       </c>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>PartCost</t>
         </is>
       </c>
       <c r="C205" s="4" t="inlineStr">
@@ -30846,7 +30838,7 @@
       </c>
       <c r="F205" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsUsedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.cost?</t>
         </is>
       </c>
       <c r="G205" s="4" t="inlineStr">
@@ -30865,12 +30857,12 @@
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
         <is>
-          <t>deviceSerialNumber</t>
+          <t>currencyCode</t>
         </is>
       </c>
       <c r="B206" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>PartCost</t>
         </is>
       </c>
       <c r="C206" s="4" t="inlineStr">
@@ -30886,7 +30878,7 @@
       </c>
       <c r="F206" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.deviceSerialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.currencyCode?</t>
         </is>
       </c>
       <c r="G206" s="4" t="inlineStr">
@@ -30905,7 +30897,7 @@
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>partCode</t>
+          <t>averageCost</t>
         </is>
       </c>
       <c r="B207" s="4" t="inlineStr">
@@ -30926,7 +30918,7 @@
       </c>
       <c r="F207" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.partCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.averageCost?</t>
         </is>
       </c>
       <c r="G207" s="4" t="inlineStr">
@@ -30945,12 +30937,12 @@
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>partCode</t>
         </is>
       </c>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C208" s="4" t="inlineStr">
@@ -30966,7 +30958,7 @@
       </c>
       <c r="F208" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.cost?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
         </is>
       </c>
       <c r="G208" s="4" t="inlineStr">
@@ -30985,12 +30977,12 @@
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t>currencyCode</t>
+          <t>modelCode</t>
         </is>
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C209" s="4" t="inlineStr">
@@ -31006,7 +30998,7 @@
       </c>
       <c r="F209" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.currencyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
         </is>
       </c>
       <c r="G209" s="4" t="inlineStr">
@@ -31025,12 +31017,12 @@
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
         <is>
-          <t>averageCost</t>
+          <t>modelDescription</t>
         </is>
       </c>
       <c r="B210" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C210" s="4" t="inlineStr">
@@ -31046,7 +31038,7 @@
       </c>
       <c r="F210" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.averageCost?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
         </is>
       </c>
       <c r="G210" s="4" t="inlineStr">
@@ -31065,12 +31057,12 @@
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
         <is>
-          <t>partCode</t>
+          <t>inventoryTransferImoId</t>
         </is>
       </c>
       <c r="B211" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C211" s="4" t="inlineStr">
@@ -31086,7 +31078,7 @@
       </c>
       <c r="F211" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.inventoryTransferImoId?</t>
         </is>
       </c>
       <c r="G211" s="4" t="inlineStr">
@@ -31105,12 +31097,12 @@
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
         <is>
-          <t>modelCode</t>
+          <t>createdDateTime</t>
         </is>
       </c>
       <c r="B212" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C212" s="4" t="inlineStr">
@@ -31126,7 +31118,7 @@
       </c>
       <c r="F212" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.createdDateTime?</t>
         </is>
       </c>
       <c r="G212" s="4" t="inlineStr">
@@ -31145,12 +31137,12 @@
     <row r="213">
       <c r="A213" s="4" t="inlineStr">
         <is>
-          <t>modelDescription</t>
+          <t>completedDateTime</t>
         </is>
       </c>
       <c r="B213" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C213" s="4" t="inlineStr">
@@ -31166,7 +31158,7 @@
       </c>
       <c r="F213" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.completedDateTime?</t>
         </is>
       </c>
       <c r="G213" s="4" t="inlineStr">
@@ -31185,7 +31177,7 @@
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
         <is>
-          <t>inventoryTransferImoId</t>
+          <t>fromWarehouseId</t>
         </is>
       </c>
       <c r="B214" s="4" t="inlineStr">
@@ -31206,7 +31198,7 @@
       </c>
       <c r="F214" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.inventoryTransferImoId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.fromWarehouseId?</t>
         </is>
       </c>
       <c r="G214" s="4" t="inlineStr">
@@ -31225,7 +31217,7 @@
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
         <is>
-          <t>createdDateTime</t>
+          <t>toWarehouseId</t>
         </is>
       </c>
       <c r="B215" s="4" t="inlineStr">
@@ -31246,7 +31238,7 @@
       </c>
       <c r="F215" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.createdDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.toWarehouseId?</t>
         </is>
       </c>
       <c r="G215" s="4" t="inlineStr">
@@ -31265,7 +31257,7 @@
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
         <is>
-          <t>completedDateTime</t>
+          <t>demandStatus</t>
         </is>
       </c>
       <c r="B216" s="4" t="inlineStr">
@@ -31286,7 +31278,7 @@
       </c>
       <c r="F216" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.completedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.demandStatus?</t>
         </is>
       </c>
       <c r="G216" s="4" t="inlineStr">
@@ -31305,7 +31297,7 @@
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t>fromWarehouseId</t>
+          <t>orderStatusIsClosed</t>
         </is>
       </c>
       <c r="B217" s="4" t="inlineStr">
@@ -31326,7 +31318,7 @@
       </c>
       <c r="F217" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.fromWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.orderStatusIsClosed?</t>
         </is>
       </c>
       <c r="G217" s="4" t="inlineStr">
@@ -31345,7 +31337,7 @@
     <row r="218">
       <c r="A218" s="4" t="inlineStr">
         <is>
-          <t>toWarehouseId</t>
+          <t>movementType</t>
         </is>
       </c>
       <c r="B218" s="4" t="inlineStr">
@@ -31366,7 +31358,7 @@
       </c>
       <c r="F218" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.toWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
         </is>
       </c>
       <c r="G218" s="4" t="inlineStr">
@@ -31385,7 +31377,7 @@
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t>demandStatus</t>
+          <t>addressId</t>
         </is>
       </c>
       <c r="B219" s="4" t="inlineStr">
@@ -31406,7 +31398,7 @@
       </c>
       <c r="F219" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.demandStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
         </is>
       </c>
       <c r="G219" s="4" t="inlineStr">
@@ -31425,7 +31417,7 @@
     <row r="220">
       <c r="A220" s="4" t="inlineStr">
         <is>
-          <t>orderStatusIsClosed</t>
+          <t>isResolved</t>
         </is>
       </c>
       <c r="B220" s="4" t="inlineStr">
@@ -31446,7 +31438,7 @@
       </c>
       <c r="F220" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.orderStatusIsClosed?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.isResolved?</t>
         </is>
       </c>
       <c r="G220" s="4" t="inlineStr">
@@ -31465,7 +31457,7 @@
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
         <is>
-          <t>movementType</t>
+          <t>partNumber</t>
         </is>
       </c>
       <c r="B221" s="4" t="inlineStr">
@@ -31486,7 +31478,7 @@
       </c>
       <c r="F221" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.partNumber?</t>
         </is>
       </c>
       <c r="G221" s="4" t="inlineStr">
@@ -31505,7 +31497,7 @@
     <row r="222">
       <c r="A222" s="4" t="inlineStr">
         <is>
-          <t>addressId</t>
+          <t>quantity</t>
         </is>
       </c>
       <c r="B222" s="4" t="inlineStr">
@@ -31526,7 +31518,7 @@
       </c>
       <c r="F222" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.quantity?</t>
         </is>
       </c>
       <c r="G222" s="4" t="inlineStr">
@@ -31545,7 +31537,7 @@
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
         <is>
-          <t>isResolved</t>
+          <t>shipListCode</t>
         </is>
       </c>
       <c r="B223" s="4" t="inlineStr">
@@ -31566,7 +31558,7 @@
       </c>
       <c r="F223" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.isResolved?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
         </is>
       </c>
       <c r="G223" s="4" t="inlineStr">
@@ -31583,54 +31575,54 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="4" t="inlineStr">
-        <is>
-          <t>partNumber</t>
-        </is>
-      </c>
-      <c r="B224" s="4" t="inlineStr">
-        <is>
-          <t>InventoryTransfers</t>
-        </is>
-      </c>
-      <c r="C224" s="4" t="inlineStr">
+      <c r="A224" s="3" t="inlineStr">
+        <is>
+          <t>demandStatus</t>
+        </is>
+      </c>
+      <c r="B224" s="3" t="inlineStr">
+        <is>
+          <t>PurchaseOrders</t>
+        </is>
+      </c>
+      <c r="C224" s="3" t="inlineStr">
         <is>
           <t>Planning V2 template</t>
         </is>
       </c>
-      <c r="D224" s="4" t="inlineStr"/>
-      <c r="E224" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F224" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.partNumber?</t>
-        </is>
-      </c>
-      <c r="G224" s="4" t="inlineStr">
+      <c r="D224" s="3" t="inlineStr"/>
+      <c r="E224" s="3" t="inlineStr">
+        <is>
+          <t>Review required</t>
+        </is>
+      </c>
+      <c r="F224" s="3" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
+        </is>
+      </c>
+      <c r="G224" s="3" t="inlineStr">
         <is>
           <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
         </is>
       </c>
-      <c r="H224" s="4" t="inlineStr"/>
-      <c r="I224" s="4" t="inlineStr"/>
-      <c r="J224" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="H224" s="3" t="inlineStr"/>
+      <c r="I224" s="3" t="inlineStr"/>
+      <c r="J224" s="3" t="inlineStr">
+        <is>
+          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.DocNum and part/SPL Master evidence also matches; current export needs reconciliation.</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="4" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>partTypeCode</t>
         </is>
       </c>
       <c r="B225" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C225" s="4" t="inlineStr">
@@ -31646,7 +31638,7 @@
       </c>
       <c r="F225" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.quantity?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeCode?</t>
         </is>
       </c>
       <c r="G225" s="4" t="inlineStr">
@@ -31665,12 +31657,12 @@
     <row r="226">
       <c r="A226" s="4" t="inlineStr">
         <is>
-          <t>shipListCode</t>
+          <t>description</t>
         </is>
       </c>
       <c r="B226" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C226" s="4" t="inlineStr">
@@ -31686,7 +31678,7 @@
       </c>
       <c r="F226" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.description?</t>
         </is>
       </c>
       <c r="G226" s="4" t="inlineStr">
@@ -31705,12 +31697,12 @@
     <row r="227">
       <c r="A227" s="4" t="inlineStr">
         <is>
-          <t>partTypeCode</t>
+          <t>partNumber</t>
         </is>
       </c>
       <c r="B227" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C227" s="4" t="inlineStr">
@@ -31726,7 +31718,7 @@
       </c>
       <c r="F227" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
         </is>
       </c>
       <c r="G227" s="4" t="inlineStr">
@@ -31745,12 +31737,12 @@
     <row r="228">
       <c r="A228" s="4" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>unitOfMeasure</t>
         </is>
       </c>
       <c r="B228" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C228" s="4" t="inlineStr">
@@ -31766,7 +31758,7 @@
       </c>
       <c r="F228" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.description?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
         </is>
       </c>
       <c r="G228" s="4" t="inlineStr">
@@ -31785,7 +31777,7 @@
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
         <is>
-          <t>partNumber</t>
+          <t>yield</t>
         </is>
       </c>
       <c r="B229" s="4" t="inlineStr">
@@ -31806,7 +31798,7 @@
       </c>
       <c r="F229" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
         </is>
       </c>
       <c r="G229" s="4" t="inlineStr">
@@ -31825,12 +31817,12 @@
     <row r="230">
       <c r="A230" s="4" t="inlineStr">
         <is>
-          <t>unitOfMeasure</t>
+          <t>warehouseId</t>
         </is>
       </c>
       <c r="B230" s="4" t="inlineStr">
         <is>
-          <t>Yields</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C230" s="4" t="inlineStr">
@@ -31846,7 +31838,7 @@
       </c>
       <c r="F230" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.warehouseId?</t>
         </is>
       </c>
       <c r="G230" s="4" t="inlineStr">
@@ -31865,12 +31857,12 @@
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
         <is>
-          <t>yield</t>
+          <t>exclusionType</t>
         </is>
       </c>
       <c r="B231" s="4" t="inlineStr">
         <is>
-          <t>Yields</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C231" s="4" t="inlineStr">
@@ -31886,7 +31878,7 @@
       </c>
       <c r="F231" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.exclusionType?</t>
         </is>
       </c>
       <c r="G231" s="4" t="inlineStr">
@@ -31905,7 +31897,7 @@
     <row r="232">
       <c r="A232" s="4" t="inlineStr">
         <is>
-          <t>warehouseId</t>
+          <t>exclusion</t>
         </is>
       </c>
       <c r="B232" s="4" t="inlineStr">
@@ -31926,7 +31918,7 @@
       </c>
       <c r="F232" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.warehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.exclusion?</t>
         </is>
       </c>
       <c r="G232" s="4" t="inlineStr">
@@ -31942,88 +31934,8 @@
         </is>
       </c>
     </row>
-    <row r="233">
-      <c r="A233" s="4" t="inlineStr">
-        <is>
-          <t>exclusionType</t>
-        </is>
-      </c>
-      <c r="B233" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C233" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D233" s="4" t="inlineStr"/>
-      <c r="E233" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F233" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.exclusionType?</t>
-        </is>
-      </c>
-      <c r="G233" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H233" s="4" t="inlineStr"/>
-      <c r="I233" s="4" t="inlineStr"/>
-      <c r="J233" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="234">
-      <c r="A234" s="4" t="inlineStr">
-        <is>
-          <t>exclusion</t>
-        </is>
-      </c>
-      <c r="B234" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C234" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D234" s="4" t="inlineStr"/>
-      <c r="E234" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F234" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.exclusion?</t>
-        </is>
-      </c>
-      <c r="G234" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H234" s="4" t="inlineStr"/>
-      <c r="I234" s="4" t="inlineStr"/>
-      <c r="J234" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J234"/>
+  <autoFilter ref="A1:J232"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -32583,31 +32495,27 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>WarehouseStockOnHand</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>WarehouseStockOnHand.csv</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>partCode, warehouseCode, inventoryType, quantityAllocated, quantityOnHand, quantityInbound, quantityOutbound, uniqueId</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>inventoryType; quantityOutbound; uniqueId</t>
-        </is>
-      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>partCode, warehouseCode, quantityAllocated, quantityOnHand, quantityInbound, uniqueId</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -32799,27 +32707,31 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>PurchaseOrders</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>PurchaseOrders.csv</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>purchaseOrderNumber, purchaseOrderStatus, creationDateTime, approvalDateTime, toWarehouseId, vendorId, demandStatus, partNumber, quantity, lineCost, quantityReceived, receivedDateTime</t>
         </is>
       </c>
-      <c r="E30" s="6" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>demandStatus</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Apply warehouse manual mappings
</commit_message>
<xml_diff>
--- a/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
+++ b/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Target Fields'!$A$1:$S$151</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Template Fields'!$A$1:$H$180</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Evidence'!$A$1:$D$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$J$232</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$J$224</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Output Objects'!$A$1:$E$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Missing Important Fields'!$A$1:$E$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'SAP Investigation Log'!$A$1:$E$10</definedName>
@@ -244,8 +244,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:J232" headerRowCount="1">
-  <autoFilter ref="A1:J232"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:J224" headerRowCount="1">
+  <autoFilter ref="A1:J224"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Field"/>
     <tableColumn id="2" name="Object"/>
@@ -16545,40 +16545,44 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>Warehouses</t>
         </is>
       </c>
-      <c r="B49" s="4" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>addressId</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>External (Client-facing) Id</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>Investigate source</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr"/>
-      <c r="G49" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H49" s="4" t="inlineStr">
-        <is>
-          <t>Expected site/address id linking to the Addresses template. Data dictionary field: warehouse.address_id.</t>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Manual fill workbook:addressId; currently warehouse code per user mapping</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -16617,116 +16621,128 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="inlineStr">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>Warehouses</t>
         </is>
       </c>
-      <c r="B51" s="4" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>returnWarehouseId</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>External (Client-facing) Id</t>
         </is>
       </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>Investigate source</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="inlineStr"/>
-      <c r="G51" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H51" s="4" t="inlineStr">
-        <is>
-          <t>Expected preferred warehouse for return/faulty stock going to repair or scrap. Data fields: return_warehouse.</t>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Manual fill workbook:returnWarehouseId</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="inlineStr">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>Warehouses</t>
         </is>
       </c>
-      <c r="B52" s="4" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>supplyWarehouseId</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>External (Client-facing) Id</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr">
-        <is>
-          <t>Investigate source</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="inlineStr"/>
-      <c r="G52" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H52" s="4" t="inlineStr">
-        <is>
-          <t>Expected preferred replenishment/source warehouse. Data fields: supply_warehouse.</t>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Manual fill workbook:supplyWarehouseId</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="inlineStr">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>Warehouses</t>
         </is>
       </c>
-      <c r="B53" s="4" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>warehouseTypeId</t>
         </is>
       </c>
-      <c r="C53" s="4" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>enum&lt;String&gt;</t>
         </is>
       </c>
-      <c r="D53" s="4" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>[BOOT,DEP,REPAIR]</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr">
-        <is>
-          <t>Investigate source</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr"/>
-      <c r="G53" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H53" s="4" t="inlineStr">
-        <is>
-          <t>Expected site type enum; sample template uses BOOT, DEP, and REPAIR. Data fields mark warehouse_type_id as critical.</t>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Manual fill workbook:warehouseTypeId</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -16799,36 +16815,40 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>Warehouses</t>
         </is>
       </c>
-      <c r="B56" s="4" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>isReplenishable</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>Boolean</t>
         </is>
       </c>
-      <c r="D56" s="4" t="inlineStr"/>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>Investigate source</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="inlineStr"/>
-      <c r="G56" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="inlineStr">
-        <is>
-          <t>Expected true when the site can be restocked. Data dictionary field: is_replenishable.</t>
+      <c r="D56" s="2" t="inlineStr"/>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Manual fill workbook:isReplenishable</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -16863,108 +16883,120 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="4" t="inlineStr">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>Warehouses</t>
         </is>
       </c>
-      <c r="B58" s="4" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>isBranchStockable</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>Boolean</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr"/>
-      <c r="E58" s="4" t="inlineStr">
-        <is>
-          <t>Investigate source</t>
-        </is>
-      </c>
-      <c r="F58" s="4" t="inlineStr"/>
-      <c r="G58" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H58" s="4" t="inlineStr">
-        <is>
-          <t>Expected true when branch/regional location can accept stock. Data fields: cst_branch_stockable.</t>
+      <c r="D58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Manual fill workbook:isBranchStockable</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="inlineStr">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>Warehouses</t>
         </is>
       </c>
-      <c r="B59" s="4" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>isRemote</t>
         </is>
       </c>
-      <c r="C59" s="4" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>Boolean</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr"/>
-      <c r="E59" s="4" t="inlineStr">
-        <is>
-          <t>Investigate source</t>
-        </is>
-      </c>
-      <c r="F59" s="4" t="inlineStr"/>
-      <c r="G59" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H59" s="4" t="inlineStr">
-        <is>
-          <t>Expected true when this is an outlying/regional location. Data fields: cst_remote.</t>
+      <c r="D59" s="2" t="inlineStr"/>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Manual fill workbook:isRemote</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="4" t="inlineStr">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>Warehouses</t>
         </is>
       </c>
-      <c r="B60" s="4" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>warehouseStatusId</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>Enum&lt;String&gt;</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>Confirm. May not be required</t>
         </is>
       </c>
-      <c r="E60" s="4" t="inlineStr">
-        <is>
-          <t>Investigate source</t>
-        </is>
-      </c>
-      <c r="F60" s="4" t="inlineStr"/>
-      <c r="G60" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H60" s="4" t="inlineStr">
-        <is>
-          <t>Expected current/inactive status if required by the importer. Template says confirm; data fields mention cst_active and is_obsolete.</t>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Manual fill workbook:isObsolete inverted to is_active flag (Y active, N obsolete)</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -21439,7 +21471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J232"/>
+  <dimension ref="A1:J224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -28297,12 +28329,12 @@
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>addressId</t>
+          <t>personId</t>
         </is>
       </c>
       <c r="B142" s="4" t="inlineStr">
         <is>
-          <t>Warehouses</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C142" s="4" t="inlineStr">
@@ -28313,12 +28345,12 @@
       <c r="D142" s="4" t="inlineStr"/>
       <c r="E142" s="4" t="inlineStr">
         <is>
-          <t>Investigate source</t>
+          <t>Investigate SAP first</t>
         </is>
       </c>
       <c r="F142" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.addressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.personId?</t>
         </is>
       </c>
       <c r="G142" s="4" t="inlineStr">
@@ -28330,19 +28362,19 @@
       <c r="I142" s="4" t="inlineStr"/>
       <c r="J142" s="4" t="inlineStr">
         <is>
-          <t>Expected site/address id linking to the Addresses template. Data dictionary field: warehouse.address_id.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>returnWarehouseId</t>
+          <t>role</t>
         </is>
       </c>
       <c r="B143" s="4" t="inlineStr">
         <is>
-          <t>Warehouses</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C143" s="4" t="inlineStr">
@@ -28353,12 +28385,12 @@
       <c r="D143" s="4" t="inlineStr"/>
       <c r="E143" s="4" t="inlineStr">
         <is>
-          <t>Investigate source</t>
+          <t>Investigate SAP first</t>
         </is>
       </c>
       <c r="F143" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.returnWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.role?</t>
         </is>
       </c>
       <c r="G143" s="4" t="inlineStr">
@@ -28370,19 +28402,19 @@
       <c r="I143" s="4" t="inlineStr"/>
       <c r="J143" s="4" t="inlineStr">
         <is>
-          <t>Expected preferred warehouse for return/faulty stock going to repair or scrap. Data fields: return_warehouse.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>supplyWarehouseId</t>
+          <t>addressId</t>
         </is>
       </c>
       <c r="B144" s="4" t="inlineStr">
         <is>
-          <t>Warehouses</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C144" s="4" t="inlineStr">
@@ -28393,12 +28425,12 @@
       <c r="D144" s="4" t="inlineStr"/>
       <c r="E144" s="4" t="inlineStr">
         <is>
-          <t>Investigate source</t>
+          <t>Investigate SAP first</t>
         </is>
       </c>
       <c r="F144" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.supplyWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.addressId?</t>
         </is>
       </c>
       <c r="G144" s="4" t="inlineStr">
@@ -28410,19 +28442,19 @@
       <c r="I144" s="4" t="inlineStr"/>
       <c r="J144" s="4" t="inlineStr">
         <is>
-          <t>Expected preferred replenishment/source warehouse. Data fields: supply_warehouse.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>warehouseTypeId</t>
+          <t>nodeId</t>
         </is>
       </c>
       <c r="B145" s="4" t="inlineStr">
         <is>
-          <t>Warehouses</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C145" s="4" t="inlineStr">
@@ -28433,12 +28465,12 @@
       <c r="D145" s="4" t="inlineStr"/>
       <c r="E145" s="4" t="inlineStr">
         <is>
-          <t>Investigate source</t>
+          <t>Investigate SAP first</t>
         </is>
       </c>
       <c r="F145" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.warehouseTypeId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.nodeId?</t>
         </is>
       </c>
       <c r="G145" s="4" t="inlineStr">
@@ -28450,19 +28482,19 @@
       <c r="I145" s="4" t="inlineStr"/>
       <c r="J145" s="4" t="inlineStr">
         <is>
-          <t>Expected site type enum; sample template uses BOOT, DEP, and REPAIR. Data fields mark warehouse_type_id as critical.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>isReplenishable</t>
+          <t>firstName</t>
         </is>
       </c>
       <c r="B146" s="4" t="inlineStr">
         <is>
-          <t>Warehouses</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C146" s="4" t="inlineStr">
@@ -28473,12 +28505,12 @@
       <c r="D146" s="4" t="inlineStr"/>
       <c r="E146" s="4" t="inlineStr">
         <is>
-          <t>Investigate source</t>
+          <t>Investigate SAP first</t>
         </is>
       </c>
       <c r="F146" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.isReplenishable?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.firstName?</t>
         </is>
       </c>
       <c r="G146" s="4" t="inlineStr">
@@ -28490,19 +28522,19 @@
       <c r="I146" s="4" t="inlineStr"/>
       <c r="J146" s="4" t="inlineStr">
         <is>
-          <t>Expected true when the site can be restocked. Data dictionary field: is_replenishable.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>isBranchStockable</t>
+          <t>middleName</t>
         </is>
       </c>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t>Warehouses</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C147" s="4" t="inlineStr">
@@ -28513,12 +28545,12 @@
       <c r="D147" s="4" t="inlineStr"/>
       <c r="E147" s="4" t="inlineStr">
         <is>
-          <t>Investigate source</t>
+          <t>Investigate SAP first</t>
         </is>
       </c>
       <c r="F147" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.isBranchStockable?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.middleName?</t>
         </is>
       </c>
       <c r="G147" s="4" t="inlineStr">
@@ -28530,19 +28562,19 @@
       <c r="I147" s="4" t="inlineStr"/>
       <c r="J147" s="4" t="inlineStr">
         <is>
-          <t>Expected true when branch/regional location can accept stock. Data fields: cst_branch_stockable.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>isRemote</t>
+          <t>surname</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
         <is>
-          <t>Warehouses</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C148" s="4" t="inlineStr">
@@ -28553,12 +28585,12 @@
       <c r="D148" s="4" t="inlineStr"/>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>Investigate source</t>
+          <t>Investigate SAP first</t>
         </is>
       </c>
       <c r="F148" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.isRemote?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.surname?</t>
         </is>
       </c>
       <c r="G148" s="4" t="inlineStr">
@@ -28570,19 +28602,19 @@
       <c r="I148" s="4" t="inlineStr"/>
       <c r="J148" s="4" t="inlineStr">
         <is>
-          <t>Expected true when this is an outlying/regional location. Data fields: cst_remote.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>warehouseStatusId</t>
+          <t>isActive</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>Warehouses</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">
@@ -28593,12 +28625,12 @@
       <c r="D149" s="4" t="inlineStr"/>
       <c r="E149" s="4" t="inlineStr">
         <is>
-          <t>Investigate source</t>
+          <t>Investigate SAP first</t>
         </is>
       </c>
       <c r="F149" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.warehouseStatusId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.isActive?</t>
         </is>
       </c>
       <c r="G149" s="4" t="inlineStr">
@@ -28610,14 +28642,14 @@
       <c r="I149" s="4" t="inlineStr"/>
       <c r="J149" s="4" t="inlineStr">
         <is>
-          <t>Expected current/inactive status if required by the importer. Template says confirm; data fields mention cst_active and is_obsolete.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>personId</t>
+          <t>telephoneNumber</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
@@ -28638,7 +28670,7 @@
       </c>
       <c r="F150" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.personId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.telephoneNumber?</t>
         </is>
       </c>
       <c r="G150" s="4" t="inlineStr">
@@ -28657,12 +28689,12 @@
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>customerCompanyCode</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
@@ -28678,7 +28710,7 @@
       </c>
       <c r="F151" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.role?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.customerCompanyCode?</t>
         </is>
       </c>
       <c r="G151" s="4" t="inlineStr">
@@ -28697,12 +28729,12 @@
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>addressId</t>
+          <t>orderType</t>
         </is>
       </c>
       <c r="B152" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C152" s="4" t="inlineStr">
@@ -28718,7 +28750,7 @@
       </c>
       <c r="F152" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.addressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderType?</t>
         </is>
       </c>
       <c r="G152" s="4" t="inlineStr">
@@ -28737,12 +28769,12 @@
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>nodeId</t>
+          <t>orderStatus</t>
         </is>
       </c>
       <c r="B153" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C153" s="4" t="inlineStr">
@@ -28758,7 +28790,7 @@
       </c>
       <c r="F153" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.nodeId?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStatus?</t>
         </is>
       </c>
       <c r="G153" s="4" t="inlineStr">
@@ -28777,12 +28809,12 @@
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>firstName</t>
+          <t>orderStartDatetime</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C154" s="4" t="inlineStr">
@@ -28798,7 +28830,7 @@
       </c>
       <c r="F154" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.firstName?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStartDatetime?</t>
         </is>
       </c>
       <c r="G154" s="4" t="inlineStr">
@@ -28817,12 +28849,12 @@
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>middleName</t>
+          <t>requestTicketDateTime</t>
         </is>
       </c>
       <c r="B155" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C155" s="4" t="inlineStr">
@@ -28838,7 +28870,7 @@
       </c>
       <c r="F155" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.middleName?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.requestTicketDateTime?</t>
         </is>
       </c>
       <c r="G155" s="4" t="inlineStr">
@@ -28857,12 +28889,12 @@
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>surname</t>
+          <t>siteCompanyCode</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C156" s="4" t="inlineStr">
@@ -28878,7 +28910,7 @@
       </c>
       <c r="F156" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.surname?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.siteCompanyCode?</t>
         </is>
       </c>
       <c r="G156" s="4" t="inlineStr">
@@ -28897,12 +28929,12 @@
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>isActive</t>
+          <t>assignedPersonCode</t>
         </is>
       </c>
       <c r="B157" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C157" s="4" t="inlineStr">
@@ -28918,7 +28950,7 @@
       </c>
       <c r="F157" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.isActive?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.assignedPersonCode?</t>
         </is>
       </c>
       <c r="G157" s="4" t="inlineStr">
@@ -28937,12 +28969,12 @@
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>telephoneNumber</t>
+          <t>resolvedDateTime</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C158" s="4" t="inlineStr">
@@ -28958,7 +28990,7 @@
       </c>
       <c r="F158" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.telephoneNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.resolvedDateTime?</t>
         </is>
       </c>
       <c r="G158" s="4" t="inlineStr">
@@ -28977,7 +29009,7 @@
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>customerCompanyCode</t>
+          <t>serialNumber</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
@@ -28998,7 +29030,7 @@
       </c>
       <c r="F159" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.customerCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.serialNumber?</t>
         </is>
       </c>
       <c r="G159" s="4" t="inlineStr">
@@ -29017,7 +29049,7 @@
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>orderType</t>
+          <t>relCompanyId</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
@@ -29038,7 +29070,7 @@
       </c>
       <c r="F160" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderType?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.relCompanyId?</t>
         </is>
       </c>
       <c r="G160" s="4" t="inlineStr">
@@ -29057,7 +29089,7 @@
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>orderStatus</t>
+          <t>deviceSerialNumber</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
@@ -29078,7 +29110,7 @@
       </c>
       <c r="F161" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.deviceSerialNumber?</t>
         </is>
       </c>
       <c r="G161" s="4" t="inlineStr">
@@ -29097,12 +29129,12 @@
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>orderStartDatetime</t>
+          <t>orderNumber</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C162" s="4" t="inlineStr">
@@ -29118,7 +29150,7 @@
       </c>
       <c r="F162" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStartDatetime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.orderNumber?</t>
         </is>
       </c>
       <c r="G162" s="4" t="inlineStr">
@@ -29137,12 +29169,12 @@
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>requestTicketDateTime</t>
+          <t>location</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C163" s="4" t="inlineStr">
@@ -29158,7 +29190,7 @@
       </c>
       <c r="F163" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.requestTicketDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.location?</t>
         </is>
       </c>
       <c r="G163" s="4" t="inlineStr">
@@ -29177,12 +29209,12 @@
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>siteCompanyCode</t>
+          <t>eta</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C164" s="4" t="inlineStr">
@@ -29198,7 +29230,7 @@
       </c>
       <c r="F164" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.siteCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.eta?</t>
         </is>
       </c>
       <c r="G164" s="4" t="inlineStr">
@@ -29217,12 +29249,12 @@
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t>assignedPersonCode</t>
+          <t>actualEta</t>
         </is>
       </c>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C165" s="4" t="inlineStr">
@@ -29238,7 +29270,7 @@
       </c>
       <c r="F165" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.assignedPersonCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualEta?</t>
         </is>
       </c>
       <c r="G165" s="4" t="inlineStr">
@@ -29257,12 +29289,12 @@
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>resolvedDateTime</t>
+          <t>actualResolveDateTime</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C166" s="4" t="inlineStr">
@@ -29278,7 +29310,7 @@
       </c>
       <c r="F166" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.resolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualResolveDateTime?</t>
         </is>
       </c>
       <c r="G166" s="4" t="inlineStr">
@@ -29297,12 +29329,12 @@
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>serialNumber</t>
+          <t>recallDateTime</t>
         </is>
       </c>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C167" s="4" t="inlineStr">
@@ -29318,7 +29350,7 @@
       </c>
       <c r="F167" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.serialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.recallDateTime?</t>
         </is>
       </c>
       <c r="G167" s="4" t="inlineStr">
@@ -29337,12 +29369,12 @@
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>relCompanyId</t>
+          <t>actualRecallDateTime</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C168" s="4" t="inlineStr">
@@ -29358,7 +29390,7 @@
       </c>
       <c r="F168" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.relCompanyId?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualRecallDateTime?</t>
         </is>
       </c>
       <c r="G168" s="4" t="inlineStr">
@@ -29377,12 +29409,12 @@
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>deviceSerialNumber</t>
+          <t>slaEtaClock</t>
         </is>
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
@@ -29398,7 +29430,7 @@
       </c>
       <c r="F169" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.deviceSerialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaClock?</t>
         </is>
       </c>
       <c r="G169" s="4" t="inlineStr">
@@ -29417,7 +29449,7 @@
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>orderNumber</t>
+          <t>slaResolveClock</t>
         </is>
       </c>
       <c r="B170" s="4" t="inlineStr">
@@ -29438,7 +29470,7 @@
       </c>
       <c r="F170" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.orderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveClock?</t>
         </is>
       </c>
       <c r="G170" s="4" t="inlineStr">
@@ -29457,7 +29489,7 @@
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>slaFailureCode</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
@@ -29478,7 +29510,7 @@
       </c>
       <c r="F171" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.location?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaFailureCode?</t>
         </is>
       </c>
       <c r="G171" s="4" t="inlineStr">
@@ -29497,7 +29529,7 @@
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>eta</t>
+          <t>slaEtaHit</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
@@ -29518,7 +29550,7 @@
       </c>
       <c r="F172" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.eta?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaHit?</t>
         </is>
       </c>
       <c r="G172" s="4" t="inlineStr">
@@ -29537,7 +29569,7 @@
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>actualEta</t>
+          <t>slaResolvedDateTime</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
@@ -29558,7 +29590,7 @@
       </c>
       <c r="F173" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualEta?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolvedDateTime?</t>
         </is>
       </c>
       <c r="G173" s="4" t="inlineStr">
@@ -29577,12 +29609,12 @@
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>actualResolveDateTime</t>
+          <t>orderNumber</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C174" s="4" t="inlineStr">
@@ -29598,7 +29630,7 @@
       </c>
       <c r="F174" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualResolveDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderNumber?</t>
         </is>
       </c>
       <c r="G174" s="4" t="inlineStr">
@@ -29617,12 +29649,12 @@
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>recallDateTime</t>
+          <t>requestId</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C175" s="4" t="inlineStr">
@@ -29638,7 +29670,7 @@
       </c>
       <c r="F175" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.recallDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.requestId?</t>
         </is>
       </c>
       <c r="G175" s="4" t="inlineStr">
@@ -29657,12 +29689,12 @@
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>actualRecallDateTime</t>
+          <t>customerCompanyCode</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C176" s="4" t="inlineStr">
@@ -29678,7 +29710,7 @@
       </c>
       <c r="F176" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualRecallDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.customerCompanyCode?</t>
         </is>
       </c>
       <c r="G176" s="4" t="inlineStr">
@@ -29697,12 +29729,12 @@
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>slaEtaClock</t>
+          <t>orderStatus</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C177" s="4" t="inlineStr">
@@ -29718,7 +29750,7 @@
       </c>
       <c r="F177" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaClock?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStatus?</t>
         </is>
       </c>
       <c r="G177" s="4" t="inlineStr">
@@ -29737,12 +29769,12 @@
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>slaResolveClock</t>
+          <t>orderStartDatetime</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C178" s="4" t="inlineStr">
@@ -29758,7 +29790,7 @@
       </c>
       <c r="F178" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveClock?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStartDatetime?</t>
         </is>
       </c>
       <c r="G178" s="4" t="inlineStr">
@@ -29777,12 +29809,12 @@
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>slaFailureCode</t>
+          <t>siteCompanyCode</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C179" s="4" t="inlineStr">
@@ -29798,7 +29830,7 @@
       </c>
       <c r="F179" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaFailureCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.siteCompanyCode?</t>
         </is>
       </c>
       <c r="G179" s="4" t="inlineStr">
@@ -29817,12 +29849,12 @@
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>slaEtaHit</t>
+          <t>repairType</t>
         </is>
       </c>
       <c r="B180" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C180" s="4" t="inlineStr">
@@ -29838,7 +29870,7 @@
       </c>
       <c r="F180" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaHit?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairType?</t>
         </is>
       </c>
       <c r="G180" s="4" t="inlineStr">
@@ -29857,12 +29889,12 @@
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>slaResolvedDateTime</t>
+          <t>partsOrderDateTime</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C181" s="4" t="inlineStr">
@@ -29878,7 +29910,7 @@
       </c>
       <c r="F181" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsOrderDateTime?</t>
         </is>
       </c>
       <c r="G181" s="4" t="inlineStr">
@@ -29897,7 +29929,7 @@
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>orderNumber</t>
+          <t>partsReceivedDateTime</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
@@ -29918,7 +29950,7 @@
       </c>
       <c r="F182" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsReceivedDateTime?</t>
         </is>
       </c>
       <c r="G182" s="4" t="inlineStr">
@@ -29937,7 +29969,7 @@
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>requestId</t>
+          <t>repairCode</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
@@ -29958,7 +29990,7 @@
       </c>
       <c r="F183" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.requestId?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCode?</t>
         </is>
       </c>
       <c r="G183" s="4" t="inlineStr">
@@ -29977,7 +30009,7 @@
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>customerCompanyCode</t>
+          <t>repairCompany</t>
         </is>
       </c>
       <c r="B184" s="4" t="inlineStr">
@@ -29998,7 +30030,7 @@
       </c>
       <c r="F184" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.customerCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCompany?</t>
         </is>
       </c>
       <c r="G184" s="4" t="inlineStr">
@@ -30017,7 +30049,7 @@
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>orderStatus</t>
+          <t>raStatus</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
@@ -30038,7 +30070,7 @@
       </c>
       <c r="F185" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.raStatus?</t>
         </is>
       </c>
       <c r="G185" s="4" t="inlineStr">
@@ -30057,7 +30089,7 @@
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>orderStartDatetime</t>
+          <t>Warehouse</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
@@ -30078,7 +30110,7 @@
       </c>
       <c r="F186" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStartDatetime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.Warehouse?</t>
         </is>
       </c>
       <c r="G186" s="4" t="inlineStr">
@@ -30097,7 +30129,7 @@
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>siteCompanyCode</t>
+          <t>assignedPerson</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
@@ -30118,7 +30150,7 @@
       </c>
       <c r="F187" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.siteCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.assignedPerson?</t>
         </is>
       </c>
       <c r="G187" s="4" t="inlineStr">
@@ -30137,7 +30169,7 @@
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>repairType</t>
+          <t>orderedPartId</t>
         </is>
       </c>
       <c r="B188" s="4" t="inlineStr">
@@ -30158,7 +30190,7 @@
       </c>
       <c r="F188" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairType?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderedPartId?</t>
         </is>
       </c>
       <c r="G188" s="4" t="inlineStr">
@@ -30177,7 +30209,7 @@
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>partsOrderDateTime</t>
+          <t>actualPartId</t>
         </is>
       </c>
       <c r="B189" s="4" t="inlineStr">
@@ -30198,7 +30230,7 @@
       </c>
       <c r="F189" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsOrderDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.actualPartId?</t>
         </is>
       </c>
       <c r="G189" s="4" t="inlineStr">
@@ -30217,7 +30249,7 @@
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>partsReceivedDateTime</t>
+          <t>resolvedDateTime</t>
         </is>
       </c>
       <c r="B190" s="4" t="inlineStr">
@@ -30238,7 +30270,7 @@
       </c>
       <c r="F190" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsReceivedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.resolvedDateTime?</t>
         </is>
       </c>
       <c r="G190" s="4" t="inlineStr">
@@ -30257,7 +30289,7 @@
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>repairCode</t>
+          <t>serialNumber</t>
         </is>
       </c>
       <c r="B191" s="4" t="inlineStr">
@@ -30278,7 +30310,7 @@
       </c>
       <c r="F191" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.serialNumber?</t>
         </is>
       </c>
       <c r="G191" s="4" t="inlineStr">
@@ -30297,7 +30329,7 @@
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>repairCompany</t>
+          <t>quantityUsed</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
@@ -30318,7 +30350,7 @@
       </c>
       <c r="F192" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCompany?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.quantityUsed?</t>
         </is>
       </c>
       <c r="G192" s="4" t="inlineStr">
@@ -30337,7 +30369,7 @@
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>raStatus</t>
+          <t>relCompanyId</t>
         </is>
       </c>
       <c r="B193" s="4" t="inlineStr">
@@ -30358,7 +30390,7 @@
       </c>
       <c r="F193" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.raStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.relCompanyId?</t>
         </is>
       </c>
       <c r="G193" s="4" t="inlineStr">
@@ -30377,7 +30409,7 @@
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>Warehouse</t>
+          <t>partsUsedDateTime</t>
         </is>
       </c>
       <c r="B194" s="4" t="inlineStr">
@@ -30398,7 +30430,7 @@
       </c>
       <c r="F194" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.Warehouse?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsUsedDateTime?</t>
         </is>
       </c>
       <c r="G194" s="4" t="inlineStr">
@@ -30417,7 +30449,7 @@
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>assignedPerson</t>
+          <t>deviceSerialNumber</t>
         </is>
       </c>
       <c r="B195" s="4" t="inlineStr">
@@ -30438,7 +30470,7 @@
       </c>
       <c r="F195" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.assignedPerson?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.deviceSerialNumber?</t>
         </is>
       </c>
       <c r="G195" s="4" t="inlineStr">
@@ -30457,12 +30489,12 @@
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>orderedPartId</t>
+          <t>partCode</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>PartCost</t>
         </is>
       </c>
       <c r="C196" s="4" t="inlineStr">
@@ -30478,7 +30510,7 @@
       </c>
       <c r="F196" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderedPartId?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.partCode?</t>
         </is>
       </c>
       <c r="G196" s="4" t="inlineStr">
@@ -30497,12 +30529,12 @@
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>actualPartId</t>
+          <t>cost</t>
         </is>
       </c>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>PartCost</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr">
@@ -30518,7 +30550,7 @@
       </c>
       <c r="F197" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.actualPartId?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.cost?</t>
         </is>
       </c>
       <c r="G197" s="4" t="inlineStr">
@@ -30537,12 +30569,12 @@
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>resolvedDateTime</t>
+          <t>currencyCode</t>
         </is>
       </c>
       <c r="B198" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>PartCost</t>
         </is>
       </c>
       <c r="C198" s="4" t="inlineStr">
@@ -30558,7 +30590,7 @@
       </c>
       <c r="F198" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.resolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.currencyCode?</t>
         </is>
       </c>
       <c r="G198" s="4" t="inlineStr">
@@ -30577,12 +30609,12 @@
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>serialNumber</t>
+          <t>averageCost</t>
         </is>
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>PartCost</t>
         </is>
       </c>
       <c r="C199" s="4" t="inlineStr">
@@ -30598,7 +30630,7 @@
       </c>
       <c r="F199" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.serialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.averageCost?</t>
         </is>
       </c>
       <c r="G199" s="4" t="inlineStr">
@@ -30617,12 +30649,12 @@
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>quantityUsed</t>
+          <t>partCode</t>
         </is>
       </c>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C200" s="4" t="inlineStr">
@@ -30638,7 +30670,7 @@
       </c>
       <c r="F200" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.quantityUsed?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
         </is>
       </c>
       <c r="G200" s="4" t="inlineStr">
@@ -30657,12 +30689,12 @@
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t>relCompanyId</t>
+          <t>modelCode</t>
         </is>
       </c>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C201" s="4" t="inlineStr">
@@ -30678,7 +30710,7 @@
       </c>
       <c r="F201" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.relCompanyId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
         </is>
       </c>
       <c r="G201" s="4" t="inlineStr">
@@ -30697,12 +30729,12 @@
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>partsUsedDateTime</t>
+          <t>modelDescription</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C202" s="4" t="inlineStr">
@@ -30718,7 +30750,7 @@
       </c>
       <c r="F202" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsUsedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
         </is>
       </c>
       <c r="G202" s="4" t="inlineStr">
@@ -30737,12 +30769,12 @@
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>deviceSerialNumber</t>
+          <t>inventoryTransferImoId</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C203" s="4" t="inlineStr">
@@ -30758,7 +30790,7 @@
       </c>
       <c r="F203" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.deviceSerialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.inventoryTransferImoId?</t>
         </is>
       </c>
       <c r="G203" s="4" t="inlineStr">
@@ -30777,12 +30809,12 @@
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>partCode</t>
+          <t>createdDateTime</t>
         </is>
       </c>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C204" s="4" t="inlineStr">
@@ -30798,7 +30830,7 @@
       </c>
       <c r="F204" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.partCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.createdDateTime?</t>
         </is>
       </c>
       <c r="G204" s="4" t="inlineStr">
@@ -30817,12 +30849,12 @@
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>completedDateTime</t>
         </is>
       </c>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C205" s="4" t="inlineStr">
@@ -30838,7 +30870,7 @@
       </c>
       <c r="F205" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.cost?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.completedDateTime?</t>
         </is>
       </c>
       <c r="G205" s="4" t="inlineStr">
@@ -30857,12 +30889,12 @@
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
         <is>
-          <t>currencyCode</t>
+          <t>fromWarehouseId</t>
         </is>
       </c>
       <c r="B206" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C206" s="4" t="inlineStr">
@@ -30878,7 +30910,7 @@
       </c>
       <c r="F206" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.currencyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.fromWarehouseId?</t>
         </is>
       </c>
       <c r="G206" s="4" t="inlineStr">
@@ -30897,12 +30929,12 @@
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>averageCost</t>
+          <t>toWarehouseId</t>
         </is>
       </c>
       <c r="B207" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C207" s="4" t="inlineStr">
@@ -30918,7 +30950,7 @@
       </c>
       <c r="F207" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.averageCost?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.toWarehouseId?</t>
         </is>
       </c>
       <c r="G207" s="4" t="inlineStr">
@@ -30937,12 +30969,12 @@
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
         <is>
-          <t>partCode</t>
+          <t>demandStatus</t>
         </is>
       </c>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C208" s="4" t="inlineStr">
@@ -30958,7 +30990,7 @@
       </c>
       <c r="F208" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.demandStatus?</t>
         </is>
       </c>
       <c r="G208" s="4" t="inlineStr">
@@ -30977,12 +31009,12 @@
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t>modelCode</t>
+          <t>orderStatusIsClosed</t>
         </is>
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C209" s="4" t="inlineStr">
@@ -30998,7 +31030,7 @@
       </c>
       <c r="F209" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.orderStatusIsClosed?</t>
         </is>
       </c>
       <c r="G209" s="4" t="inlineStr">
@@ -31017,12 +31049,12 @@
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
         <is>
-          <t>modelDescription</t>
+          <t>movementType</t>
         </is>
       </c>
       <c r="B210" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C210" s="4" t="inlineStr">
@@ -31038,7 +31070,7 @@
       </c>
       <c r="F210" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
         </is>
       </c>
       <c r="G210" s="4" t="inlineStr">
@@ -31057,7 +31089,7 @@
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
         <is>
-          <t>inventoryTransferImoId</t>
+          <t>addressId</t>
         </is>
       </c>
       <c r="B211" s="4" t="inlineStr">
@@ -31078,7 +31110,7 @@
       </c>
       <c r="F211" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.inventoryTransferImoId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
         </is>
       </c>
       <c r="G211" s="4" t="inlineStr">
@@ -31097,7 +31129,7 @@
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
         <is>
-          <t>createdDateTime</t>
+          <t>isResolved</t>
         </is>
       </c>
       <c r="B212" s="4" t="inlineStr">
@@ -31118,7 +31150,7 @@
       </c>
       <c r="F212" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.createdDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.isResolved?</t>
         </is>
       </c>
       <c r="G212" s="4" t="inlineStr">
@@ -31137,7 +31169,7 @@
     <row r="213">
       <c r="A213" s="4" t="inlineStr">
         <is>
-          <t>completedDateTime</t>
+          <t>partNumber</t>
         </is>
       </c>
       <c r="B213" s="4" t="inlineStr">
@@ -31158,7 +31190,7 @@
       </c>
       <c r="F213" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.completedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.partNumber?</t>
         </is>
       </c>
       <c r="G213" s="4" t="inlineStr">
@@ -31177,7 +31209,7 @@
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
         <is>
-          <t>fromWarehouseId</t>
+          <t>quantity</t>
         </is>
       </c>
       <c r="B214" s="4" t="inlineStr">
@@ -31198,7 +31230,7 @@
       </c>
       <c r="F214" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.fromWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.quantity?</t>
         </is>
       </c>
       <c r="G214" s="4" t="inlineStr">
@@ -31217,7 +31249,7 @@
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
         <is>
-          <t>toWarehouseId</t>
+          <t>shipListCode</t>
         </is>
       </c>
       <c r="B215" s="4" t="inlineStr">
@@ -31238,7 +31270,7 @@
       </c>
       <c r="F215" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.toWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
         </is>
       </c>
       <c r="G215" s="4" t="inlineStr">
@@ -31255,54 +31287,54 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="4" t="inlineStr">
+      <c r="A216" s="3" t="inlineStr">
         <is>
           <t>demandStatus</t>
         </is>
       </c>
-      <c r="B216" s="4" t="inlineStr">
-        <is>
-          <t>InventoryTransfers</t>
-        </is>
-      </c>
-      <c r="C216" s="4" t="inlineStr">
+      <c r="B216" s="3" t="inlineStr">
+        <is>
+          <t>PurchaseOrders</t>
+        </is>
+      </c>
+      <c r="C216" s="3" t="inlineStr">
         <is>
           <t>Planning V2 template</t>
         </is>
       </c>
-      <c r="D216" s="4" t="inlineStr"/>
-      <c r="E216" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F216" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.demandStatus?</t>
-        </is>
-      </c>
-      <c r="G216" s="4" t="inlineStr">
+      <c r="D216" s="3" t="inlineStr"/>
+      <c r="E216" s="3" t="inlineStr">
+        <is>
+          <t>Review required</t>
+        </is>
+      </c>
+      <c r="F216" s="3" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
+        </is>
+      </c>
+      <c r="G216" s="3" t="inlineStr">
         <is>
           <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
         </is>
       </c>
-      <c r="H216" s="4" t="inlineStr"/>
-      <c r="I216" s="4" t="inlineStr"/>
-      <c r="J216" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="H216" s="3" t="inlineStr"/>
+      <c r="I216" s="3" t="inlineStr"/>
+      <c r="J216" s="3" t="inlineStr">
+        <is>
+          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.DocNum and part/SPL Master evidence also matches; current export needs reconciliation.</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t>orderStatusIsClosed</t>
+          <t>partTypeCode</t>
         </is>
       </c>
       <c r="B217" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C217" s="4" t="inlineStr">
@@ -31318,7 +31350,7 @@
       </c>
       <c r="F217" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.orderStatusIsClosed?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeCode?</t>
         </is>
       </c>
       <c r="G217" s="4" t="inlineStr">
@@ -31337,12 +31369,12 @@
     <row r="218">
       <c r="A218" s="4" t="inlineStr">
         <is>
-          <t>movementType</t>
+          <t>description</t>
         </is>
       </c>
       <c r="B218" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C218" s="4" t="inlineStr">
@@ -31358,7 +31390,7 @@
       </c>
       <c r="F218" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.description?</t>
         </is>
       </c>
       <c r="G218" s="4" t="inlineStr">
@@ -31377,12 +31409,12 @@
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t>addressId</t>
+          <t>partNumber</t>
         </is>
       </c>
       <c r="B219" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C219" s="4" t="inlineStr">
@@ -31398,7 +31430,7 @@
       </c>
       <c r="F219" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
         </is>
       </c>
       <c r="G219" s="4" t="inlineStr">
@@ -31417,12 +31449,12 @@
     <row r="220">
       <c r="A220" s="4" t="inlineStr">
         <is>
-          <t>isResolved</t>
+          <t>unitOfMeasure</t>
         </is>
       </c>
       <c r="B220" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C220" s="4" t="inlineStr">
@@ -31438,7 +31470,7 @@
       </c>
       <c r="F220" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.isResolved?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
         </is>
       </c>
       <c r="G220" s="4" t="inlineStr">
@@ -31457,12 +31489,12 @@
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
         <is>
-          <t>partNumber</t>
+          <t>yield</t>
         </is>
       </c>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C221" s="4" t="inlineStr">
@@ -31478,7 +31510,7 @@
       </c>
       <c r="F221" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.partNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
         </is>
       </c>
       <c r="G221" s="4" t="inlineStr">
@@ -31497,12 +31529,12 @@
     <row r="222">
       <c r="A222" s="4" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>warehouseId</t>
         </is>
       </c>
       <c r="B222" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C222" s="4" t="inlineStr">
@@ -31518,7 +31550,7 @@
       </c>
       <c r="F222" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.quantity?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.warehouseId?</t>
         </is>
       </c>
       <c r="G222" s="4" t="inlineStr">
@@ -31537,12 +31569,12 @@
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
         <is>
-          <t>shipListCode</t>
+          <t>exclusionType</t>
         </is>
       </c>
       <c r="B223" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C223" s="4" t="inlineStr">
@@ -31558,7 +31590,7 @@
       </c>
       <c r="F223" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.exclusionType?</t>
         </is>
       </c>
       <c r="G223" s="4" t="inlineStr">
@@ -31575,367 +31607,47 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="3" t="inlineStr">
-        <is>
-          <t>demandStatus</t>
-        </is>
-      </c>
-      <c r="B224" s="3" t="inlineStr">
-        <is>
-          <t>PurchaseOrders</t>
-        </is>
-      </c>
-      <c r="C224" s="3" t="inlineStr">
+      <c r="A224" s="4" t="inlineStr">
+        <is>
+          <t>exclusion</t>
+        </is>
+      </c>
+      <c r="B224" s="4" t="inlineStr">
+        <is>
+          <t>WarehouseExclusions</t>
+        </is>
+      </c>
+      <c r="C224" s="4" t="inlineStr">
         <is>
           <t>Planning V2 template</t>
         </is>
       </c>
-      <c r="D224" s="3" t="inlineStr"/>
-      <c r="E224" s="3" t="inlineStr">
-        <is>
-          <t>Review required</t>
-        </is>
-      </c>
-      <c r="F224" s="3" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
-        </is>
-      </c>
-      <c r="G224" s="3" t="inlineStr">
+      <c r="D224" s="4" t="inlineStr"/>
+      <c r="E224" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F224" s="4" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.exclusion?</t>
+        </is>
+      </c>
+      <c r="G224" s="4" t="inlineStr">
         <is>
           <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
         </is>
       </c>
-      <c r="H224" s="3" t="inlineStr"/>
-      <c r="I224" s="3" t="inlineStr"/>
-      <c r="J224" s="3" t="inlineStr">
-        <is>
-          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.DocNum and part/SPL Master evidence also matches; current export needs reconciliation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" s="4" t="inlineStr">
-        <is>
-          <t>partTypeCode</t>
-        </is>
-      </c>
-      <c r="B225" s="4" t="inlineStr">
-        <is>
-          <t>PartTypes</t>
-        </is>
-      </c>
-      <c r="C225" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D225" s="4" t="inlineStr"/>
-      <c r="E225" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F225" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeCode?</t>
-        </is>
-      </c>
-      <c r="G225" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H225" s="4" t="inlineStr"/>
-      <c r="I225" s="4" t="inlineStr"/>
-      <c r="J225" s="4" t="inlineStr">
+      <c r="H224" s="4" t="inlineStr"/>
+      <c r="I224" s="4" t="inlineStr"/>
+      <c r="J224" s="4" t="inlineStr">
         <is>
           <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
-    <row r="226">
-      <c r="A226" s="4" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="B226" s="4" t="inlineStr">
-        <is>
-          <t>PartTypes</t>
-        </is>
-      </c>
-      <c r="C226" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D226" s="4" t="inlineStr"/>
-      <c r="E226" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F226" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.description?</t>
-        </is>
-      </c>
-      <c r="G226" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H226" s="4" t="inlineStr"/>
-      <c r="I226" s="4" t="inlineStr"/>
-      <c r="J226" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" s="4" t="inlineStr">
-        <is>
-          <t>partNumber</t>
-        </is>
-      </c>
-      <c r="B227" s="4" t="inlineStr">
-        <is>
-          <t>Yields</t>
-        </is>
-      </c>
-      <c r="C227" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D227" s="4" t="inlineStr"/>
-      <c r="E227" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F227" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
-        </is>
-      </c>
-      <c r="G227" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H227" s="4" t="inlineStr"/>
-      <c r="I227" s="4" t="inlineStr"/>
-      <c r="J227" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" s="4" t="inlineStr">
-        <is>
-          <t>unitOfMeasure</t>
-        </is>
-      </c>
-      <c r="B228" s="4" t="inlineStr">
-        <is>
-          <t>Yields</t>
-        </is>
-      </c>
-      <c r="C228" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D228" s="4" t="inlineStr"/>
-      <c r="E228" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F228" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
-        </is>
-      </c>
-      <c r="G228" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H228" s="4" t="inlineStr"/>
-      <c r="I228" s="4" t="inlineStr"/>
-      <c r="J228" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" s="4" t="inlineStr">
-        <is>
-          <t>yield</t>
-        </is>
-      </c>
-      <c r="B229" s="4" t="inlineStr">
-        <is>
-          <t>Yields</t>
-        </is>
-      </c>
-      <c r="C229" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D229" s="4" t="inlineStr"/>
-      <c r="E229" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F229" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
-        </is>
-      </c>
-      <c r="G229" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H229" s="4" t="inlineStr"/>
-      <c r="I229" s="4" t="inlineStr"/>
-      <c r="J229" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" s="4" t="inlineStr">
-        <is>
-          <t>warehouseId</t>
-        </is>
-      </c>
-      <c r="B230" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C230" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D230" s="4" t="inlineStr"/>
-      <c r="E230" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F230" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.warehouseId?</t>
-        </is>
-      </c>
-      <c r="G230" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H230" s="4" t="inlineStr"/>
-      <c r="I230" s="4" t="inlineStr"/>
-      <c r="J230" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" s="4" t="inlineStr">
-        <is>
-          <t>exclusionType</t>
-        </is>
-      </c>
-      <c r="B231" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C231" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D231" s="4" t="inlineStr"/>
-      <c r="E231" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F231" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.exclusionType?</t>
-        </is>
-      </c>
-      <c r="G231" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H231" s="4" t="inlineStr"/>
-      <c r="I231" s="4" t="inlineStr"/>
-      <c r="J231" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" s="4" t="inlineStr">
-        <is>
-          <t>exclusion</t>
-        </is>
-      </c>
-      <c r="B232" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C232" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D232" s="4" t="inlineStr"/>
-      <c r="E232" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F232" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.exclusion?</t>
-        </is>
-      </c>
-      <c r="G232" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H232" s="4" t="inlineStr"/>
-      <c r="I232" s="4" t="inlineStr"/>
-      <c r="J232" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J232"/>
+  <autoFilter ref="A1:J224"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -32468,31 +32180,27 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Warehouses</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Warehouses.csv</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>warehouseId, addressId, returnWarehouseId, supplyWarehouseId, warehouseTypeId, warehouseDescription, isReplenishable, isBranchStockable, isRemote, warehouseStatusId</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>addressId; returnWarehouseId; supplyWarehouseId; warehouseTypeId; isReplenishable; isBranchStockable; isRemote; warehouseStatusId</t>
-        </is>
-      </c>
+      <c r="E21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Map parts usage from HelpDesk tickets
</commit_message>
<xml_diff>
--- a/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
+++ b/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Target Fields'!$A$1:$S$151</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Template Fields'!$A$1:$H$177</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Evidence'!$A$1:$D$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$J$224</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$J$219</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Output Objects'!$A$1:$E$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Missing Important Fields'!$A$1:$E$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'SAP Investigation Log'!$A$1:$E$10</definedName>
@@ -244,8 +244,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:J224" headerRowCount="1">
-  <autoFilter ref="A1:J224"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:J219" headerRowCount="1">
+  <autoFilter ref="A1:J219"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Field"/>
     <tableColumn id="2" name="Object"/>
@@ -17922,7 +17922,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Stock Audit Report 3Y:Document for DN rows</t>
+          <t>CoCre8 HelpDesk issue tracker:Call Number</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -18005,116 +18005,128 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="4" t="inlineStr">
+      <c r="A83" s="2" t="inlineStr">
         <is>
           <t>PartsUsage</t>
         </is>
       </c>
-      <c r="B83" s="4" t="inlineStr">
+      <c r="B83" s="2" t="inlineStr">
         <is>
           <t>customerCompanyCode</t>
         </is>
       </c>
-      <c r="C83" s="4" t="inlineStr">
+      <c r="C83" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D83" s="4" t="inlineStr">
+      <c r="D83" s="2" t="inlineStr">
         <is>
           <t>Canonical header from PartsUsage.xlsx</t>
         </is>
       </c>
-      <c r="E83" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F83" s="4" t="inlineStr"/>
-      <c r="G83" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H83" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>CoCre8 HelpDesk issue tracker:CustomerNormalized/Customer</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="4" t="inlineStr">
+      <c r="A84" s="2" t="inlineStr">
         <is>
           <t>PartsUsage</t>
         </is>
       </c>
-      <c r="B84" s="4" t="inlineStr">
+      <c r="B84" s="2" t="inlineStr">
         <is>
           <t>orderStartDatetime</t>
         </is>
       </c>
-      <c r="C84" s="4" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr">
         <is>
           <t>DateTime</t>
         </is>
       </c>
-      <c r="D84" s="4" t="inlineStr">
+      <c r="D84" s="2" t="inlineStr">
         <is>
           <t>Canonical header from PartsUsage.xlsx</t>
         </is>
       </c>
-      <c r="E84" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F84" s="4" t="inlineStr"/>
-      <c r="G84" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H84" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>CoCre8 HelpDesk issue tracker:Created</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="4" t="inlineStr">
+      <c r="A85" s="2" t="inlineStr">
         <is>
           <t>PartsUsage</t>
         </is>
       </c>
-      <c r="B85" s="4" t="inlineStr">
+      <c r="B85" s="2" t="inlineStr">
         <is>
           <t>orderStatus</t>
         </is>
       </c>
-      <c r="C85" s="4" t="inlineStr">
+      <c r="C85" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D85" s="4" t="inlineStr">
+      <c r="D85" s="2" t="inlineStr">
         <is>
           <t>Canonical header from PartsUsage.xlsx</t>
         </is>
       </c>
-      <c r="E85" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F85" s="4" t="inlineStr"/>
-      <c r="G85" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H85" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>CoCre8 HelpDesk issue tracker:Status</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -18184,7 +18196,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Stock Audit Report 3Y:Item No.</t>
+          <t>CoCre8 HelpDesk issue tracker:DispatchPartNo when present, otherwise Part Nr</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -18199,40 +18211,44 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="4" t="inlineStr">
+      <c r="A88" s="2" t="inlineStr">
         <is>
           <t>PartsUsage</t>
         </is>
       </c>
-      <c r="B88" s="4" t="inlineStr">
+      <c r="B88" s="2" t="inlineStr">
         <is>
           <t>serialNumber</t>
         </is>
       </c>
-      <c r="C88" s="4" t="inlineStr">
+      <c r="C88" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D88" s="4" t="inlineStr">
+      <c r="D88" s="2" t="inlineStr">
         <is>
           <t>Canonical header from PartsUsage.xlsx</t>
         </is>
       </c>
-      <c r="E88" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F88" s="4" t="inlineStr"/>
-      <c r="G88" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H88" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>CoCre8 HelpDesk issue tracker:Serial Nr</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -18264,7 +18280,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Stock Audit Report 3Y:absolute Quantity for negative DN rows</t>
+          <t>CoCre8 HelpDesk issue tracker:Quantity</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -18344,7 +18360,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>Stock Audit Report 3Y:Posting Date</t>
+          <t>CoCre8 HelpDesk issue tracker:Created used as demand/usage date</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -18386,7 +18402,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>Stock Audit Report 3Y:Whse</t>
+          <t>CoCre8 HelpDesk issue tracker:DispatchWarehouse</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -18439,40 +18455,44 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="4" t="inlineStr">
+      <c r="A94" s="2" t="inlineStr">
         <is>
           <t>PartsUsage</t>
         </is>
       </c>
-      <c r="B94" s="4" t="inlineStr">
+      <c r="B94" s="2" t="inlineStr">
         <is>
           <t>deviceSerialNumber</t>
         </is>
       </c>
-      <c r="C94" s="4" t="inlineStr">
+      <c r="C94" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D94" s="4" t="inlineStr">
+      <c r="D94" s="2" t="inlineStr">
         <is>
           <t>Canonical header from PartsUsage.xlsx</t>
         </is>
       </c>
-      <c r="E94" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F94" s="4" t="inlineStr"/>
-      <c r="G94" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H94" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>CoCre8 HelpDesk issue tracker:Serial Nr</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -18500,7 +18520,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>Reference masters.csv:SPL Master by used part</t>
+          <t>CoCre8 HelpDesk issue tracker:SPLMaster or masters.csv by part</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -21949,7 +21969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J224"/>
+  <dimension ref="A1:J219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -29247,7 +29267,7 @@
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>customerCompanyCode</t>
+          <t>resolvedDateTime</t>
         </is>
       </c>
       <c r="B153" s="4" t="inlineStr">
@@ -29268,7 +29288,7 @@
       </c>
       <c r="F153" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.customerCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.resolvedDateTime?</t>
         </is>
       </c>
       <c r="G153" s="4" t="inlineStr">
@@ -29287,7 +29307,7 @@
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>orderStartDatetime</t>
+          <t>relCompanyId</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
@@ -29308,7 +29328,7 @@
       </c>
       <c r="F154" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStartDatetime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.relCompanyId?</t>
         </is>
       </c>
       <c r="G154" s="4" t="inlineStr">
@@ -29327,7 +29347,7 @@
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>orderStatus</t>
+          <t>assignedPersonCode</t>
         </is>
       </c>
       <c r="B155" s="4" t="inlineStr">
@@ -29348,7 +29368,7 @@
       </c>
       <c r="F155" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.assignedPersonCode?</t>
         </is>
       </c>
       <c r="G155" s="4" t="inlineStr">
@@ -29367,12 +29387,12 @@
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>resolvedDateTime</t>
+          <t>orderNumber</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C156" s="4" t="inlineStr">
@@ -29388,7 +29408,7 @@
       </c>
       <c r="F156" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.resolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.orderNumber?</t>
         </is>
       </c>
       <c r="G156" s="4" t="inlineStr">
@@ -29407,12 +29427,12 @@
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>serialNumber</t>
+          <t>RequestID</t>
         </is>
       </c>
       <c r="B157" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C157" s="4" t="inlineStr">
@@ -29428,7 +29448,7 @@
       </c>
       <c r="F157" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.serialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.RequestID?</t>
         </is>
       </c>
       <c r="G157" s="4" t="inlineStr">
@@ -29447,12 +29467,12 @@
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>relCompanyId</t>
+          <t>location</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C158" s="4" t="inlineStr">
@@ -29468,7 +29488,7 @@
       </c>
       <c r="F158" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.relCompanyId?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.location?</t>
         </is>
       </c>
       <c r="G158" s="4" t="inlineStr">
@@ -29487,12 +29507,12 @@
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>assignedPersonCode</t>
+          <t>eta</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C159" s="4" t="inlineStr">
@@ -29508,7 +29528,7 @@
       </c>
       <c r="F159" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.assignedPersonCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.eta?</t>
         </is>
       </c>
       <c r="G159" s="4" t="inlineStr">
@@ -29527,12 +29547,12 @@
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>deviceSerialNumber</t>
+          <t>actualEta</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C160" s="4" t="inlineStr">
@@ -29548,7 +29568,7 @@
       </c>
       <c r="F160" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.deviceSerialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualEta?</t>
         </is>
       </c>
       <c r="G160" s="4" t="inlineStr">
@@ -29567,7 +29587,7 @@
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>orderNumber</t>
+          <t>actualResolveDateTime</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
@@ -29588,7 +29608,7 @@
       </c>
       <c r="F161" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.orderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualResolveDateTime?</t>
         </is>
       </c>
       <c r="G161" s="4" t="inlineStr">
@@ -29607,7 +29627,7 @@
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>RequestID</t>
+          <t>recallDateTime</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
@@ -29628,7 +29648,7 @@
       </c>
       <c r="F162" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.RequestID?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.recallDateTime?</t>
         </is>
       </c>
       <c r="G162" s="4" t="inlineStr">
@@ -29647,7 +29667,7 @@
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>actualRecallDateTime</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
@@ -29668,7 +29688,7 @@
       </c>
       <c r="F163" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.location?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualRecallDateTime?</t>
         </is>
       </c>
       <c r="G163" s="4" t="inlineStr">
@@ -29687,7 +29707,7 @@
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>eta</t>
+          <t>slaEtaClock</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
@@ -29708,7 +29728,7 @@
       </c>
       <c r="F164" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.eta?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaClock?</t>
         </is>
       </c>
       <c r="G164" s="4" t="inlineStr">
@@ -29727,7 +29747,7 @@
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t>actualEta</t>
+          <t>slaResolveClock</t>
         </is>
       </c>
       <c r="B165" s="4" t="inlineStr">
@@ -29748,7 +29768,7 @@
       </c>
       <c r="F165" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualEta?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveClock?</t>
         </is>
       </c>
       <c r="G165" s="4" t="inlineStr">
@@ -29767,7 +29787,7 @@
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>actualResolveDateTime</t>
+          <t>slaFailureCode</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
@@ -29788,7 +29808,7 @@
       </c>
       <c r="F166" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualResolveDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaFailureCode?</t>
         </is>
       </c>
       <c r="G166" s="4" t="inlineStr">
@@ -29807,7 +29827,7 @@
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>recallDateTime</t>
+          <t>slaEtaHit</t>
         </is>
       </c>
       <c r="B167" s="4" t="inlineStr">
@@ -29828,7 +29848,7 @@
       </c>
       <c r="F167" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.recallDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaHit?</t>
         </is>
       </c>
       <c r="G167" s="4" t="inlineStr">
@@ -29847,7 +29867,7 @@
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>actualRecallDateTime</t>
+          <t>slaResolveDateTime</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
@@ -29868,7 +29888,7 @@
       </c>
       <c r="F168" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualRecallDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveDateTime?</t>
         </is>
       </c>
       <c r="G168" s="4" t="inlineStr">
@@ -29887,12 +29907,12 @@
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>slaEtaClock</t>
+          <t>orderNumber</t>
         </is>
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
@@ -29908,7 +29928,7 @@
       </c>
       <c r="F169" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaClock?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderNumber?</t>
         </is>
       </c>
       <c r="G169" s="4" t="inlineStr">
@@ -29927,12 +29947,12 @@
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>slaResolveClock</t>
+          <t>requestId</t>
         </is>
       </c>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C170" s="4" t="inlineStr">
@@ -29948,7 +29968,7 @@
       </c>
       <c r="F170" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveClock?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.requestId?</t>
         </is>
       </c>
       <c r="G170" s="4" t="inlineStr">
@@ -29967,12 +29987,12 @@
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>slaFailureCode</t>
+          <t>customerCompanyCode</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
@@ -29988,7 +30008,7 @@
       </c>
       <c r="F171" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaFailureCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.customerCompanyCode?</t>
         </is>
       </c>
       <c r="G171" s="4" t="inlineStr">
@@ -30007,12 +30027,12 @@
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>slaEtaHit</t>
+          <t>orderStatus</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C172" s="4" t="inlineStr">
@@ -30028,7 +30048,7 @@
       </c>
       <c r="F172" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaHit?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStatus?</t>
         </is>
       </c>
       <c r="G172" s="4" t="inlineStr">
@@ -30047,12 +30067,12 @@
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>slaResolveDateTime</t>
+          <t>orderStartDatetime</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
@@ -30068,7 +30088,7 @@
       </c>
       <c r="F173" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStartDatetime?</t>
         </is>
       </c>
       <c r="G173" s="4" t="inlineStr">
@@ -30087,7 +30107,7 @@
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>orderNumber</t>
+          <t>siteCompanyCode</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
@@ -30108,7 +30128,7 @@
       </c>
       <c r="F174" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.siteCompanyCode?</t>
         </is>
       </c>
       <c r="G174" s="4" t="inlineStr">
@@ -30127,7 +30147,7 @@
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>requestId</t>
+          <t>repairType</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
@@ -30148,7 +30168,7 @@
       </c>
       <c r="F175" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.requestId?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairType?</t>
         </is>
       </c>
       <c r="G175" s="4" t="inlineStr">
@@ -30167,7 +30187,7 @@
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>customerCompanyCode</t>
+          <t>partsOrderDateTime</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
@@ -30188,7 +30208,7 @@
       </c>
       <c r="F176" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.customerCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsOrderDateTime?</t>
         </is>
       </c>
       <c r="G176" s="4" t="inlineStr">
@@ -30207,7 +30227,7 @@
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>orderStatus</t>
+          <t>partsReceivedDateTime</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
@@ -30228,7 +30248,7 @@
       </c>
       <c r="F177" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsReceivedDateTime?</t>
         </is>
       </c>
       <c r="G177" s="4" t="inlineStr">
@@ -30247,7 +30267,7 @@
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>orderStartDatetime</t>
+          <t>repairCode</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
@@ -30268,7 +30288,7 @@
       </c>
       <c r="F178" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStartDatetime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCode?</t>
         </is>
       </c>
       <c r="G178" s="4" t="inlineStr">
@@ -30287,7 +30307,7 @@
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>siteCompanyCode</t>
+          <t>repairCompany</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
@@ -30308,7 +30328,7 @@
       </c>
       <c r="F179" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.siteCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCompany?</t>
         </is>
       </c>
       <c r="G179" s="4" t="inlineStr">
@@ -30327,7 +30347,7 @@
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>repairType</t>
+          <t>raStatus</t>
         </is>
       </c>
       <c r="B180" s="4" t="inlineStr">
@@ -30348,7 +30368,7 @@
       </c>
       <c r="F180" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairType?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.raStatus?</t>
         </is>
       </c>
       <c r="G180" s="4" t="inlineStr">
@@ -30367,7 +30387,7 @@
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>partsOrderDateTime</t>
+          <t>Warehouse</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
@@ -30388,7 +30408,7 @@
       </c>
       <c r="F181" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsOrderDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.Warehouse?</t>
         </is>
       </c>
       <c r="G181" s="4" t="inlineStr">
@@ -30407,7 +30427,7 @@
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>partsReceivedDateTime</t>
+          <t>assignedPerson</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
@@ -30428,7 +30448,7 @@
       </c>
       <c r="F182" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsReceivedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.assignedPerson?</t>
         </is>
       </c>
       <c r="G182" s="4" t="inlineStr">
@@ -30447,7 +30467,7 @@
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>repairCode</t>
+          <t>resolvedDateTime</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
@@ -30468,7 +30488,7 @@
       </c>
       <c r="F183" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.resolvedDateTime?</t>
         </is>
       </c>
       <c r="G183" s="4" t="inlineStr">
@@ -30487,7 +30507,7 @@
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>repairCompany</t>
+          <t>serialNumber</t>
         </is>
       </c>
       <c r="B184" s="4" t="inlineStr">
@@ -30508,7 +30528,7 @@
       </c>
       <c r="F184" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCompany?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.serialNumber?</t>
         </is>
       </c>
       <c r="G184" s="4" t="inlineStr">
@@ -30527,7 +30547,7 @@
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>raStatus</t>
+          <t>quantityUsed</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
@@ -30548,7 +30568,7 @@
       </c>
       <c r="F185" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.raStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.quantityUsed?</t>
         </is>
       </c>
       <c r="G185" s="4" t="inlineStr">
@@ -30567,7 +30587,7 @@
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>Warehouse</t>
+          <t>deviceSerialNumber</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
@@ -30588,7 +30608,7 @@
       </c>
       <c r="F186" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.Warehouse?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.deviceSerialNumber?</t>
         </is>
       </c>
       <c r="G186" s="4" t="inlineStr">
@@ -30607,7 +30627,7 @@
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>assignedPerson</t>
+          <t>orderedPartId</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
@@ -30628,7 +30648,7 @@
       </c>
       <c r="F187" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.assignedPerson?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderedPartId?</t>
         </is>
       </c>
       <c r="G187" s="4" t="inlineStr">
@@ -30647,7 +30667,7 @@
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>resolvedDateTime</t>
+          <t>actualPartId</t>
         </is>
       </c>
       <c r="B188" s="4" t="inlineStr">
@@ -30668,7 +30688,7 @@
       </c>
       <c r="F188" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.resolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.actualPartId?</t>
         </is>
       </c>
       <c r="G188" s="4" t="inlineStr">
@@ -30687,12 +30707,12 @@
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>serialNumber</t>
+          <t>partCode</t>
         </is>
       </c>
       <c r="B189" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>PartCost</t>
         </is>
       </c>
       <c r="C189" s="4" t="inlineStr">
@@ -30708,7 +30728,7 @@
       </c>
       <c r="F189" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.serialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.partCode?</t>
         </is>
       </c>
       <c r="G189" s="4" t="inlineStr">
@@ -30727,12 +30747,12 @@
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>quantityUsed</t>
+          <t>cost</t>
         </is>
       </c>
       <c r="B190" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>PartCost</t>
         </is>
       </c>
       <c r="C190" s="4" t="inlineStr">
@@ -30748,7 +30768,7 @@
       </c>
       <c r="F190" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.quantityUsed?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.cost?</t>
         </is>
       </c>
       <c r="G190" s="4" t="inlineStr">
@@ -30767,12 +30787,12 @@
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>deviceSerialNumber</t>
+          <t>currencyCode</t>
         </is>
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>PartCost</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr">
@@ -30788,7 +30808,7 @@
       </c>
       <c r="F191" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.deviceSerialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.currencyCode?</t>
         </is>
       </c>
       <c r="G191" s="4" t="inlineStr">
@@ -30807,12 +30827,12 @@
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>orderedPartId</t>
+          <t>averageCost</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>PartCost</t>
         </is>
       </c>
       <c r="C192" s="4" t="inlineStr">
@@ -30828,7 +30848,7 @@
       </c>
       <c r="F192" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderedPartId?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.averageCost?</t>
         </is>
       </c>
       <c r="G192" s="4" t="inlineStr">
@@ -30847,12 +30867,12 @@
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>actualPartId</t>
+          <t>partCode</t>
         </is>
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C193" s="4" t="inlineStr">
@@ -30868,7 +30888,7 @@
       </c>
       <c r="F193" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.actualPartId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
         </is>
       </c>
       <c r="G193" s="4" t="inlineStr">
@@ -30887,12 +30907,12 @@
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>partCode</t>
+          <t>modelCode</t>
         </is>
       </c>
       <c r="B194" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C194" s="4" t="inlineStr">
@@ -30908,7 +30928,7 @@
       </c>
       <c r="F194" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.partCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
         </is>
       </c>
       <c r="G194" s="4" t="inlineStr">
@@ -30927,12 +30947,12 @@
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>modelDescription</t>
         </is>
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
@@ -30948,7 +30968,7 @@
       </c>
       <c r="F195" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.cost?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
         </is>
       </c>
       <c r="G195" s="4" t="inlineStr">
@@ -30967,12 +30987,12 @@
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>currencyCode</t>
+          <t>inventoryTransferImoId</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C196" s="4" t="inlineStr">
@@ -30988,7 +31008,7 @@
       </c>
       <c r="F196" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.currencyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.inventoryTransferImoId?</t>
         </is>
       </c>
       <c r="G196" s="4" t="inlineStr">
@@ -31007,12 +31027,12 @@
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>averageCost</t>
+          <t>createdDateTime</t>
         </is>
       </c>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr">
@@ -31028,7 +31048,7 @@
       </c>
       <c r="F197" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.averageCost?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.createdDateTime?</t>
         </is>
       </c>
       <c r="G197" s="4" t="inlineStr">
@@ -31047,12 +31067,12 @@
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>partCode</t>
+          <t>completedDateTime</t>
         </is>
       </c>
       <c r="B198" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C198" s="4" t="inlineStr">
@@ -31068,7 +31088,7 @@
       </c>
       <c r="F198" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.completedDateTime?</t>
         </is>
       </c>
       <c r="G198" s="4" t="inlineStr">
@@ -31087,12 +31107,12 @@
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>modelCode</t>
+          <t>fromWarehouseId</t>
         </is>
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C199" s="4" t="inlineStr">
@@ -31108,7 +31128,7 @@
       </c>
       <c r="F199" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.fromWarehouseId?</t>
         </is>
       </c>
       <c r="G199" s="4" t="inlineStr">
@@ -31127,12 +31147,12 @@
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>modelDescription</t>
+          <t>toWarehouseId</t>
         </is>
       </c>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C200" s="4" t="inlineStr">
@@ -31148,7 +31168,7 @@
       </c>
       <c r="F200" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.toWarehouseId?</t>
         </is>
       </c>
       <c r="G200" s="4" t="inlineStr">
@@ -31167,7 +31187,7 @@
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t>inventoryTransferImoId</t>
+          <t>demandStatus</t>
         </is>
       </c>
       <c r="B201" s="4" t="inlineStr">
@@ -31188,7 +31208,7 @@
       </c>
       <c r="F201" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.inventoryTransferImoId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.demandStatus?</t>
         </is>
       </c>
       <c r="G201" s="4" t="inlineStr">
@@ -31207,7 +31227,7 @@
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>createdDateTime</t>
+          <t>orderStatusIsClosed</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
@@ -31228,7 +31248,7 @@
       </c>
       <c r="F202" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.createdDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.orderStatusIsClosed?</t>
         </is>
       </c>
       <c r="G202" s="4" t="inlineStr">
@@ -31247,7 +31267,7 @@
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>completedDateTime</t>
+          <t>movementType</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
@@ -31268,7 +31288,7 @@
       </c>
       <c r="F203" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.completedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
         </is>
       </c>
       <c r="G203" s="4" t="inlineStr">
@@ -31287,7 +31307,7 @@
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>fromWarehouseId</t>
+          <t>addressId</t>
         </is>
       </c>
       <c r="B204" s="4" t="inlineStr">
@@ -31308,7 +31328,7 @@
       </c>
       <c r="F204" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.fromWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
         </is>
       </c>
       <c r="G204" s="4" t="inlineStr">
@@ -31327,7 +31347,7 @@
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>toWarehouseId</t>
+          <t>Bpart</t>
         </is>
       </c>
       <c r="B205" s="4" t="inlineStr">
@@ -31348,7 +31368,7 @@
       </c>
       <c r="F205" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.toWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.Bpart?</t>
         </is>
       </c>
       <c r="G205" s="4" t="inlineStr">
@@ -31367,7 +31387,7 @@
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
         <is>
-          <t>demandStatus</t>
+          <t>quantity</t>
         </is>
       </c>
       <c r="B206" s="4" t="inlineStr">
@@ -31388,7 +31408,7 @@
       </c>
       <c r="F206" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.demandStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.quantity?</t>
         </is>
       </c>
       <c r="G206" s="4" t="inlineStr">
@@ -31407,7 +31427,7 @@
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>orderStatusIsClosed</t>
+          <t>shipListCode</t>
         </is>
       </c>
       <c r="B207" s="4" t="inlineStr">
@@ -31428,7 +31448,7 @@
       </c>
       <c r="F207" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.orderStatusIsClosed?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
         </is>
       </c>
       <c r="G207" s="4" t="inlineStr">
@@ -31445,54 +31465,54 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="4" t="inlineStr">
-        <is>
-          <t>movementType</t>
-        </is>
-      </c>
-      <c r="B208" s="4" t="inlineStr">
-        <is>
-          <t>InventoryTransfers</t>
-        </is>
-      </c>
-      <c r="C208" s="4" t="inlineStr">
+      <c r="A208" s="3" t="inlineStr">
+        <is>
+          <t>demandStatus</t>
+        </is>
+      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t>PurchaseOrders</t>
+        </is>
+      </c>
+      <c r="C208" s="3" t="inlineStr">
         <is>
           <t>Planning V2 template</t>
         </is>
       </c>
-      <c r="D208" s="4" t="inlineStr"/>
-      <c r="E208" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F208" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
-        </is>
-      </c>
-      <c r="G208" s="4" t="inlineStr">
+      <c r="D208" s="3" t="inlineStr"/>
+      <c r="E208" s="3" t="inlineStr">
+        <is>
+          <t>Review required</t>
+        </is>
+      </c>
+      <c r="F208" s="3" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
+        </is>
+      </c>
+      <c r="G208" s="3" t="inlineStr">
         <is>
           <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
         </is>
       </c>
-      <c r="H208" s="4" t="inlineStr"/>
-      <c r="I208" s="4" t="inlineStr"/>
-      <c r="J208" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="H208" s="3" t="inlineStr"/>
+      <c r="I208" s="3" t="inlineStr"/>
+      <c r="J208" s="3" t="inlineStr">
+        <is>
+          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.DocNum and part/SPL Master evidence also matches; current export needs reconciliation.</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t>addressId</t>
+          <t>partType</t>
         </is>
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C209" s="4" t="inlineStr">
@@ -31508,7 +31528,7 @@
       </c>
       <c r="F209" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.partType?</t>
         </is>
       </c>
       <c r="G209" s="4" t="inlineStr">
@@ -31527,12 +31547,12 @@
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
         <is>
-          <t>Bpart</t>
+          <t>partTypeDescription</t>
         </is>
       </c>
       <c r="B210" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C210" s="4" t="inlineStr">
@@ -31548,7 +31568,7 @@
       </c>
       <c r="F210" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.Bpart?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeDescription?</t>
         </is>
       </c>
       <c r="G210" s="4" t="inlineStr">
@@ -31567,12 +31587,12 @@
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>isReworkable</t>
         </is>
       </c>
       <c r="B211" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C211" s="4" t="inlineStr">
@@ -31588,7 +31608,7 @@
       </c>
       <c r="F211" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.quantity?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.isReworkable?</t>
         </is>
       </c>
       <c r="G211" s="4" t="inlineStr">
@@ -31607,12 +31627,12 @@
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
         <is>
-          <t>shipListCode</t>
+          <t>partNumber</t>
         </is>
       </c>
       <c r="B212" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C212" s="4" t="inlineStr">
@@ -31628,7 +31648,7 @@
       </c>
       <c r="F212" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
         </is>
       </c>
       <c r="G212" s="4" t="inlineStr">
@@ -31645,54 +31665,54 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="3" t="inlineStr">
-        <is>
-          <t>demandStatus</t>
-        </is>
-      </c>
-      <c r="B213" s="3" t="inlineStr">
-        <is>
-          <t>PurchaseOrders</t>
-        </is>
-      </c>
-      <c r="C213" s="3" t="inlineStr">
+      <c r="A213" s="4" t="inlineStr">
+        <is>
+          <t>unitOfMeasure</t>
+        </is>
+      </c>
+      <c r="B213" s="4" t="inlineStr">
+        <is>
+          <t>Yields</t>
+        </is>
+      </c>
+      <c r="C213" s="4" t="inlineStr">
         <is>
           <t>Planning V2 template</t>
         </is>
       </c>
-      <c r="D213" s="3" t="inlineStr"/>
-      <c r="E213" s="3" t="inlineStr">
-        <is>
-          <t>Review required</t>
-        </is>
-      </c>
-      <c r="F213" s="3" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
-        </is>
-      </c>
-      <c r="G213" s="3" t="inlineStr">
+      <c r="D213" s="4" t="inlineStr"/>
+      <c r="E213" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F213" s="4" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
+        </is>
+      </c>
+      <c r="G213" s="4" t="inlineStr">
         <is>
           <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
         </is>
       </c>
-      <c r="H213" s="3" t="inlineStr"/>
-      <c r="I213" s="3" t="inlineStr"/>
-      <c r="J213" s="3" t="inlineStr">
-        <is>
-          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.DocNum and part/SPL Master evidence also matches; current export needs reconciliation.</t>
+      <c r="H213" s="4" t="inlineStr"/>
+      <c r="I213" s="4" t="inlineStr"/>
+      <c r="J213" s="4" t="inlineStr">
+        <is>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
         <is>
-          <t>partType</t>
+          <t>yield</t>
         </is>
       </c>
       <c r="B214" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C214" s="4" t="inlineStr">
@@ -31708,7 +31728,7 @@
       </c>
       <c r="F214" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partType?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
         </is>
       </c>
       <c r="G214" s="4" t="inlineStr">
@@ -31727,12 +31747,12 @@
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
         <is>
-          <t>partTypeDescription</t>
+          <t>Secondary TO</t>
         </is>
       </c>
       <c r="B215" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C215" s="4" t="inlineStr">
@@ -31748,7 +31768,7 @@
       </c>
       <c r="F215" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeDescription?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary TO?</t>
         </is>
       </c>
       <c r="G215" s="4" t="inlineStr">
@@ -31767,12 +31787,12 @@
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
         <is>
-          <t>isReworkable</t>
+          <t>Secondary FROM</t>
         </is>
       </c>
       <c r="B216" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C216" s="4" t="inlineStr">
@@ -31788,7 +31808,7 @@
       </c>
       <c r="F216" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.isReworkable?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary FROM?</t>
         </is>
       </c>
       <c r="G216" s="4" t="inlineStr">
@@ -31807,12 +31827,12 @@
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t>partNumber</t>
+          <t>Cross TO</t>
         </is>
       </c>
       <c r="B217" s="4" t="inlineStr">
         <is>
-          <t>Yields</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C217" s="4" t="inlineStr">
@@ -31828,7 +31848,7 @@
       </c>
       <c r="F217" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross TO?</t>
         </is>
       </c>
       <c r="G217" s="4" t="inlineStr">
@@ -31847,12 +31867,12 @@
     <row r="218">
       <c r="A218" s="4" t="inlineStr">
         <is>
-          <t>unitOfMeasure</t>
+          <t>Cross FROM</t>
         </is>
       </c>
       <c r="B218" s="4" t="inlineStr">
         <is>
-          <t>Yields</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C218" s="4" t="inlineStr">
@@ -31868,7 +31888,7 @@
       </c>
       <c r="F218" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross FROM?</t>
         </is>
       </c>
       <c r="G218" s="4" t="inlineStr">
@@ -31887,12 +31907,12 @@
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t>yield</t>
+          <t>Primary TO</t>
         </is>
       </c>
       <c r="B219" s="4" t="inlineStr">
         <is>
-          <t>Yields</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C219" s="4" t="inlineStr">
@@ -31908,7 +31928,7 @@
       </c>
       <c r="F219" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Primary TO?</t>
         </is>
       </c>
       <c r="G219" s="4" t="inlineStr">
@@ -31924,208 +31944,8 @@
         </is>
       </c>
     </row>
-    <row r="220">
-      <c r="A220" s="4" t="inlineStr">
-        <is>
-          <t>Secondary TO</t>
-        </is>
-      </c>
-      <c r="B220" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C220" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D220" s="4" t="inlineStr"/>
-      <c r="E220" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F220" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary TO?</t>
-        </is>
-      </c>
-      <c r="G220" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H220" s="4" t="inlineStr"/>
-      <c r="I220" s="4" t="inlineStr"/>
-      <c r="J220" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" s="4" t="inlineStr">
-        <is>
-          <t>Secondary FROM</t>
-        </is>
-      </c>
-      <c r="B221" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C221" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D221" s="4" t="inlineStr"/>
-      <c r="E221" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F221" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary FROM?</t>
-        </is>
-      </c>
-      <c r="G221" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H221" s="4" t="inlineStr"/>
-      <c r="I221" s="4" t="inlineStr"/>
-      <c r="J221" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" s="4" t="inlineStr">
-        <is>
-          <t>Cross TO</t>
-        </is>
-      </c>
-      <c r="B222" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C222" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D222" s="4" t="inlineStr"/>
-      <c r="E222" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F222" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross TO?</t>
-        </is>
-      </c>
-      <c r="G222" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H222" s="4" t="inlineStr"/>
-      <c r="I222" s="4" t="inlineStr"/>
-      <c r="J222" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" s="4" t="inlineStr">
-        <is>
-          <t>Cross FROM</t>
-        </is>
-      </c>
-      <c r="B223" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C223" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D223" s="4" t="inlineStr"/>
-      <c r="E223" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F223" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross FROM?</t>
-        </is>
-      </c>
-      <c r="G223" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H223" s="4" t="inlineStr"/>
-      <c r="I223" s="4" t="inlineStr"/>
-      <c r="J223" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" s="4" t="inlineStr">
-        <is>
-          <t>Primary TO</t>
-        </is>
-      </c>
-      <c r="B224" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C224" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D224" s="4" t="inlineStr"/>
-      <c r="E224" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F224" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Primary TO?</t>
-        </is>
-      </c>
-      <c r="G224" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H224" s="4" t="inlineStr"/>
-      <c r="I224" s="4" t="inlineStr"/>
-      <c r="J224" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J224"/>
+  <autoFilter ref="A1:J219"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -32753,7 +32573,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>OrderType; customerCompanyCode; orderStartDatetime; orderStatus; resolvedDateTime; serialNumber; relCompanyId; assignedPersonCode; deviceSerialNumber</t>
+          <t>OrderType; resolvedDateTime; relCompanyId; assignedPersonCode</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore delivery note usage as source of truth
</commit_message>
<xml_diff>
--- a/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
+++ b/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Target Fields'!$A$1:$S$151</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Template Fields'!$A$1:$H$177</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Evidence'!$A$1:$D$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$J$219</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$J$224</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Output Objects'!$A$1:$E$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Missing Important Fields'!$A$1:$E$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'SAP Investigation Log'!$A$1:$E$10</definedName>
@@ -244,8 +244,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:J219" headerRowCount="1">
-  <autoFilter ref="A1:J219"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:J224" headerRowCount="1">
+  <autoFilter ref="A1:J224"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Field"/>
     <tableColumn id="2" name="Object"/>
@@ -17922,7 +17922,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>CoCre8 HelpDesk issue tracker:Call Number</t>
+          <t>Stock Audit Report 3Y:Document for DN rows</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -18005,128 +18005,116 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="inlineStr">
+      <c r="A83" s="4" t="inlineStr">
         <is>
           <t>PartsUsage</t>
         </is>
       </c>
-      <c r="B83" s="2" t="inlineStr">
+      <c r="B83" s="4" t="inlineStr">
         <is>
           <t>customerCompanyCode</t>
         </is>
       </c>
-      <c r="C83" s="2" t="inlineStr">
+      <c r="C83" s="4" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D83" s="2" t="inlineStr">
+      <c r="D83" s="4" t="inlineStr">
         <is>
           <t>Canonical header from PartsUsage.xlsx</t>
         </is>
       </c>
-      <c r="E83" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="F83" s="2" t="inlineStr">
-        <is>
-          <t>CoCre8 HelpDesk issue tracker:CustomerNormalized/Customer</t>
-        </is>
-      </c>
-      <c r="G83" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H83" s="2" t="inlineStr">
-        <is>
-          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr"/>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="inlineStr">
+      <c r="A84" s="4" t="inlineStr">
         <is>
           <t>PartsUsage</t>
         </is>
       </c>
-      <c r="B84" s="2" t="inlineStr">
+      <c r="B84" s="4" t="inlineStr">
         <is>
           <t>orderStartDatetime</t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr">
+      <c r="C84" s="4" t="inlineStr">
         <is>
           <t>DateTime</t>
         </is>
       </c>
-      <c r="D84" s="2" t="inlineStr">
+      <c r="D84" s="4" t="inlineStr">
         <is>
           <t>Canonical header from PartsUsage.xlsx</t>
         </is>
       </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="F84" s="2" t="inlineStr">
-        <is>
-          <t>CoCre8 HelpDesk issue tracker:Created</t>
-        </is>
-      </c>
-      <c r="G84" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
-        <is>
-          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr"/>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="inlineStr">
+        <is>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="inlineStr">
+      <c r="A85" s="4" t="inlineStr">
         <is>
           <t>PartsUsage</t>
         </is>
       </c>
-      <c r="B85" s="2" t="inlineStr">
+      <c r="B85" s="4" t="inlineStr">
         <is>
           <t>orderStatus</t>
         </is>
       </c>
-      <c r="C85" s="2" t="inlineStr">
+      <c r="C85" s="4" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D85" s="2" t="inlineStr">
+      <c r="D85" s="4" t="inlineStr">
         <is>
           <t>Canonical header from PartsUsage.xlsx</t>
         </is>
       </c>
-      <c r="E85" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="F85" s="2" t="inlineStr">
-        <is>
-          <t>CoCre8 HelpDesk issue tracker:Status</t>
-        </is>
-      </c>
-      <c r="G85" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H85" s="2" t="inlineStr">
-        <is>
-          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr"/>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
@@ -18196,7 +18184,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>CoCre8 HelpDesk issue tracker:DispatchPartNo when present, otherwise Part Nr</t>
+          <t>Stock Audit Report 3Y:Item No.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -18211,44 +18199,40 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="inlineStr">
+      <c r="A88" s="4" t="inlineStr">
         <is>
           <t>PartsUsage</t>
         </is>
       </c>
-      <c r="B88" s="2" t="inlineStr">
+      <c r="B88" s="4" t="inlineStr">
         <is>
           <t>serialNumber</t>
         </is>
       </c>
-      <c r="C88" s="2" t="inlineStr">
+      <c r="C88" s="4" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D88" s="2" t="inlineStr">
+      <c r="D88" s="4" t="inlineStr">
         <is>
           <t>Canonical header from PartsUsage.xlsx</t>
         </is>
       </c>
-      <c r="E88" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="F88" s="2" t="inlineStr">
-        <is>
-          <t>CoCre8 HelpDesk issue tracker:Serial Nr</t>
-        </is>
-      </c>
-      <c r="G88" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H88" s="2" t="inlineStr">
-        <is>
-          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F88" s="4" t="inlineStr"/>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H88" s="4" t="inlineStr">
+        <is>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
@@ -18280,7 +18264,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>CoCre8 HelpDesk issue tracker:Quantity</t>
+          <t>Stock Audit Report 3Y:absolute Quantity for negative DN rows</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -18360,7 +18344,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>CoCre8 HelpDesk issue tracker:Created used as demand/usage date</t>
+          <t>Stock Audit Report 3Y:Posting Date</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -18402,7 +18386,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>CoCre8 HelpDesk issue tracker:DispatchWarehouse</t>
+          <t>Stock Audit Report 3Y:Whse</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -18455,44 +18439,40 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="inlineStr">
+      <c r="A94" s="4" t="inlineStr">
         <is>
           <t>PartsUsage</t>
         </is>
       </c>
-      <c r="B94" s="2" t="inlineStr">
+      <c r="B94" s="4" t="inlineStr">
         <is>
           <t>deviceSerialNumber</t>
         </is>
       </c>
-      <c r="C94" s="2" t="inlineStr">
+      <c r="C94" s="4" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D94" s="2" t="inlineStr">
+      <c r="D94" s="4" t="inlineStr">
         <is>
           <t>Canonical header from PartsUsage.xlsx</t>
         </is>
       </c>
-      <c r="E94" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="F94" s="2" t="inlineStr">
-        <is>
-          <t>CoCre8 HelpDesk issue tracker:Serial Nr</t>
-        </is>
-      </c>
-      <c r="G94" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H94" s="2" t="inlineStr">
-        <is>
-          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
+      <c r="E94" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F94" s="4" t="inlineStr"/>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H94" s="4" t="inlineStr">
+        <is>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
@@ -18520,7 +18500,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>CoCre8 HelpDesk issue tracker:SPLMaster or masters.csv by part</t>
+          <t>Reference masters.csv:SPL Master by used part</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -21969,7 +21949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J219"/>
+  <dimension ref="A1:J224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -29267,7 +29247,7 @@
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>resolvedDateTime</t>
+          <t>customerCompanyCode</t>
         </is>
       </c>
       <c r="B153" s="4" t="inlineStr">
@@ -29288,7 +29268,7 @@
       </c>
       <c r="F153" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.resolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.customerCompanyCode?</t>
         </is>
       </c>
       <c r="G153" s="4" t="inlineStr">
@@ -29307,7 +29287,7 @@
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>relCompanyId</t>
+          <t>orderStartDatetime</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
@@ -29328,7 +29308,7 @@
       </c>
       <c r="F154" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.relCompanyId?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStartDatetime?</t>
         </is>
       </c>
       <c r="G154" s="4" t="inlineStr">
@@ -29347,7 +29327,7 @@
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>assignedPersonCode</t>
+          <t>orderStatus</t>
         </is>
       </c>
       <c r="B155" s="4" t="inlineStr">
@@ -29368,7 +29348,7 @@
       </c>
       <c r="F155" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.assignedPersonCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStatus?</t>
         </is>
       </c>
       <c r="G155" s="4" t="inlineStr">
@@ -29387,12 +29367,12 @@
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>orderNumber</t>
+          <t>resolvedDateTime</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C156" s="4" t="inlineStr">
@@ -29408,7 +29388,7 @@
       </c>
       <c r="F156" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.orderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.resolvedDateTime?</t>
         </is>
       </c>
       <c r="G156" s="4" t="inlineStr">
@@ -29427,12 +29407,12 @@
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>RequestID</t>
+          <t>serialNumber</t>
         </is>
       </c>
       <c r="B157" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C157" s="4" t="inlineStr">
@@ -29448,7 +29428,7 @@
       </c>
       <c r="F157" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.RequestID?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.serialNumber?</t>
         </is>
       </c>
       <c r="G157" s="4" t="inlineStr">
@@ -29467,12 +29447,12 @@
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>relCompanyId</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C158" s="4" t="inlineStr">
@@ -29488,7 +29468,7 @@
       </c>
       <c r="F158" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.location?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.relCompanyId?</t>
         </is>
       </c>
       <c r="G158" s="4" t="inlineStr">
@@ -29507,12 +29487,12 @@
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>eta</t>
+          <t>assignedPersonCode</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C159" s="4" t="inlineStr">
@@ -29528,7 +29508,7 @@
       </c>
       <c r="F159" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.eta?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.assignedPersonCode?</t>
         </is>
       </c>
       <c r="G159" s="4" t="inlineStr">
@@ -29547,12 +29527,12 @@
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>actualEta</t>
+          <t>deviceSerialNumber</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C160" s="4" t="inlineStr">
@@ -29568,7 +29548,7 @@
       </c>
       <c r="F160" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualEta?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.deviceSerialNumber?</t>
         </is>
       </c>
       <c r="G160" s="4" t="inlineStr">
@@ -29587,7 +29567,7 @@
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>actualResolveDateTime</t>
+          <t>orderNumber</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
@@ -29608,7 +29588,7 @@
       </c>
       <c r="F161" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualResolveDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.orderNumber?</t>
         </is>
       </c>
       <c r="G161" s="4" t="inlineStr">
@@ -29627,7 +29607,7 @@
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>recallDateTime</t>
+          <t>RequestID</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
@@ -29648,7 +29628,7 @@
       </c>
       <c r="F162" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.recallDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.RequestID?</t>
         </is>
       </c>
       <c r="G162" s="4" t="inlineStr">
@@ -29667,7 +29647,7 @@
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>actualRecallDateTime</t>
+          <t>location</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
@@ -29688,7 +29668,7 @@
       </c>
       <c r="F163" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualRecallDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.location?</t>
         </is>
       </c>
       <c r="G163" s="4" t="inlineStr">
@@ -29707,7 +29687,7 @@
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>slaEtaClock</t>
+          <t>eta</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
@@ -29728,7 +29708,7 @@
       </c>
       <c r="F164" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaClock?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.eta?</t>
         </is>
       </c>
       <c r="G164" s="4" t="inlineStr">
@@ -29747,7 +29727,7 @@
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t>slaResolveClock</t>
+          <t>actualEta</t>
         </is>
       </c>
       <c r="B165" s="4" t="inlineStr">
@@ -29768,7 +29748,7 @@
       </c>
       <c r="F165" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveClock?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualEta?</t>
         </is>
       </c>
       <c r="G165" s="4" t="inlineStr">
@@ -29787,7 +29767,7 @@
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>slaFailureCode</t>
+          <t>actualResolveDateTime</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
@@ -29808,7 +29788,7 @@
       </c>
       <c r="F166" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaFailureCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualResolveDateTime?</t>
         </is>
       </c>
       <c r="G166" s="4" t="inlineStr">
@@ -29827,7 +29807,7 @@
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>slaEtaHit</t>
+          <t>recallDateTime</t>
         </is>
       </c>
       <c r="B167" s="4" t="inlineStr">
@@ -29848,7 +29828,7 @@
       </c>
       <c r="F167" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaHit?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.recallDateTime?</t>
         </is>
       </c>
       <c r="G167" s="4" t="inlineStr">
@@ -29867,7 +29847,7 @@
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>slaResolveDateTime</t>
+          <t>actualRecallDateTime</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
@@ -29888,7 +29868,7 @@
       </c>
       <c r="F168" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualRecallDateTime?</t>
         </is>
       </c>
       <c r="G168" s="4" t="inlineStr">
@@ -29907,12 +29887,12 @@
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>orderNumber</t>
+          <t>slaEtaClock</t>
         </is>
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
@@ -29928,7 +29908,7 @@
       </c>
       <c r="F169" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaClock?</t>
         </is>
       </c>
       <c r="G169" s="4" t="inlineStr">
@@ -29947,12 +29927,12 @@
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>requestId</t>
+          <t>slaResolveClock</t>
         </is>
       </c>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C170" s="4" t="inlineStr">
@@ -29968,7 +29948,7 @@
       </c>
       <c r="F170" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.requestId?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveClock?</t>
         </is>
       </c>
       <c r="G170" s="4" t="inlineStr">
@@ -29987,12 +29967,12 @@
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>customerCompanyCode</t>
+          <t>slaFailureCode</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
@@ -30008,7 +29988,7 @@
       </c>
       <c r="F171" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.customerCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaFailureCode?</t>
         </is>
       </c>
       <c r="G171" s="4" t="inlineStr">
@@ -30027,12 +30007,12 @@
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>orderStatus</t>
+          <t>slaEtaHit</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C172" s="4" t="inlineStr">
@@ -30048,7 +30028,7 @@
       </c>
       <c r="F172" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaHit?</t>
         </is>
       </c>
       <c r="G172" s="4" t="inlineStr">
@@ -30067,12 +30047,12 @@
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>orderStartDatetime</t>
+          <t>slaResolveDateTime</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
@@ -30088,7 +30068,7 @@
       </c>
       <c r="F173" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStartDatetime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveDateTime?</t>
         </is>
       </c>
       <c r="G173" s="4" t="inlineStr">
@@ -30107,7 +30087,7 @@
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>siteCompanyCode</t>
+          <t>orderNumber</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
@@ -30128,7 +30108,7 @@
       </c>
       <c r="F174" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.siteCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderNumber?</t>
         </is>
       </c>
       <c r="G174" s="4" t="inlineStr">
@@ -30147,7 +30127,7 @@
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>repairType</t>
+          <t>requestId</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
@@ -30168,7 +30148,7 @@
       </c>
       <c r="F175" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairType?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.requestId?</t>
         </is>
       </c>
       <c r="G175" s="4" t="inlineStr">
@@ -30187,7 +30167,7 @@
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>partsOrderDateTime</t>
+          <t>customerCompanyCode</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
@@ -30208,7 +30188,7 @@
       </c>
       <c r="F176" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsOrderDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.customerCompanyCode?</t>
         </is>
       </c>
       <c r="G176" s="4" t="inlineStr">
@@ -30227,7 +30207,7 @@
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>partsReceivedDateTime</t>
+          <t>orderStatus</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
@@ -30248,7 +30228,7 @@
       </c>
       <c r="F177" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsReceivedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStatus?</t>
         </is>
       </c>
       <c r="G177" s="4" t="inlineStr">
@@ -30267,7 +30247,7 @@
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>repairCode</t>
+          <t>orderStartDatetime</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
@@ -30288,7 +30268,7 @@
       </c>
       <c r="F178" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStartDatetime?</t>
         </is>
       </c>
       <c r="G178" s="4" t="inlineStr">
@@ -30307,7 +30287,7 @@
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>repairCompany</t>
+          <t>siteCompanyCode</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
@@ -30328,7 +30308,7 @@
       </c>
       <c r="F179" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCompany?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.siteCompanyCode?</t>
         </is>
       </c>
       <c r="G179" s="4" t="inlineStr">
@@ -30347,7 +30327,7 @@
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>raStatus</t>
+          <t>repairType</t>
         </is>
       </c>
       <c r="B180" s="4" t="inlineStr">
@@ -30368,7 +30348,7 @@
       </c>
       <c r="F180" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.raStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairType?</t>
         </is>
       </c>
       <c r="G180" s="4" t="inlineStr">
@@ -30387,7 +30367,7 @@
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>Warehouse</t>
+          <t>partsOrderDateTime</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
@@ -30408,7 +30388,7 @@
       </c>
       <c r="F181" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.Warehouse?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsOrderDateTime?</t>
         </is>
       </c>
       <c r="G181" s="4" t="inlineStr">
@@ -30427,7 +30407,7 @@
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>assignedPerson</t>
+          <t>partsReceivedDateTime</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
@@ -30448,7 +30428,7 @@
       </c>
       <c r="F182" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.assignedPerson?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsReceivedDateTime?</t>
         </is>
       </c>
       <c r="G182" s="4" t="inlineStr">
@@ -30467,7 +30447,7 @@
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>resolvedDateTime</t>
+          <t>repairCode</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
@@ -30488,7 +30468,7 @@
       </c>
       <c r="F183" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.resolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCode?</t>
         </is>
       </c>
       <c r="G183" s="4" t="inlineStr">
@@ -30507,7 +30487,7 @@
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>serialNumber</t>
+          <t>repairCompany</t>
         </is>
       </c>
       <c r="B184" s="4" t="inlineStr">
@@ -30528,7 +30508,7 @@
       </c>
       <c r="F184" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.serialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCompany?</t>
         </is>
       </c>
       <c r="G184" s="4" t="inlineStr">
@@ -30547,7 +30527,7 @@
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>quantityUsed</t>
+          <t>raStatus</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
@@ -30568,7 +30548,7 @@
       </c>
       <c r="F185" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.quantityUsed?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.raStatus?</t>
         </is>
       </c>
       <c r="G185" s="4" t="inlineStr">
@@ -30587,7 +30567,7 @@
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>deviceSerialNumber</t>
+          <t>Warehouse</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
@@ -30608,7 +30588,7 @@
       </c>
       <c r="F186" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.deviceSerialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.Warehouse?</t>
         </is>
       </c>
       <c r="G186" s="4" t="inlineStr">
@@ -30627,7 +30607,7 @@
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>orderedPartId</t>
+          <t>assignedPerson</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
@@ -30648,7 +30628,7 @@
       </c>
       <c r="F187" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderedPartId?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.assignedPerson?</t>
         </is>
       </c>
       <c r="G187" s="4" t="inlineStr">
@@ -30667,7 +30647,7 @@
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>actualPartId</t>
+          <t>resolvedDateTime</t>
         </is>
       </c>
       <c r="B188" s="4" t="inlineStr">
@@ -30688,7 +30668,7 @@
       </c>
       <c r="F188" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.actualPartId?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.resolvedDateTime?</t>
         </is>
       </c>
       <c r="G188" s="4" t="inlineStr">
@@ -30707,12 +30687,12 @@
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>partCode</t>
+          <t>serialNumber</t>
         </is>
       </c>
       <c r="B189" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C189" s="4" t="inlineStr">
@@ -30728,7 +30708,7 @@
       </c>
       <c r="F189" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.partCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.serialNumber?</t>
         </is>
       </c>
       <c r="G189" s="4" t="inlineStr">
@@ -30747,12 +30727,12 @@
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>quantityUsed</t>
         </is>
       </c>
       <c r="B190" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C190" s="4" t="inlineStr">
@@ -30768,7 +30748,7 @@
       </c>
       <c r="F190" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.cost?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.quantityUsed?</t>
         </is>
       </c>
       <c r="G190" s="4" t="inlineStr">
@@ -30787,12 +30767,12 @@
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>currencyCode</t>
+          <t>deviceSerialNumber</t>
         </is>
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr">
@@ -30808,7 +30788,7 @@
       </c>
       <c r="F191" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.currencyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.deviceSerialNumber?</t>
         </is>
       </c>
       <c r="G191" s="4" t="inlineStr">
@@ -30827,12 +30807,12 @@
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>averageCost</t>
+          <t>orderedPartId</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C192" s="4" t="inlineStr">
@@ -30848,7 +30828,7 @@
       </c>
       <c r="F192" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.averageCost?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderedPartId?</t>
         </is>
       </c>
       <c r="G192" s="4" t="inlineStr">
@@ -30867,12 +30847,12 @@
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>partCode</t>
+          <t>actualPartId</t>
         </is>
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C193" s="4" t="inlineStr">
@@ -30888,7 +30868,7 @@
       </c>
       <c r="F193" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.actualPartId?</t>
         </is>
       </c>
       <c r="G193" s="4" t="inlineStr">
@@ -30907,12 +30887,12 @@
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>modelCode</t>
+          <t>partCode</t>
         </is>
       </c>
       <c r="B194" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>PartCost</t>
         </is>
       </c>
       <c r="C194" s="4" t="inlineStr">
@@ -30928,7 +30908,7 @@
       </c>
       <c r="F194" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.partCode?</t>
         </is>
       </c>
       <c r="G194" s="4" t="inlineStr">
@@ -30947,12 +30927,12 @@
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>modelDescription</t>
+          <t>cost</t>
         </is>
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>PartCost</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
@@ -30968,7 +30948,7 @@
       </c>
       <c r="F195" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.cost?</t>
         </is>
       </c>
       <c r="G195" s="4" t="inlineStr">
@@ -30987,12 +30967,12 @@
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>inventoryTransferImoId</t>
+          <t>currencyCode</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartCost</t>
         </is>
       </c>
       <c r="C196" s="4" t="inlineStr">
@@ -31008,7 +30988,7 @@
       </c>
       <c r="F196" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.inventoryTransferImoId?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.currencyCode?</t>
         </is>
       </c>
       <c r="G196" s="4" t="inlineStr">
@@ -31027,12 +31007,12 @@
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>createdDateTime</t>
+          <t>averageCost</t>
         </is>
       </c>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartCost</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr">
@@ -31048,7 +31028,7 @@
       </c>
       <c r="F197" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.createdDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.averageCost?</t>
         </is>
       </c>
       <c r="G197" s="4" t="inlineStr">
@@ -31067,12 +31047,12 @@
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>completedDateTime</t>
+          <t>partCode</t>
         </is>
       </c>
       <c r="B198" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C198" s="4" t="inlineStr">
@@ -31088,7 +31068,7 @@
       </c>
       <c r="F198" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.completedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
         </is>
       </c>
       <c r="G198" s="4" t="inlineStr">
@@ -31107,12 +31087,12 @@
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>fromWarehouseId</t>
+          <t>modelCode</t>
         </is>
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C199" s="4" t="inlineStr">
@@ -31128,7 +31108,7 @@
       </c>
       <c r="F199" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.fromWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
         </is>
       </c>
       <c r="G199" s="4" t="inlineStr">
@@ -31147,12 +31127,12 @@
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>toWarehouseId</t>
+          <t>modelDescription</t>
         </is>
       </c>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C200" s="4" t="inlineStr">
@@ -31168,7 +31148,7 @@
       </c>
       <c r="F200" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.toWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
         </is>
       </c>
       <c r="G200" s="4" t="inlineStr">
@@ -31187,7 +31167,7 @@
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t>demandStatus</t>
+          <t>inventoryTransferImoId</t>
         </is>
       </c>
       <c r="B201" s="4" t="inlineStr">
@@ -31208,7 +31188,7 @@
       </c>
       <c r="F201" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.demandStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.inventoryTransferImoId?</t>
         </is>
       </c>
       <c r="G201" s="4" t="inlineStr">
@@ -31227,7 +31207,7 @@
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>orderStatusIsClosed</t>
+          <t>createdDateTime</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
@@ -31248,7 +31228,7 @@
       </c>
       <c r="F202" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.orderStatusIsClosed?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.createdDateTime?</t>
         </is>
       </c>
       <c r="G202" s="4" t="inlineStr">
@@ -31267,7 +31247,7 @@
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>movementType</t>
+          <t>completedDateTime</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
@@ -31288,7 +31268,7 @@
       </c>
       <c r="F203" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.completedDateTime?</t>
         </is>
       </c>
       <c r="G203" s="4" t="inlineStr">
@@ -31307,7 +31287,7 @@
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>addressId</t>
+          <t>fromWarehouseId</t>
         </is>
       </c>
       <c r="B204" s="4" t="inlineStr">
@@ -31328,7 +31308,7 @@
       </c>
       <c r="F204" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.fromWarehouseId?</t>
         </is>
       </c>
       <c r="G204" s="4" t="inlineStr">
@@ -31347,7 +31327,7 @@
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>Bpart</t>
+          <t>toWarehouseId</t>
         </is>
       </c>
       <c r="B205" s="4" t="inlineStr">
@@ -31368,7 +31348,7 @@
       </c>
       <c r="F205" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.Bpart?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.toWarehouseId?</t>
         </is>
       </c>
       <c r="G205" s="4" t="inlineStr">
@@ -31387,7 +31367,7 @@
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>demandStatus</t>
         </is>
       </c>
       <c r="B206" s="4" t="inlineStr">
@@ -31408,7 +31388,7 @@
       </c>
       <c r="F206" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.quantity?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.demandStatus?</t>
         </is>
       </c>
       <c r="G206" s="4" t="inlineStr">
@@ -31427,7 +31407,7 @@
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>shipListCode</t>
+          <t>orderStatusIsClosed</t>
         </is>
       </c>
       <c r="B207" s="4" t="inlineStr">
@@ -31448,7 +31428,7 @@
       </c>
       <c r="F207" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.orderStatusIsClosed?</t>
         </is>
       </c>
       <c r="G207" s="4" t="inlineStr">
@@ -31465,54 +31445,54 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="3" t="inlineStr">
-        <is>
-          <t>demandStatus</t>
-        </is>
-      </c>
-      <c r="B208" s="3" t="inlineStr">
-        <is>
-          <t>PurchaseOrders</t>
-        </is>
-      </c>
-      <c r="C208" s="3" t="inlineStr">
+      <c r="A208" s="4" t="inlineStr">
+        <is>
+          <t>movementType</t>
+        </is>
+      </c>
+      <c r="B208" s="4" t="inlineStr">
+        <is>
+          <t>InventoryTransfers</t>
+        </is>
+      </c>
+      <c r="C208" s="4" t="inlineStr">
         <is>
           <t>Planning V2 template</t>
         </is>
       </c>
-      <c r="D208" s="3" t="inlineStr"/>
-      <c r="E208" s="3" t="inlineStr">
-        <is>
-          <t>Review required</t>
-        </is>
-      </c>
-      <c r="F208" s="3" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
-        </is>
-      </c>
-      <c r="G208" s="3" t="inlineStr">
+      <c r="D208" s="4" t="inlineStr"/>
+      <c r="E208" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F208" s="4" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
+        </is>
+      </c>
+      <c r="G208" s="4" t="inlineStr">
         <is>
           <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
         </is>
       </c>
-      <c r="H208" s="3" t="inlineStr"/>
-      <c r="I208" s="3" t="inlineStr"/>
-      <c r="J208" s="3" t="inlineStr">
-        <is>
-          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.DocNum and part/SPL Master evidence also matches; current export needs reconciliation.</t>
+      <c r="H208" s="4" t="inlineStr"/>
+      <c r="I208" s="4" t="inlineStr"/>
+      <c r="J208" s="4" t="inlineStr">
+        <is>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t>partType</t>
+          <t>addressId</t>
         </is>
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C209" s="4" t="inlineStr">
@@ -31528,7 +31508,7 @@
       </c>
       <c r="F209" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partType?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
         </is>
       </c>
       <c r="G209" s="4" t="inlineStr">
@@ -31547,12 +31527,12 @@
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
         <is>
-          <t>partTypeDescription</t>
+          <t>Bpart</t>
         </is>
       </c>
       <c r="B210" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C210" s="4" t="inlineStr">
@@ -31568,7 +31548,7 @@
       </c>
       <c r="F210" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeDescription?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.Bpart?</t>
         </is>
       </c>
       <c r="G210" s="4" t="inlineStr">
@@ -31587,12 +31567,12 @@
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
         <is>
-          <t>isReworkable</t>
+          <t>quantity</t>
         </is>
       </c>
       <c r="B211" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C211" s="4" t="inlineStr">
@@ -31608,7 +31588,7 @@
       </c>
       <c r="F211" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.isReworkable?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.quantity?</t>
         </is>
       </c>
       <c r="G211" s="4" t="inlineStr">
@@ -31627,12 +31607,12 @@
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
         <is>
-          <t>partNumber</t>
+          <t>shipListCode</t>
         </is>
       </c>
       <c r="B212" s="4" t="inlineStr">
         <is>
-          <t>Yields</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C212" s="4" t="inlineStr">
@@ -31648,7 +31628,7 @@
       </c>
       <c r="F212" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
         </is>
       </c>
       <c r="G212" s="4" t="inlineStr">
@@ -31665,54 +31645,54 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="4" t="inlineStr">
-        <is>
-          <t>unitOfMeasure</t>
-        </is>
-      </c>
-      <c r="B213" s="4" t="inlineStr">
-        <is>
-          <t>Yields</t>
-        </is>
-      </c>
-      <c r="C213" s="4" t="inlineStr">
+      <c r="A213" s="3" t="inlineStr">
+        <is>
+          <t>demandStatus</t>
+        </is>
+      </c>
+      <c r="B213" s="3" t="inlineStr">
+        <is>
+          <t>PurchaseOrders</t>
+        </is>
+      </c>
+      <c r="C213" s="3" t="inlineStr">
         <is>
           <t>Planning V2 template</t>
         </is>
       </c>
-      <c r="D213" s="4" t="inlineStr"/>
-      <c r="E213" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F213" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
-        </is>
-      </c>
-      <c r="G213" s="4" t="inlineStr">
+      <c r="D213" s="3" t="inlineStr"/>
+      <c r="E213" s="3" t="inlineStr">
+        <is>
+          <t>Review required</t>
+        </is>
+      </c>
+      <c r="F213" s="3" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
+        </is>
+      </c>
+      <c r="G213" s="3" t="inlineStr">
         <is>
           <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
         </is>
       </c>
-      <c r="H213" s="4" t="inlineStr"/>
-      <c r="I213" s="4" t="inlineStr"/>
-      <c r="J213" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="H213" s="3" t="inlineStr"/>
+      <c r="I213" s="3" t="inlineStr"/>
+      <c r="J213" s="3" t="inlineStr">
+        <is>
+          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.DocNum and part/SPL Master evidence also matches; current export needs reconciliation.</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
         <is>
-          <t>yield</t>
+          <t>partType</t>
         </is>
       </c>
       <c r="B214" s="4" t="inlineStr">
         <is>
-          <t>Yields</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C214" s="4" t="inlineStr">
@@ -31728,7 +31708,7 @@
       </c>
       <c r="F214" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.partType?</t>
         </is>
       </c>
       <c r="G214" s="4" t="inlineStr">
@@ -31747,12 +31727,12 @@
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
         <is>
-          <t>Secondary TO</t>
+          <t>partTypeDescription</t>
         </is>
       </c>
       <c r="B215" s="4" t="inlineStr">
         <is>
-          <t>WarehouseExclusions</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C215" s="4" t="inlineStr">
@@ -31768,7 +31748,7 @@
       </c>
       <c r="F215" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary TO?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeDescription?</t>
         </is>
       </c>
       <c r="G215" s="4" t="inlineStr">
@@ -31787,12 +31767,12 @@
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
         <is>
-          <t>Secondary FROM</t>
+          <t>isReworkable</t>
         </is>
       </c>
       <c r="B216" s="4" t="inlineStr">
         <is>
-          <t>WarehouseExclusions</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C216" s="4" t="inlineStr">
@@ -31808,7 +31788,7 @@
       </c>
       <c r="F216" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary FROM?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.isReworkable?</t>
         </is>
       </c>
       <c r="G216" s="4" t="inlineStr">
@@ -31827,12 +31807,12 @@
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t>Cross TO</t>
+          <t>partNumber</t>
         </is>
       </c>
       <c r="B217" s="4" t="inlineStr">
         <is>
-          <t>WarehouseExclusions</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C217" s="4" t="inlineStr">
@@ -31848,7 +31828,7 @@
       </c>
       <c r="F217" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross TO?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
         </is>
       </c>
       <c r="G217" s="4" t="inlineStr">
@@ -31867,12 +31847,12 @@
     <row r="218">
       <c r="A218" s="4" t="inlineStr">
         <is>
-          <t>Cross FROM</t>
+          <t>unitOfMeasure</t>
         </is>
       </c>
       <c r="B218" s="4" t="inlineStr">
         <is>
-          <t>WarehouseExclusions</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C218" s="4" t="inlineStr">
@@ -31888,7 +31868,7 @@
       </c>
       <c r="F218" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross FROM?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
         </is>
       </c>
       <c r="G218" s="4" t="inlineStr">
@@ -31907,12 +31887,12 @@
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t>Primary TO</t>
+          <t>yield</t>
         </is>
       </c>
       <c r="B219" s="4" t="inlineStr">
         <is>
-          <t>WarehouseExclusions</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C219" s="4" t="inlineStr">
@@ -31928,7 +31908,7 @@
       </c>
       <c r="F219" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Primary TO?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
         </is>
       </c>
       <c r="G219" s="4" t="inlineStr">
@@ -31944,8 +31924,208 @@
         </is>
       </c>
     </row>
+    <row r="220">
+      <c r="A220" s="4" t="inlineStr">
+        <is>
+          <t>Secondary TO</t>
+        </is>
+      </c>
+      <c r="B220" s="4" t="inlineStr">
+        <is>
+          <t>WarehouseExclusions</t>
+        </is>
+      </c>
+      <c r="C220" s="4" t="inlineStr">
+        <is>
+          <t>Planning V2 template</t>
+        </is>
+      </c>
+      <c r="D220" s="4" t="inlineStr"/>
+      <c r="E220" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F220" s="4" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary TO?</t>
+        </is>
+      </c>
+      <c r="G220" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
+        </is>
+      </c>
+      <c r="H220" s="4" t="inlineStr"/>
+      <c r="I220" s="4" t="inlineStr"/>
+      <c r="J220" s="4" t="inlineStr">
+        <is>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="4" t="inlineStr">
+        <is>
+          <t>Secondary FROM</t>
+        </is>
+      </c>
+      <c r="B221" s="4" t="inlineStr">
+        <is>
+          <t>WarehouseExclusions</t>
+        </is>
+      </c>
+      <c r="C221" s="4" t="inlineStr">
+        <is>
+          <t>Planning V2 template</t>
+        </is>
+      </c>
+      <c r="D221" s="4" t="inlineStr"/>
+      <c r="E221" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F221" s="4" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary FROM?</t>
+        </is>
+      </c>
+      <c r="G221" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
+        </is>
+      </c>
+      <c r="H221" s="4" t="inlineStr"/>
+      <c r="I221" s="4" t="inlineStr"/>
+      <c r="J221" s="4" t="inlineStr">
+        <is>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="4" t="inlineStr">
+        <is>
+          <t>Cross TO</t>
+        </is>
+      </c>
+      <c r="B222" s="4" t="inlineStr">
+        <is>
+          <t>WarehouseExclusions</t>
+        </is>
+      </c>
+      <c r="C222" s="4" t="inlineStr">
+        <is>
+          <t>Planning V2 template</t>
+        </is>
+      </c>
+      <c r="D222" s="4" t="inlineStr"/>
+      <c r="E222" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F222" s="4" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross TO?</t>
+        </is>
+      </c>
+      <c r="G222" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
+        </is>
+      </c>
+      <c r="H222" s="4" t="inlineStr"/>
+      <c r="I222" s="4" t="inlineStr"/>
+      <c r="J222" s="4" t="inlineStr">
+        <is>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="4" t="inlineStr">
+        <is>
+          <t>Cross FROM</t>
+        </is>
+      </c>
+      <c r="B223" s="4" t="inlineStr">
+        <is>
+          <t>WarehouseExclusions</t>
+        </is>
+      </c>
+      <c r="C223" s="4" t="inlineStr">
+        <is>
+          <t>Planning V2 template</t>
+        </is>
+      </c>
+      <c r="D223" s="4" t="inlineStr"/>
+      <c r="E223" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F223" s="4" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross FROM?</t>
+        </is>
+      </c>
+      <c r="G223" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
+        </is>
+      </c>
+      <c r="H223" s="4" t="inlineStr"/>
+      <c r="I223" s="4" t="inlineStr"/>
+      <c r="J223" s="4" t="inlineStr">
+        <is>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="4" t="inlineStr">
+        <is>
+          <t>Primary TO</t>
+        </is>
+      </c>
+      <c r="B224" s="4" t="inlineStr">
+        <is>
+          <t>WarehouseExclusions</t>
+        </is>
+      </c>
+      <c r="C224" s="4" t="inlineStr">
+        <is>
+          <t>Planning V2 template</t>
+        </is>
+      </c>
+      <c r="D224" s="4" t="inlineStr"/>
+      <c r="E224" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F224" s="4" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Primary TO?</t>
+        </is>
+      </c>
+      <c r="G224" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
+        </is>
+      </c>
+      <c r="H224" s="4" t="inlineStr"/>
+      <c r="I224" s="4" t="inlineStr"/>
+      <c r="J224" s="4" t="inlineStr">
+        <is>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J219"/>
+  <autoFilter ref="A1:J224"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -32573,7 +32753,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>OrderType; resolvedDateTime; relCompanyId; assignedPersonCode</t>
+          <t>OrderType; customerCompanyCode; orderStartDatetime; orderStatus; resolvedDateTime; serialNumber; relCompanyId; assignedPersonCode; deviceSerialNumber</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use external SAP PO numbers for purchase orders
</commit_message>
<xml_diff>
--- a/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
+++ b/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
@@ -20552,7 +20552,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>SAP Service Layer SQLQueries:OPOR.DocNum</t>
+          <t>SAP Service Layer SQLQueries:OPOR.NumAtCard, falling back to OPOR.DocNum</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -20810,7 +20810,7 @@
       </c>
       <c r="H155" s="3" t="inlineStr">
         <is>
-          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.DocNum and part/SPL Master evidence also matches; current export needs reconciliation.</t>
+          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.NumAtCard and part/SPL Master evidence also matches.</t>
         </is>
       </c>
     </row>
@@ -31572,7 +31572,7 @@
       <c r="I210" s="3" t="inlineStr"/>
       <c r="J210" s="3" t="inlineStr">
         <is>
-          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.DocNum and part/SPL Master evidence also matches; current export needs reconciliation.</t>
+          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.NumAtCard and part/SPL Master evidence also matches.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Backfill PO costs from historical SPI files
</commit_message>
<xml_diff>
--- a/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
+++ b/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Target Fields'!$A$1:$S$151</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Template Fields'!$A$1:$H$177</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Evidence'!$A$1:$D$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Evidence'!$A$1:$D$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$J$221</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Output Objects'!$A$1:$E$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Missing Important Fields'!$A$1:$E$88</definedName>
@@ -231,8 +231,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceEvidence" displayName="SourceEvidence" ref="A1:D14" headerRowCount="1">
-  <autoFilter ref="A1:D14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceEvidence" displayName="SourceEvidence" ref="A1:D15" headerRowCount="1">
+  <autoFilter ref="A1:D15"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="Path"/>
@@ -20926,7 +20926,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>SPI_DATA.csv:ListPrice multiplied by 0.72 CoCre8 cost factor</t>
+          <t>Current SPI_DATA.csv then Reference/SPI_Historical newest-first:ListPrice multiplied by 0.72 CoCre8 cost factor</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -21629,7 +21629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -21773,12 +21773,12 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>MinStock3 usage</t>
+          <t>Historical SPI prices</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>C:\dev\cc8\MinStock3\enrich_dimensions.py</t>
+          <t>Reference\SPI_Historical</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -21788,63 +21788,63 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Stock audit DN rows aggregate annual usage.</t>
+          <t>Older SPI CSV/XLSX files backfill ListPrice where the current SPI file has deleted parts; current SPI is preferred, then historical files newest-first.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Planning V2 live stock extract</t>
+          <t>MinStock3 usage</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Service Layer SQLQueries on OITW/OITM</t>
+          <t>C:\dev\cc8\MinStock3\enrich_dimensions.py</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Current stock metrics are fetched live from OITW: OnHand, IsCommited, OnOrder, MinStock, MaxStock, AvgPrice.</t>
+          <t>Stock audit DN rows aggregate annual usage.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Manual stock audit report</t>
+          <t>Planning V2 live stock extract</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>C:\dev\cc8\Exco\source_data\Stock Audit Report.txt</t>
+          <t>Service Layer SQLQueries on OITW/OITM</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Allowed manual SAP report source for usage once mapped to the template.</t>
+          <t>Current stock metrics are fetched live from OITW: OnHand, IsCommited, OnOrder, MinStock, MaxStock, AvgPrice.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Reference target fields</t>
+          <t>Manual stock audit report</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Reference\SPL Planning Data Fields edited.xlsx</t>
+          <t>C:\dev\cc8\Exco\source_data\Stock Audit Report.txt</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -21854,19 +21854,19 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Planning V2 target field metadata and CC8 relevance hints.</t>
+          <t>Allowed manual SAP report source for usage once mapped to the template.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Planning V2 sample templates</t>
+          <t>Reference target fields</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Samples\Templates raw.xlsx</t>
+          <t>Reference\SPL Planning Data Fields edited.xlsx</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -21876,19 +21876,19 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Canonical onboarding template fields used for template-shaped CSV outputs.</t>
+          <t>Planning V2 target field metadata and CC8 relevance hints.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>CoCre8 HelpDesk issue tracker</t>
+          <t>Planning V2 sample templates</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>C:\Users\richa\Downloads\CoCre8 Issue Tracker V3.2.csv</t>
+          <t>Samples\Templates raw.xlsx</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -21898,19 +21898,19 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>External SharePoint-list export used only for strict ticket/PO evidence; not committed to git.</t>
+          <t>Canonical onboarding template fields used for template-shaped CSV outputs.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>HelpDesk Power Automate flow</t>
+          <t>CoCre8 HelpDesk issue tracker</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Reference\HelpdeskFlow.txt</t>
+          <t>C:\Users\richa\Downloads\CoCre8 Issue Tracker V3.2.csv</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -21920,34 +21920,56 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Reference flow for ticket lifecycle and improvement recommendations.</t>
+          <t>External SharePoint-list export used only for strict ticket/PO evidence; not committed to git.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
+          <t>HelpDesk Power Automate flow</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Reference\HelpdeskFlow.txt</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Reference flow for ticket lifecycle and improvement recommendations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
           <t>Live SAP item group check</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>MinStock3 SAP Service Layer credentials</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Checked Items and ItemGroups while VPN was connected. ItemGroups are broad customer/manufacturer groups such as FUJITSU, ACER, and CHOICE; sampled item master fields ItemType, ItemClass, and MaterialType are generic SAP classifications.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D14"/>
+  <autoFilter ref="A1:D15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Generate part cost template from SPI history
</commit_message>
<xml_diff>
--- a/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
+++ b/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Target Fields'!$A$1:$S$151</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Template Fields'!$A$1:$H$177</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Evidence'!$A$1:$D$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$J$221</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$J$217</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Output Objects'!$A$1:$E$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Missing Important Fields'!$A$1:$E$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'SAP Investigation Log'!$A$1:$E$10</definedName>
@@ -244,8 +244,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:J221" headerRowCount="1">
-  <autoFilter ref="A1:J221"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:J217" headerRowCount="1">
+  <autoFilter ref="A1:J217"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Field"/>
     <tableColumn id="2" name="Object"/>
@@ -19773,154 +19773,170 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="4" t="inlineStr">
+      <c r="A129" s="2" t="inlineStr">
         <is>
           <t>PartCost</t>
         </is>
       </c>
-      <c r="B129" s="4" t="inlineStr">
+      <c r="B129" s="2" t="inlineStr">
         <is>
           <t>partCode</t>
         </is>
       </c>
-      <c r="C129" s="4" t="inlineStr">
+      <c r="C129" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D129" s="4" t="inlineStr">
+      <c r="D129" s="2" t="inlineStr">
         <is>
           <t>Canonical header from PartCosts.xlsx</t>
         </is>
       </c>
-      <c r="E129" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F129" s="4" t="inlineStr"/>
-      <c r="G129" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H129" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>Actual SAP/Fujitsu part id from live SAP parts and PO lines</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="4" t="inlineStr">
+      <c r="A130" s="2" t="inlineStr">
         <is>
           <t>PartCost</t>
         </is>
       </c>
-      <c r="B130" s="4" t="inlineStr">
+      <c r="B130" s="2" t="inlineStr">
         <is>
           <t>cost</t>
         </is>
       </c>
-      <c r="C130" s="4" t="inlineStr">
+      <c r="C130" s="2" t="inlineStr">
         <is>
           <t>Double</t>
         </is>
       </c>
-      <c r="D130" s="4" t="inlineStr">
+      <c r="D130" s="2" t="inlineStr">
         <is>
           <t>Canonical header from PartCosts.xlsx</t>
         </is>
       </c>
-      <c r="E130" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F130" s="4" t="inlineStr"/>
-      <c r="G130" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H130" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>Current SPI_DATA.csv then Reference/SPI_Historical newest-first:ListPrice multiplied by 0.72, selected as of last PO month where possible</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="4" t="inlineStr">
+      <c r="A131" s="2" t="inlineStr">
         <is>
           <t>PartCost</t>
         </is>
       </c>
-      <c r="B131" s="4" t="inlineStr">
+      <c r="B131" s="2" t="inlineStr">
         <is>
           <t>currencyCode</t>
         </is>
       </c>
-      <c r="C131" s="4" t="inlineStr">
+      <c r="C131" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D131" s="4" t="inlineStr">
+      <c r="D131" s="2" t="inlineStr">
         <is>
           <t>Canonical header from PartCosts.xlsx</t>
         </is>
       </c>
-      <c r="E131" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F131" s="4" t="inlineStr"/>
-      <c r="G131" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H131" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>Business rule: EUR for SPI CoCre8 costs</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="4" t="inlineStr">
+      <c r="A132" s="2" t="inlineStr">
         <is>
           <t>PartCost</t>
         </is>
       </c>
-      <c r="B132" s="4" t="inlineStr">
+      <c r="B132" s="2" t="inlineStr">
         <is>
           <t>averageCost</t>
         </is>
       </c>
-      <c r="C132" s="4" t="inlineStr">
+      <c r="C132" s="2" t="inlineStr">
         <is>
           <t>Double</t>
         </is>
       </c>
-      <c r="D132" s="4" t="inlineStr">
+      <c r="D132" s="2" t="inlineStr">
         <is>
           <t>Canonical header from PartCosts.xlsx</t>
         </is>
       </c>
-      <c r="E132" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F132" s="4" t="inlineStr"/>
-      <c r="G132" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H132" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>PO quantity-weighted average of SPI-derived CoCre8 costs across SAP PO history</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -21983,7 +21999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J221"/>
+  <dimension ref="A1:J217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -30806,7 +30822,7 @@
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr">
@@ -30822,7 +30838,7 @@
       </c>
       <c r="F191" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.partCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
         </is>
       </c>
       <c r="G191" s="4" t="inlineStr">
@@ -30841,12 +30857,12 @@
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>modelCode</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C192" s="4" t="inlineStr">
@@ -30862,7 +30878,7 @@
       </c>
       <c r="F192" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.cost?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
         </is>
       </c>
       <c r="G192" s="4" t="inlineStr">
@@ -30881,12 +30897,12 @@
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>currencyCode</t>
+          <t>modelDescription</t>
         </is>
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C193" s="4" t="inlineStr">
@@ -30902,7 +30918,7 @@
       </c>
       <c r="F193" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.currencyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
         </is>
       </c>
       <c r="G193" s="4" t="inlineStr">
@@ -30921,12 +30937,12 @@
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>averageCost</t>
+          <t>inventoryTransferImoId</t>
         </is>
       </c>
       <c r="B194" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C194" s="4" t="inlineStr">
@@ -30942,7 +30958,7 @@
       </c>
       <c r="F194" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.averageCost?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.inventoryTransferImoId?</t>
         </is>
       </c>
       <c r="G194" s="4" t="inlineStr">
@@ -30961,12 +30977,12 @@
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>partCode</t>
+          <t>createdDateTime</t>
         </is>
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
@@ -30982,7 +30998,7 @@
       </c>
       <c r="F195" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.createdDateTime?</t>
         </is>
       </c>
       <c r="G195" s="4" t="inlineStr">
@@ -31001,12 +31017,12 @@
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>modelCode</t>
+          <t>completedDateTime</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C196" s="4" t="inlineStr">
@@ -31022,7 +31038,7 @@
       </c>
       <c r="F196" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.completedDateTime?</t>
         </is>
       </c>
       <c r="G196" s="4" t="inlineStr">
@@ -31041,12 +31057,12 @@
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>modelDescription</t>
+          <t>fromWarehouseId</t>
         </is>
       </c>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr">
@@ -31062,7 +31078,7 @@
       </c>
       <c r="F197" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.fromWarehouseId?</t>
         </is>
       </c>
       <c r="G197" s="4" t="inlineStr">
@@ -31081,7 +31097,7 @@
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>inventoryTransferImoId</t>
+          <t>toWarehouseId</t>
         </is>
       </c>
       <c r="B198" s="4" t="inlineStr">
@@ -31102,7 +31118,7 @@
       </c>
       <c r="F198" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.inventoryTransferImoId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.toWarehouseId?</t>
         </is>
       </c>
       <c r="G198" s="4" t="inlineStr">
@@ -31121,7 +31137,7 @@
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>createdDateTime</t>
+          <t>demandStatus</t>
         </is>
       </c>
       <c r="B199" s="4" t="inlineStr">
@@ -31142,7 +31158,7 @@
       </c>
       <c r="F199" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.createdDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.demandStatus?</t>
         </is>
       </c>
       <c r="G199" s="4" t="inlineStr">
@@ -31161,7 +31177,7 @@
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>completedDateTime</t>
+          <t>orderStatusIsClosed</t>
         </is>
       </c>
       <c r="B200" s="4" t="inlineStr">
@@ -31182,7 +31198,7 @@
       </c>
       <c r="F200" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.completedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.orderStatusIsClosed?</t>
         </is>
       </c>
       <c r="G200" s="4" t="inlineStr">
@@ -31201,7 +31217,7 @@
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t>fromWarehouseId</t>
+          <t>movementType</t>
         </is>
       </c>
       <c r="B201" s="4" t="inlineStr">
@@ -31222,7 +31238,7 @@
       </c>
       <c r="F201" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.fromWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
         </is>
       </c>
       <c r="G201" s="4" t="inlineStr">
@@ -31241,7 +31257,7 @@
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>toWarehouseId</t>
+          <t>addressId</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
@@ -31262,7 +31278,7 @@
       </c>
       <c r="F202" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.toWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
         </is>
       </c>
       <c r="G202" s="4" t="inlineStr">
@@ -31281,7 +31297,7 @@
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>demandStatus</t>
+          <t>Bpart</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
@@ -31302,7 +31318,7 @@
       </c>
       <c r="F203" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.demandStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.Bpart?</t>
         </is>
       </c>
       <c r="G203" s="4" t="inlineStr">
@@ -31321,7 +31337,7 @@
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>orderStatusIsClosed</t>
+          <t>quantity</t>
         </is>
       </c>
       <c r="B204" s="4" t="inlineStr">
@@ -31342,7 +31358,7 @@
       </c>
       <c r="F204" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.orderStatusIsClosed?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.quantity?</t>
         </is>
       </c>
       <c r="G204" s="4" t="inlineStr">
@@ -31361,7 +31377,7 @@
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>movementType</t>
+          <t>shipListCode</t>
         </is>
       </c>
       <c r="B205" s="4" t="inlineStr">
@@ -31382,7 +31398,7 @@
       </c>
       <c r="F205" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
         </is>
       </c>
       <c r="G205" s="4" t="inlineStr">
@@ -31399,54 +31415,54 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="4" t="inlineStr">
-        <is>
-          <t>addressId</t>
-        </is>
-      </c>
-      <c r="B206" s="4" t="inlineStr">
-        <is>
-          <t>InventoryTransfers</t>
-        </is>
-      </c>
-      <c r="C206" s="4" t="inlineStr">
+      <c r="A206" s="3" t="inlineStr">
+        <is>
+          <t>demandStatus</t>
+        </is>
+      </c>
+      <c r="B206" s="3" t="inlineStr">
+        <is>
+          <t>PurchaseOrders</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
         <is>
           <t>Planning V2 template</t>
         </is>
       </c>
-      <c r="D206" s="4" t="inlineStr"/>
-      <c r="E206" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F206" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
-        </is>
-      </c>
-      <c r="G206" s="4" t="inlineStr">
+      <c r="D206" s="3" t="inlineStr"/>
+      <c r="E206" s="3" t="inlineStr">
+        <is>
+          <t>Review required</t>
+        </is>
+      </c>
+      <c r="F206" s="3" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
+        </is>
+      </c>
+      <c r="G206" s="3" t="inlineStr">
         <is>
           <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
         </is>
       </c>
-      <c r="H206" s="4" t="inlineStr"/>
-      <c r="I206" s="4" t="inlineStr"/>
-      <c r="J206" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="H206" s="3" t="inlineStr"/>
+      <c r="I206" s="3" t="inlineStr"/>
+      <c r="J206" s="3" t="inlineStr">
+        <is>
+          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.NumAtCard and part/SPL Master evidence also matches.</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>Bpart</t>
+          <t>partType</t>
         </is>
       </c>
       <c r="B207" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C207" s="4" t="inlineStr">
@@ -31462,7 +31478,7 @@
       </c>
       <c r="F207" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.Bpart?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.partType?</t>
         </is>
       </c>
       <c r="G207" s="4" t="inlineStr">
@@ -31481,12 +31497,12 @@
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>partTypeDescription</t>
         </is>
       </c>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C208" s="4" t="inlineStr">
@@ -31502,7 +31518,7 @@
       </c>
       <c r="F208" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.quantity?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeDescription?</t>
         </is>
       </c>
       <c r="G208" s="4" t="inlineStr">
@@ -31521,12 +31537,12 @@
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t>shipListCode</t>
+          <t>isReworkable</t>
         </is>
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C209" s="4" t="inlineStr">
@@ -31542,7 +31558,7 @@
       </c>
       <c r="F209" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.isReworkable?</t>
         </is>
       </c>
       <c r="G209" s="4" t="inlineStr">
@@ -31559,54 +31575,54 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="3" t="inlineStr">
-        <is>
-          <t>demandStatus</t>
-        </is>
-      </c>
-      <c r="B210" s="3" t="inlineStr">
-        <is>
-          <t>PurchaseOrders</t>
-        </is>
-      </c>
-      <c r="C210" s="3" t="inlineStr">
+      <c r="A210" s="4" t="inlineStr">
+        <is>
+          <t>partNumber</t>
+        </is>
+      </c>
+      <c r="B210" s="4" t="inlineStr">
+        <is>
+          <t>Yields</t>
+        </is>
+      </c>
+      <c r="C210" s="4" t="inlineStr">
         <is>
           <t>Planning V2 template</t>
         </is>
       </c>
-      <c r="D210" s="3" t="inlineStr"/>
-      <c r="E210" s="3" t="inlineStr">
-        <is>
-          <t>Review required</t>
-        </is>
-      </c>
-      <c r="F210" s="3" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
-        </is>
-      </c>
-      <c r="G210" s="3" t="inlineStr">
+      <c r="D210" s="4" t="inlineStr"/>
+      <c r="E210" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F210" s="4" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
+        </is>
+      </c>
+      <c r="G210" s="4" t="inlineStr">
         <is>
           <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
         </is>
       </c>
-      <c r="H210" s="3" t="inlineStr"/>
-      <c r="I210" s="3" t="inlineStr"/>
-      <c r="J210" s="3" t="inlineStr">
-        <is>
-          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.NumAtCard and part/SPL Master evidence also matches.</t>
+      <c r="H210" s="4" t="inlineStr"/>
+      <c r="I210" s="4" t="inlineStr"/>
+      <c r="J210" s="4" t="inlineStr">
+        <is>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
         <is>
-          <t>partType</t>
+          <t>unitOfMeasure</t>
         </is>
       </c>
       <c r="B211" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C211" s="4" t="inlineStr">
@@ -31622,7 +31638,7 @@
       </c>
       <c r="F211" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partType?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
         </is>
       </c>
       <c r="G211" s="4" t="inlineStr">
@@ -31641,12 +31657,12 @@
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
         <is>
-          <t>partTypeDescription</t>
+          <t>yield</t>
         </is>
       </c>
       <c r="B212" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C212" s="4" t="inlineStr">
@@ -31662,7 +31678,7 @@
       </c>
       <c r="F212" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeDescription?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
         </is>
       </c>
       <c r="G212" s="4" t="inlineStr">
@@ -31681,12 +31697,12 @@
     <row r="213">
       <c r="A213" s="4" t="inlineStr">
         <is>
-          <t>isReworkable</t>
+          <t>Secondary TO</t>
         </is>
       </c>
       <c r="B213" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C213" s="4" t="inlineStr">
@@ -31702,7 +31718,7 @@
       </c>
       <c r="F213" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.isReworkable?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary TO?</t>
         </is>
       </c>
       <c r="G213" s="4" t="inlineStr">
@@ -31721,12 +31737,12 @@
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
         <is>
-          <t>partNumber</t>
+          <t>Secondary FROM</t>
         </is>
       </c>
       <c r="B214" s="4" t="inlineStr">
         <is>
-          <t>Yields</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C214" s="4" t="inlineStr">
@@ -31742,7 +31758,7 @@
       </c>
       <c r="F214" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary FROM?</t>
         </is>
       </c>
       <c r="G214" s="4" t="inlineStr">
@@ -31761,12 +31777,12 @@
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
         <is>
-          <t>unitOfMeasure</t>
+          <t>Cross TO</t>
         </is>
       </c>
       <c r="B215" s="4" t="inlineStr">
         <is>
-          <t>Yields</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C215" s="4" t="inlineStr">
@@ -31782,7 +31798,7 @@
       </c>
       <c r="F215" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross TO?</t>
         </is>
       </c>
       <c r="G215" s="4" t="inlineStr">
@@ -31801,12 +31817,12 @@
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
         <is>
-          <t>yield</t>
+          <t>Cross FROM</t>
         </is>
       </c>
       <c r="B216" s="4" t="inlineStr">
         <is>
-          <t>Yields</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C216" s="4" t="inlineStr">
@@ -31822,7 +31838,7 @@
       </c>
       <c r="F216" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross FROM?</t>
         </is>
       </c>
       <c r="G216" s="4" t="inlineStr">
@@ -31841,7 +31857,7 @@
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t>Secondary TO</t>
+          <t>Primary TO</t>
         </is>
       </c>
       <c r="B217" s="4" t="inlineStr">
@@ -31862,7 +31878,7 @@
       </c>
       <c r="F217" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary TO?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Primary TO?</t>
         </is>
       </c>
       <c r="G217" s="4" t="inlineStr">
@@ -31878,168 +31894,8 @@
         </is>
       </c>
     </row>
-    <row r="218">
-      <c r="A218" s="4" t="inlineStr">
-        <is>
-          <t>Secondary FROM</t>
-        </is>
-      </c>
-      <c r="B218" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C218" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D218" s="4" t="inlineStr"/>
-      <c r="E218" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F218" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary FROM?</t>
-        </is>
-      </c>
-      <c r="G218" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H218" s="4" t="inlineStr"/>
-      <c r="I218" s="4" t="inlineStr"/>
-      <c r="J218" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" s="4" t="inlineStr">
-        <is>
-          <t>Cross TO</t>
-        </is>
-      </c>
-      <c r="B219" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C219" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D219" s="4" t="inlineStr"/>
-      <c r="E219" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F219" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross TO?</t>
-        </is>
-      </c>
-      <c r="G219" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H219" s="4" t="inlineStr"/>
-      <c r="I219" s="4" t="inlineStr"/>
-      <c r="J219" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" s="4" t="inlineStr">
-        <is>
-          <t>Cross FROM</t>
-        </is>
-      </c>
-      <c r="B220" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C220" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D220" s="4" t="inlineStr"/>
-      <c r="E220" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F220" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross FROM?</t>
-        </is>
-      </c>
-      <c r="G220" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H220" s="4" t="inlineStr"/>
-      <c r="I220" s="4" t="inlineStr"/>
-      <c r="J220" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" s="4" t="inlineStr">
-        <is>
-          <t>Primary TO</t>
-        </is>
-      </c>
-      <c r="B221" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C221" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D221" s="4" t="inlineStr"/>
-      <c r="E221" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F221" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Primary TO?</t>
-        </is>
-      </c>
-      <c r="G221" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H221" s="4" t="inlineStr"/>
-      <c r="I221" s="4" t="inlineStr"/>
-      <c r="J221" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J221"/>
+  <autoFilter ref="A1:J217"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -32726,31 +32582,27 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>PartCost</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>PartCost.csv</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>Pending/header only</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>partCode, cost, currencyCode, averageCost</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>partCode; cost; currencyCode; averageCost</t>
-        </is>
-      </c>
+      <c r="E27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Apply confirmed CoCre8 part defaults
</commit_message>
<xml_diff>
--- a/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
+++ b/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Target Fields'!$A$1:$S$151</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Template Fields'!$A$1:$H$177</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Evidence'!$A$1:$D$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$J$217</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$J$212</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Output Objects'!$A$1:$E$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Missing Important Fields'!$A$1:$E$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'SAP Investigation Log'!$A$1:$E$10</definedName>
@@ -244,8 +244,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:J217" headerRowCount="1">
-  <autoFilter ref="A1:J217"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:J212" headerRowCount="1">
+  <autoFilter ref="A1:J212"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Field"/>
     <tableColumn id="2" name="Object"/>
@@ -15576,7 +15576,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>SPI_DATA.csv:Main alternative par equals material/part number</t>
+          <t>SPI_DATA.csv:Main alternative par equals material/part number; defaults true when no main alternative is listed</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -15618,7 +15618,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>SPI_DATA.csv:Main alternative par</t>
+          <t>SPI_DATA.csv:Main alternative par; defaults to own part number when no main alternative is listed</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -15675,78 +15675,86 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Parts</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>isBootStockable</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Boolean</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Canonical header from Parts.xlsx</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr"/>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Business rule: N for all CoCre8 stock</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Parts</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>isBranchStockable</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Boolean</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Canonical header from Parts.xlsx</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr"/>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Business rule: Y for all CoCre8 stock</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -15941,40 +15949,44 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Parts</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>isObsolete</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Boolean</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Canonical header from Parts.xlsx</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr"/>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Business rule: N for all CoCre8 stock for now</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -16047,40 +16059,44 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Parts</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>isExcludeFromReplenishment</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Boolean</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Canonical header from Parts.xlsx</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr"/>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Business rule: N for all CoCre8 stock for now</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -16119,40 +16135,44 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Parts</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>purchaseLeadTimeDays</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Number</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Canonical header from Parts.xlsx</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr"/>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Business rule: default 3 days; 180 days when description contains BBU</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -21999,7 +22019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J217"/>
+  <dimension ref="A1:J212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -27937,7 +27957,7 @@
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>isBootStockable</t>
+          <t>productClass</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
@@ -27953,12 +27973,12 @@
       <c r="D119" s="4" t="inlineStr"/>
       <c r="E119" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Not available in checked source</t>
         </is>
       </c>
       <c r="F119" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isBootStockable?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.productClass?</t>
         </is>
       </c>
       <c r="G119" s="4" t="inlineStr">
@@ -27970,14 +27990,14 @@
       <c r="I119" s="4" t="inlineStr"/>
       <c r="J119" s="4" t="inlineStr">
         <is>
-          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
+          <t>Left blank. Live SAP item master check found broad ItemGroups such as FUJITSU/ACER/CHOICE and generic ItemType/ItemClass/MaterialType values, not Planning V2 class/type semantics.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>isBranchStockable</t>
+          <t>productType</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
@@ -27993,12 +28013,12 @@
       <c r="D120" s="4" t="inlineStr"/>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Not available in checked source</t>
         </is>
       </c>
       <c r="F120" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isBranchStockable?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.productType?</t>
         </is>
       </c>
       <c r="G120" s="4" t="inlineStr">
@@ -28010,14 +28030,14 @@
       <c r="I120" s="4" t="inlineStr"/>
       <c r="J120" s="4" t="inlineStr">
         <is>
-          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
+          <t>Left blank. Live SAP item master check found broad ItemGroups such as FUJITSU/ACER/CHOICE and generic ItemType/ItemClass/MaterialType values, not Planning V2 class/type semantics.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>productClass</t>
+          <t>costCategory</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
@@ -28033,12 +28053,12 @@
       <c r="D121" s="4" t="inlineStr"/>
       <c r="E121" s="4" t="inlineStr">
         <is>
-          <t>Not available in checked source</t>
+          <t>Investigate SAP first</t>
         </is>
       </c>
       <c r="F121" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.productClass?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.costCategory?</t>
         </is>
       </c>
       <c r="G121" s="4" t="inlineStr">
@@ -28050,14 +28070,14 @@
       <c r="I121" s="4" t="inlineStr"/>
       <c r="J121" s="4" t="inlineStr">
         <is>
-          <t>Left blank. Live SAP item master check found broad ItemGroups such as FUJITSU/ACER/CHOICE and generic ItemType/ItemClass/MaterialType values, not Planning V2 class/type semantics.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>productType</t>
+          <t>partType</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
@@ -28078,7 +28098,7 @@
       </c>
       <c r="F122" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.productType?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.partType?</t>
         </is>
       </c>
       <c r="G122" s="4" t="inlineStr">
@@ -28097,7 +28117,7 @@
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>costCategory</t>
+          <t>isKit</t>
         </is>
       </c>
       <c r="B123" s="4" t="inlineStr">
@@ -28118,7 +28138,7 @@
       </c>
       <c r="F123" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.costCategory?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.isKit?</t>
         </is>
       </c>
       <c r="G123" s="4" t="inlineStr">
@@ -28137,7 +28157,7 @@
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t>partType</t>
+          <t>isCritical</t>
         </is>
       </c>
       <c r="B124" s="4" t="inlineStr">
@@ -28153,12 +28173,12 @@
       <c r="D124" s="4" t="inlineStr"/>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>Not available in checked source</t>
+          <t>Investigate SAP first</t>
         </is>
       </c>
       <c r="F124" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.partType?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.isCritical?</t>
         </is>
       </c>
       <c r="G124" s="4" t="inlineStr">
@@ -28170,19 +28190,19 @@
       <c r="I124" s="4" t="inlineStr"/>
       <c r="J124" s="4" t="inlineStr">
         <is>
-          <t>Left blank. Live SAP item master check found broad ItemGroups such as FUJITSU/ACER/CHOICE and generic ItemType/ItemClass/MaterialType values, not Planning V2 class/type semantics.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
         <is>
-          <t>isKit</t>
+          <t>externalAddressId</t>
         </is>
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
-          <t>Parts</t>
+          <t>Addresses</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
@@ -28198,7 +28218,7 @@
       </c>
       <c r="F125" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isKit?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.externalAddressId?</t>
         </is>
       </c>
       <c r="G125" s="4" t="inlineStr">
@@ -28210,19 +28230,19 @@
       <c r="I125" s="4" t="inlineStr"/>
       <c r="J125" s="4" t="inlineStr">
         <is>
-          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
         <is>
-          <t>isObsolete</t>
+          <t>customerExternalId</t>
         </is>
       </c>
       <c r="B126" s="4" t="inlineStr">
         <is>
-          <t>Parts</t>
+          <t>Addresses</t>
         </is>
       </c>
       <c r="C126" s="4" t="inlineStr">
@@ -28238,7 +28258,7 @@
       </c>
       <c r="F126" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isObsolete?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.customerExternalId?</t>
         </is>
       </c>
       <c r="G126" s="4" t="inlineStr">
@@ -28250,19 +28270,19 @@
       <c r="I126" s="4" t="inlineStr"/>
       <c r="J126" s="4" t="inlineStr">
         <is>
-          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
         <is>
-          <t>isExcludeFromReplenishment</t>
+          <t>6,0</t>
         </is>
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
-          <t>Parts</t>
+          <t>Addresses</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
@@ -28278,7 +28298,7 @@
       </c>
       <c r="F127" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isExcludeFromReplenishment?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.6,0?</t>
         </is>
       </c>
       <c r="G127" s="4" t="inlineStr">
@@ -28290,19 +28310,19 @@
       <c r="I127" s="4" t="inlineStr"/>
       <c r="J127" s="4" t="inlineStr">
         <is>
-          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
         <is>
-          <t>purchaseLeadTimeDays</t>
+          <t>addressLine2</t>
         </is>
       </c>
       <c r="B128" s="4" t="inlineStr">
         <is>
-          <t>Parts</t>
+          <t>Addresses</t>
         </is>
       </c>
       <c r="C128" s="4" t="inlineStr">
@@ -28318,7 +28338,7 @@
       </c>
       <c r="F128" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.purchaseLeadTimeDays?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.addressLine2?</t>
         </is>
       </c>
       <c r="G128" s="4" t="inlineStr">
@@ -28330,19 +28350,19 @@
       <c r="I128" s="4" t="inlineStr"/>
       <c r="J128" s="4" t="inlineStr">
         <is>
-          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t>isCritical</t>
+          <t>addressLine3</t>
         </is>
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t>Parts</t>
+          <t>Addresses</t>
         </is>
       </c>
       <c r="C129" s="4" t="inlineStr">
@@ -28358,7 +28378,7 @@
       </c>
       <c r="F129" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isCritical?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.addressLine3?</t>
         </is>
       </c>
       <c r="G129" s="4" t="inlineStr">
@@ -28370,14 +28390,14 @@
       <c r="I129" s="4" t="inlineStr"/>
       <c r="J129" s="4" t="inlineStr">
         <is>
-          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>externalAddressId</t>
+          <t>city</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
@@ -28398,7 +28418,7 @@
       </c>
       <c r="F130" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.externalAddressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.city?</t>
         </is>
       </c>
       <c r="G130" s="4" t="inlineStr">
@@ -28417,7 +28437,7 @@
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>customerExternalId</t>
+          <t>stateProvince</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
@@ -28438,7 +28458,7 @@
       </c>
       <c r="F131" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.customerExternalId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.stateProvince?</t>
         </is>
       </c>
       <c r="G131" s="4" t="inlineStr">
@@ -28457,7 +28477,7 @@
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>6,0</t>
+          <t>countryCode</t>
         </is>
       </c>
       <c r="B132" s="4" t="inlineStr">
@@ -28478,7 +28498,7 @@
       </c>
       <c r="F132" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.6,0?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.countryCode?</t>
         </is>
       </c>
       <c r="G132" s="4" t="inlineStr">
@@ -28497,7 +28517,7 @@
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
         <is>
-          <t>addressLine2</t>
+          <t>latitude</t>
         </is>
       </c>
       <c r="B133" s="4" t="inlineStr">
@@ -28518,7 +28538,7 @@
       </c>
       <c r="F133" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.addressLine2?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.latitude?</t>
         </is>
       </c>
       <c r="G133" s="4" t="inlineStr">
@@ -28537,7 +28557,7 @@
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
         <is>
-          <t>addressLine3</t>
+          <t>longitude</t>
         </is>
       </c>
       <c r="B134" s="4" t="inlineStr">
@@ -28558,7 +28578,7 @@
       </c>
       <c r="F134" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.addressLine3?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.longitude?</t>
         </is>
       </c>
       <c r="G134" s="4" t="inlineStr">
@@ -28577,7 +28597,7 @@
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>timeZone</t>
         </is>
       </c>
       <c r="B135" s="4" t="inlineStr">
@@ -28598,7 +28618,7 @@
       </c>
       <c r="F135" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.city?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.timeZone?</t>
         </is>
       </c>
       <c r="G135" s="4" t="inlineStr">
@@ -28617,7 +28637,7 @@
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>stateProvince</t>
+          <t>nodeId</t>
         </is>
       </c>
       <c r="B136" s="4" t="inlineStr">
@@ -28638,7 +28658,7 @@
       </c>
       <c r="F136" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.stateProvince?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.nodeId?</t>
         </is>
       </c>
       <c r="G136" s="4" t="inlineStr">
@@ -28657,12 +28677,12 @@
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
         <is>
-          <t>countryCode</t>
+          <t>personId</t>
         </is>
       </c>
       <c r="B137" s="4" t="inlineStr">
         <is>
-          <t>Addresses</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C137" s="4" t="inlineStr">
@@ -28678,7 +28698,7 @@
       </c>
       <c r="F137" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.countryCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.personId?</t>
         </is>
       </c>
       <c r="G137" s="4" t="inlineStr">
@@ -28697,12 +28717,12 @@
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
         <is>
-          <t>latitude</t>
+          <t>role</t>
         </is>
       </c>
       <c r="B138" s="4" t="inlineStr">
         <is>
-          <t>Addresses</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C138" s="4" t="inlineStr">
@@ -28718,7 +28738,7 @@
       </c>
       <c r="F138" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.latitude?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.role?</t>
         </is>
       </c>
       <c r="G138" s="4" t="inlineStr">
@@ -28737,12 +28757,12 @@
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>longitude</t>
+          <t>addressId</t>
         </is>
       </c>
       <c r="B139" s="4" t="inlineStr">
         <is>
-          <t>Addresses</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C139" s="4" t="inlineStr">
@@ -28758,7 +28778,7 @@
       </c>
       <c r="F139" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.longitude?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.addressId?</t>
         </is>
       </c>
       <c r="G139" s="4" t="inlineStr">
@@ -28777,12 +28797,12 @@
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>timeZone</t>
+          <t>nodeId</t>
         </is>
       </c>
       <c r="B140" s="4" t="inlineStr">
         <is>
-          <t>Addresses</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C140" s="4" t="inlineStr">
@@ -28798,7 +28818,7 @@
       </c>
       <c r="F140" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.timeZone?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.nodeId?</t>
         </is>
       </c>
       <c r="G140" s="4" t="inlineStr">
@@ -28817,12 +28837,12 @@
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
         <is>
-          <t>nodeId</t>
+          <t>firstName</t>
         </is>
       </c>
       <c r="B141" s="4" t="inlineStr">
         <is>
-          <t>Addresses</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C141" s="4" t="inlineStr">
@@ -28838,7 +28858,7 @@
       </c>
       <c r="F141" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.nodeId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.firstName?</t>
         </is>
       </c>
       <c r="G141" s="4" t="inlineStr">
@@ -28857,7 +28877,7 @@
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>personId</t>
+          <t>middleName</t>
         </is>
       </c>
       <c r="B142" s="4" t="inlineStr">
@@ -28878,7 +28898,7 @@
       </c>
       <c r="F142" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.personId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.middleName?</t>
         </is>
       </c>
       <c r="G142" s="4" t="inlineStr">
@@ -28897,7 +28917,7 @@
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>surname</t>
         </is>
       </c>
       <c r="B143" s="4" t="inlineStr">
@@ -28918,7 +28938,7 @@
       </c>
       <c r="F143" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.role?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.surname?</t>
         </is>
       </c>
       <c r="G143" s="4" t="inlineStr">
@@ -28937,7 +28957,7 @@
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>addressId</t>
+          <t>isActive</t>
         </is>
       </c>
       <c r="B144" s="4" t="inlineStr">
@@ -28958,7 +28978,7 @@
       </c>
       <c r="F144" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.addressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.isActive?</t>
         </is>
       </c>
       <c r="G144" s="4" t="inlineStr">
@@ -28977,7 +28997,7 @@
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>nodeId</t>
+          <t>telephoneNumber</t>
         </is>
       </c>
       <c r="B145" s="4" t="inlineStr">
@@ -28998,7 +29018,7 @@
       </c>
       <c r="F145" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.nodeId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.telephoneNumber?</t>
         </is>
       </c>
       <c r="G145" s="4" t="inlineStr">
@@ -29017,7 +29037,7 @@
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>firstName</t>
+          <t>whs id</t>
         </is>
       </c>
       <c r="B146" s="4" t="inlineStr">
@@ -29038,7 +29058,7 @@
       </c>
       <c r="F146" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.firstName?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.whs id?</t>
         </is>
       </c>
       <c r="G146" s="4" t="inlineStr">
@@ -29057,12 +29077,12 @@
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>middleName</t>
+          <t>OrderType</t>
         </is>
       </c>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C147" s="4" t="inlineStr">
@@ -29078,7 +29098,7 @@
       </c>
       <c r="F147" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.middleName?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.OrderType?</t>
         </is>
       </c>
       <c r="G147" s="4" t="inlineStr">
@@ -29097,12 +29117,12 @@
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>surname</t>
+          <t>orderStartDatetime</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C148" s="4" t="inlineStr">
@@ -29118,7 +29138,7 @@
       </c>
       <c r="F148" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.surname?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStartDatetime?</t>
         </is>
       </c>
       <c r="G148" s="4" t="inlineStr">
@@ -29137,12 +29157,12 @@
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>isActive</t>
+          <t>orderStatus</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">
@@ -29158,7 +29178,7 @@
       </c>
       <c r="F149" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.isActive?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStatus?</t>
         </is>
       </c>
       <c r="G149" s="4" t="inlineStr">
@@ -29177,12 +29197,12 @@
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>telephoneNumber</t>
+          <t>resolvedDateTime</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C150" s="4" t="inlineStr">
@@ -29198,7 +29218,7 @@
       </c>
       <c r="F150" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.telephoneNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.resolvedDateTime?</t>
         </is>
       </c>
       <c r="G150" s="4" t="inlineStr">
@@ -29217,12 +29237,12 @@
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>whs id</t>
+          <t>relCompanyId</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
@@ -29238,7 +29258,7 @@
       </c>
       <c r="F151" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.whs id?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.relCompanyId?</t>
         </is>
       </c>
       <c r="G151" s="4" t="inlineStr">
@@ -29257,7 +29277,7 @@
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>OrderType</t>
+          <t>assignedPersonCode</t>
         </is>
       </c>
       <c r="B152" s="4" t="inlineStr">
@@ -29278,7 +29298,7 @@
       </c>
       <c r="F152" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.OrderType?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.assignedPersonCode?</t>
         </is>
       </c>
       <c r="G152" s="4" t="inlineStr">
@@ -29297,12 +29317,12 @@
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>orderStartDatetime</t>
+          <t>orderNumber</t>
         </is>
       </c>
       <c r="B153" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C153" s="4" t="inlineStr">
@@ -29318,7 +29338,7 @@
       </c>
       <c r="F153" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStartDatetime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.orderNumber?</t>
         </is>
       </c>
       <c r="G153" s="4" t="inlineStr">
@@ -29337,12 +29357,12 @@
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>orderStatus</t>
+          <t>RequestID</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C154" s="4" t="inlineStr">
@@ -29358,7 +29378,7 @@
       </c>
       <c r="F154" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.RequestID?</t>
         </is>
       </c>
       <c r="G154" s="4" t="inlineStr">
@@ -29377,12 +29397,12 @@
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>resolvedDateTime</t>
+          <t>location</t>
         </is>
       </c>
       <c r="B155" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C155" s="4" t="inlineStr">
@@ -29398,7 +29418,7 @@
       </c>
       <c r="F155" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.resolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.location?</t>
         </is>
       </c>
       <c r="G155" s="4" t="inlineStr">
@@ -29417,12 +29437,12 @@
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>relCompanyId</t>
+          <t>eta</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C156" s="4" t="inlineStr">
@@ -29438,7 +29458,7 @@
       </c>
       <c r="F156" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.relCompanyId?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.eta?</t>
         </is>
       </c>
       <c r="G156" s="4" t="inlineStr">
@@ -29457,12 +29477,12 @@
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>assignedPersonCode</t>
+          <t>actualEta</t>
         </is>
       </c>
       <c r="B157" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C157" s="4" t="inlineStr">
@@ -29478,7 +29498,7 @@
       </c>
       <c r="F157" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.assignedPersonCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualEta?</t>
         </is>
       </c>
       <c r="G157" s="4" t="inlineStr">
@@ -29497,7 +29517,7 @@
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>orderNumber</t>
+          <t>actualResolveDateTime</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
@@ -29518,7 +29538,7 @@
       </c>
       <c r="F158" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.orderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualResolveDateTime?</t>
         </is>
       </c>
       <c r="G158" s="4" t="inlineStr">
@@ -29537,7 +29557,7 @@
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>RequestID</t>
+          <t>recallDateTime</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
@@ -29558,7 +29578,7 @@
       </c>
       <c r="F159" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.RequestID?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.recallDateTime?</t>
         </is>
       </c>
       <c r="G159" s="4" t="inlineStr">
@@ -29577,7 +29597,7 @@
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>actualRecallDateTime</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
@@ -29598,7 +29618,7 @@
       </c>
       <c r="F160" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.location?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualRecallDateTime?</t>
         </is>
       </c>
       <c r="G160" s="4" t="inlineStr">
@@ -29617,7 +29637,7 @@
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>eta</t>
+          <t>slaEtaClock</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
@@ -29638,7 +29658,7 @@
       </c>
       <c r="F161" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.eta?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaClock?</t>
         </is>
       </c>
       <c r="G161" s="4" t="inlineStr">
@@ -29657,7 +29677,7 @@
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>actualEta</t>
+          <t>slaResolveClock</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
@@ -29678,7 +29698,7 @@
       </c>
       <c r="F162" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualEta?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveClock?</t>
         </is>
       </c>
       <c r="G162" s="4" t="inlineStr">
@@ -29697,7 +29717,7 @@
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>actualResolveDateTime</t>
+          <t>slaFailureCode</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
@@ -29718,7 +29738,7 @@
       </c>
       <c r="F163" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualResolveDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaFailureCode?</t>
         </is>
       </c>
       <c r="G163" s="4" t="inlineStr">
@@ -29737,7 +29757,7 @@
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>recallDateTime</t>
+          <t>slaEtaHit</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
@@ -29758,7 +29778,7 @@
       </c>
       <c r="F164" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.recallDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaHit?</t>
         </is>
       </c>
       <c r="G164" s="4" t="inlineStr">
@@ -29777,7 +29797,7 @@
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t>actualRecallDateTime</t>
+          <t>slaResolveDateTime</t>
         </is>
       </c>
       <c r="B165" s="4" t="inlineStr">
@@ -29798,7 +29818,7 @@
       </c>
       <c r="F165" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualRecallDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveDateTime?</t>
         </is>
       </c>
       <c r="G165" s="4" t="inlineStr">
@@ -29817,12 +29837,12 @@
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>slaEtaClock</t>
+          <t>orderNumber</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C166" s="4" t="inlineStr">
@@ -29838,7 +29858,7 @@
       </c>
       <c r="F166" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaClock?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderNumber?</t>
         </is>
       </c>
       <c r="G166" s="4" t="inlineStr">
@@ -29857,12 +29877,12 @@
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>slaResolveClock</t>
+          <t>requestId</t>
         </is>
       </c>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C167" s="4" t="inlineStr">
@@ -29878,7 +29898,7 @@
       </c>
       <c r="F167" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveClock?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.requestId?</t>
         </is>
       </c>
       <c r="G167" s="4" t="inlineStr">
@@ -29897,12 +29917,12 @@
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>slaFailureCode</t>
+          <t>customerCompanyCode</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C168" s="4" t="inlineStr">
@@ -29918,7 +29938,7 @@
       </c>
       <c r="F168" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaFailureCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.customerCompanyCode?</t>
         </is>
       </c>
       <c r="G168" s="4" t="inlineStr">
@@ -29937,12 +29957,12 @@
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>slaEtaHit</t>
+          <t>orderStatus</t>
         </is>
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
@@ -29958,7 +29978,7 @@
       </c>
       <c r="F169" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaHit?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStatus?</t>
         </is>
       </c>
       <c r="G169" s="4" t="inlineStr">
@@ -29977,12 +29997,12 @@
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>slaResolveDateTime</t>
+          <t>orderStartDatetime</t>
         </is>
       </c>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C170" s="4" t="inlineStr">
@@ -29998,7 +30018,7 @@
       </c>
       <c r="F170" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStartDatetime?</t>
         </is>
       </c>
       <c r="G170" s="4" t="inlineStr">
@@ -30017,7 +30037,7 @@
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>orderNumber</t>
+          <t>siteCompanyCode</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
@@ -30038,7 +30058,7 @@
       </c>
       <c r="F171" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.siteCompanyCode?</t>
         </is>
       </c>
       <c r="G171" s="4" t="inlineStr">
@@ -30057,7 +30077,7 @@
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>requestId</t>
+          <t>repairType</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
@@ -30078,7 +30098,7 @@
       </c>
       <c r="F172" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.requestId?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairType?</t>
         </is>
       </c>
       <c r="G172" s="4" t="inlineStr">
@@ -30097,7 +30117,7 @@
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>customerCompanyCode</t>
+          <t>partsOrderDateTime</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
@@ -30118,7 +30138,7 @@
       </c>
       <c r="F173" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.customerCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsOrderDateTime?</t>
         </is>
       </c>
       <c r="G173" s="4" t="inlineStr">
@@ -30137,7 +30157,7 @@
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>orderStatus</t>
+          <t>partsReceivedDateTime</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
@@ -30158,7 +30178,7 @@
       </c>
       <c r="F174" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsReceivedDateTime?</t>
         </is>
       </c>
       <c r="G174" s="4" t="inlineStr">
@@ -30177,7 +30197,7 @@
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>orderStartDatetime</t>
+          <t>repairCode</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
@@ -30198,7 +30218,7 @@
       </c>
       <c r="F175" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStartDatetime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCode?</t>
         </is>
       </c>
       <c r="G175" s="4" t="inlineStr">
@@ -30217,7 +30237,7 @@
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>siteCompanyCode</t>
+          <t>repairCompany</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
@@ -30238,7 +30258,7 @@
       </c>
       <c r="F176" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.siteCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCompany?</t>
         </is>
       </c>
       <c r="G176" s="4" t="inlineStr">
@@ -30257,7 +30277,7 @@
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>repairType</t>
+          <t>raStatus</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
@@ -30278,7 +30298,7 @@
       </c>
       <c r="F177" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairType?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.raStatus?</t>
         </is>
       </c>
       <c r="G177" s="4" t="inlineStr">
@@ -30297,7 +30317,7 @@
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>partsOrderDateTime</t>
+          <t>Warehouse</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
@@ -30318,7 +30338,7 @@
       </c>
       <c r="F178" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsOrderDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.Warehouse?</t>
         </is>
       </c>
       <c r="G178" s="4" t="inlineStr">
@@ -30337,7 +30357,7 @@
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>partsReceivedDateTime</t>
+          <t>assignedPerson</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
@@ -30358,7 +30378,7 @@
       </c>
       <c r="F179" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsReceivedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.assignedPerson?</t>
         </is>
       </c>
       <c r="G179" s="4" t="inlineStr">
@@ -30377,7 +30397,7 @@
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>repairCode</t>
+          <t>resolvedDateTime</t>
         </is>
       </c>
       <c r="B180" s="4" t="inlineStr">
@@ -30398,7 +30418,7 @@
       </c>
       <c r="F180" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.resolvedDateTime?</t>
         </is>
       </c>
       <c r="G180" s="4" t="inlineStr">
@@ -30417,7 +30437,7 @@
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>repairCompany</t>
+          <t>serialNumber</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
@@ -30438,7 +30458,7 @@
       </c>
       <c r="F181" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCompany?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.serialNumber?</t>
         </is>
       </c>
       <c r="G181" s="4" t="inlineStr">
@@ -30457,7 +30477,7 @@
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>raStatus</t>
+          <t>quantityUsed</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
@@ -30478,7 +30498,7 @@
       </c>
       <c r="F182" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.raStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.quantityUsed?</t>
         </is>
       </c>
       <c r="G182" s="4" t="inlineStr">
@@ -30497,7 +30517,7 @@
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>Warehouse</t>
+          <t>deviceSerialNumber</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
@@ -30518,7 +30538,7 @@
       </c>
       <c r="F183" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.Warehouse?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.deviceSerialNumber?</t>
         </is>
       </c>
       <c r="G183" s="4" t="inlineStr">
@@ -30537,7 +30557,7 @@
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>assignedPerson</t>
+          <t>orderedPartId</t>
         </is>
       </c>
       <c r="B184" s="4" t="inlineStr">
@@ -30558,7 +30578,7 @@
       </c>
       <c r="F184" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.assignedPerson?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderedPartId?</t>
         </is>
       </c>
       <c r="G184" s="4" t="inlineStr">
@@ -30577,7 +30597,7 @@
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>resolvedDateTime</t>
+          <t>actualPartId</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
@@ -30598,7 +30618,7 @@
       </c>
       <c r="F185" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.resolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.actualPartId?</t>
         </is>
       </c>
       <c r="G185" s="4" t="inlineStr">
@@ -30617,12 +30637,12 @@
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>serialNumber</t>
+          <t>partCode</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C186" s="4" t="inlineStr">
@@ -30638,7 +30658,7 @@
       </c>
       <c r="F186" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.serialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
         </is>
       </c>
       <c r="G186" s="4" t="inlineStr">
@@ -30657,12 +30677,12 @@
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>quantityUsed</t>
+          <t>modelCode</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C187" s="4" t="inlineStr">
@@ -30678,7 +30698,7 @@
       </c>
       <c r="F187" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.quantityUsed?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
         </is>
       </c>
       <c r="G187" s="4" t="inlineStr">
@@ -30697,12 +30717,12 @@
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>deviceSerialNumber</t>
+          <t>modelDescription</t>
         </is>
       </c>
       <c r="B188" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C188" s="4" t="inlineStr">
@@ -30718,7 +30738,7 @@
       </c>
       <c r="F188" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.deviceSerialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
         </is>
       </c>
       <c r="G188" s="4" t="inlineStr">
@@ -30737,12 +30757,12 @@
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>orderedPartId</t>
+          <t>inventoryTransferImoId</t>
         </is>
       </c>
       <c r="B189" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C189" s="4" t="inlineStr">
@@ -30758,7 +30778,7 @@
       </c>
       <c r="F189" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderedPartId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.inventoryTransferImoId?</t>
         </is>
       </c>
       <c r="G189" s="4" t="inlineStr">
@@ -30777,12 +30797,12 @@
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>actualPartId</t>
+          <t>createdDateTime</t>
         </is>
       </c>
       <c r="B190" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C190" s="4" t="inlineStr">
@@ -30798,7 +30818,7 @@
       </c>
       <c r="F190" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.actualPartId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.createdDateTime?</t>
         </is>
       </c>
       <c r="G190" s="4" t="inlineStr">
@@ -30817,12 +30837,12 @@
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>partCode</t>
+          <t>completedDateTime</t>
         </is>
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr">
@@ -30838,7 +30858,7 @@
       </c>
       <c r="F191" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.completedDateTime?</t>
         </is>
       </c>
       <c r="G191" s="4" t="inlineStr">
@@ -30857,12 +30877,12 @@
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>modelCode</t>
+          <t>fromWarehouseId</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C192" s="4" t="inlineStr">
@@ -30878,7 +30898,7 @@
       </c>
       <c r="F192" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.fromWarehouseId?</t>
         </is>
       </c>
       <c r="G192" s="4" t="inlineStr">
@@ -30897,12 +30917,12 @@
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>modelDescription</t>
+          <t>toWarehouseId</t>
         </is>
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C193" s="4" t="inlineStr">
@@ -30918,7 +30938,7 @@
       </c>
       <c r="F193" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.toWarehouseId?</t>
         </is>
       </c>
       <c r="G193" s="4" t="inlineStr">
@@ -30937,7 +30957,7 @@
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>inventoryTransferImoId</t>
+          <t>demandStatus</t>
         </is>
       </c>
       <c r="B194" s="4" t="inlineStr">
@@ -30958,7 +30978,7 @@
       </c>
       <c r="F194" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.inventoryTransferImoId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.demandStatus?</t>
         </is>
       </c>
       <c r="G194" s="4" t="inlineStr">
@@ -30977,7 +30997,7 @@
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>createdDateTime</t>
+          <t>orderStatusIsClosed</t>
         </is>
       </c>
       <c r="B195" s="4" t="inlineStr">
@@ -30998,7 +31018,7 @@
       </c>
       <c r="F195" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.createdDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.orderStatusIsClosed?</t>
         </is>
       </c>
       <c r="G195" s="4" t="inlineStr">
@@ -31017,7 +31037,7 @@
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>completedDateTime</t>
+          <t>movementType</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
@@ -31038,7 +31058,7 @@
       </c>
       <c r="F196" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.completedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
         </is>
       </c>
       <c r="G196" s="4" t="inlineStr">
@@ -31057,7 +31077,7 @@
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>fromWarehouseId</t>
+          <t>addressId</t>
         </is>
       </c>
       <c r="B197" s="4" t="inlineStr">
@@ -31078,7 +31098,7 @@
       </c>
       <c r="F197" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.fromWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
         </is>
       </c>
       <c r="G197" s="4" t="inlineStr">
@@ -31097,7 +31117,7 @@
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>toWarehouseId</t>
+          <t>Bpart</t>
         </is>
       </c>
       <c r="B198" s="4" t="inlineStr">
@@ -31118,7 +31138,7 @@
       </c>
       <c r="F198" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.toWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.Bpart?</t>
         </is>
       </c>
       <c r="G198" s="4" t="inlineStr">
@@ -31137,7 +31157,7 @@
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>demandStatus</t>
+          <t>quantity</t>
         </is>
       </c>
       <c r="B199" s="4" t="inlineStr">
@@ -31158,7 +31178,7 @@
       </c>
       <c r="F199" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.demandStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.quantity?</t>
         </is>
       </c>
       <c r="G199" s="4" t="inlineStr">
@@ -31177,7 +31197,7 @@
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>orderStatusIsClosed</t>
+          <t>shipListCode</t>
         </is>
       </c>
       <c r="B200" s="4" t="inlineStr">
@@ -31198,7 +31218,7 @@
       </c>
       <c r="F200" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.orderStatusIsClosed?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
         </is>
       </c>
       <c r="G200" s="4" t="inlineStr">
@@ -31215,54 +31235,54 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="4" t="inlineStr">
-        <is>
-          <t>movementType</t>
-        </is>
-      </c>
-      <c r="B201" s="4" t="inlineStr">
-        <is>
-          <t>InventoryTransfers</t>
-        </is>
-      </c>
-      <c r="C201" s="4" t="inlineStr">
+      <c r="A201" s="3" t="inlineStr">
+        <is>
+          <t>demandStatus</t>
+        </is>
+      </c>
+      <c r="B201" s="3" t="inlineStr">
+        <is>
+          <t>PurchaseOrders</t>
+        </is>
+      </c>
+      <c r="C201" s="3" t="inlineStr">
         <is>
           <t>Planning V2 template</t>
         </is>
       </c>
-      <c r="D201" s="4" t="inlineStr"/>
-      <c r="E201" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F201" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
-        </is>
-      </c>
-      <c r="G201" s="4" t="inlineStr">
+      <c r="D201" s="3" t="inlineStr"/>
+      <c r="E201" s="3" t="inlineStr">
+        <is>
+          <t>Review required</t>
+        </is>
+      </c>
+      <c r="F201" s="3" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
+        </is>
+      </c>
+      <c r="G201" s="3" t="inlineStr">
         <is>
           <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
         </is>
       </c>
-      <c r="H201" s="4" t="inlineStr"/>
-      <c r="I201" s="4" t="inlineStr"/>
-      <c r="J201" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="H201" s="3" t="inlineStr"/>
+      <c r="I201" s="3" t="inlineStr"/>
+      <c r="J201" s="3" t="inlineStr">
+        <is>
+          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.NumAtCard and part/SPL Master evidence also matches.</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>addressId</t>
+          <t>partType</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C202" s="4" t="inlineStr">
@@ -31278,7 +31298,7 @@
       </c>
       <c r="F202" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.partType?</t>
         </is>
       </c>
       <c r="G202" s="4" t="inlineStr">
@@ -31297,12 +31317,12 @@
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>Bpart</t>
+          <t>partTypeDescription</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C203" s="4" t="inlineStr">
@@ -31318,7 +31338,7 @@
       </c>
       <c r="F203" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.Bpart?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeDescription?</t>
         </is>
       </c>
       <c r="G203" s="4" t="inlineStr">
@@ -31337,12 +31357,12 @@
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>isReworkable</t>
         </is>
       </c>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C204" s="4" t="inlineStr">
@@ -31358,7 +31378,7 @@
       </c>
       <c r="F204" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.quantity?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.isReworkable?</t>
         </is>
       </c>
       <c r="G204" s="4" t="inlineStr">
@@ -31377,12 +31397,12 @@
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>shipListCode</t>
+          <t>partNumber</t>
         </is>
       </c>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C205" s="4" t="inlineStr">
@@ -31398,7 +31418,7 @@
       </c>
       <c r="F205" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
         </is>
       </c>
       <c r="G205" s="4" t="inlineStr">
@@ -31415,54 +31435,54 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="3" t="inlineStr">
-        <is>
-          <t>demandStatus</t>
-        </is>
-      </c>
-      <c r="B206" s="3" t="inlineStr">
-        <is>
-          <t>PurchaseOrders</t>
-        </is>
-      </c>
-      <c r="C206" s="3" t="inlineStr">
+      <c r="A206" s="4" t="inlineStr">
+        <is>
+          <t>unitOfMeasure</t>
+        </is>
+      </c>
+      <c r="B206" s="4" t="inlineStr">
+        <is>
+          <t>Yields</t>
+        </is>
+      </c>
+      <c r="C206" s="4" t="inlineStr">
         <is>
           <t>Planning V2 template</t>
         </is>
       </c>
-      <c r="D206" s="3" t="inlineStr"/>
-      <c r="E206" s="3" t="inlineStr">
-        <is>
-          <t>Review required</t>
-        </is>
-      </c>
-      <c r="F206" s="3" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
-        </is>
-      </c>
-      <c r="G206" s="3" t="inlineStr">
+      <c r="D206" s="4" t="inlineStr"/>
+      <c r="E206" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F206" s="4" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
+        </is>
+      </c>
+      <c r="G206" s="4" t="inlineStr">
         <is>
           <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
         </is>
       </c>
-      <c r="H206" s="3" t="inlineStr"/>
-      <c r="I206" s="3" t="inlineStr"/>
-      <c r="J206" s="3" t="inlineStr">
-        <is>
-          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.NumAtCard and part/SPL Master evidence also matches.</t>
+      <c r="H206" s="4" t="inlineStr"/>
+      <c r="I206" s="4" t="inlineStr"/>
+      <c r="J206" s="4" t="inlineStr">
+        <is>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>partType</t>
+          <t>yield</t>
         </is>
       </c>
       <c r="B207" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C207" s="4" t="inlineStr">
@@ -31478,7 +31498,7 @@
       </c>
       <c r="F207" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partType?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
         </is>
       </c>
       <c r="G207" s="4" t="inlineStr">
@@ -31497,12 +31517,12 @@
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
         <is>
-          <t>partTypeDescription</t>
+          <t>Secondary TO</t>
         </is>
       </c>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C208" s="4" t="inlineStr">
@@ -31518,7 +31538,7 @@
       </c>
       <c r="F208" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeDescription?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary TO?</t>
         </is>
       </c>
       <c r="G208" s="4" t="inlineStr">
@@ -31537,12 +31557,12 @@
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t>isReworkable</t>
+          <t>Secondary FROM</t>
         </is>
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C209" s="4" t="inlineStr">
@@ -31558,7 +31578,7 @@
       </c>
       <c r="F209" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.isReworkable?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary FROM?</t>
         </is>
       </c>
       <c r="G209" s="4" t="inlineStr">
@@ -31577,12 +31597,12 @@
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
         <is>
-          <t>partNumber</t>
+          <t>Cross TO</t>
         </is>
       </c>
       <c r="B210" s="4" t="inlineStr">
         <is>
-          <t>Yields</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C210" s="4" t="inlineStr">
@@ -31598,7 +31618,7 @@
       </c>
       <c r="F210" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross TO?</t>
         </is>
       </c>
       <c r="G210" s="4" t="inlineStr">
@@ -31617,12 +31637,12 @@
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
         <is>
-          <t>unitOfMeasure</t>
+          <t>Cross FROM</t>
         </is>
       </c>
       <c r="B211" s="4" t="inlineStr">
         <is>
-          <t>Yields</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C211" s="4" t="inlineStr">
@@ -31638,7 +31658,7 @@
       </c>
       <c r="F211" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross FROM?</t>
         </is>
       </c>
       <c r="G211" s="4" t="inlineStr">
@@ -31657,12 +31677,12 @@
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
         <is>
-          <t>yield</t>
+          <t>Primary TO</t>
         </is>
       </c>
       <c r="B212" s="4" t="inlineStr">
         <is>
-          <t>Yields</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C212" s="4" t="inlineStr">
@@ -31678,7 +31698,7 @@
       </c>
       <c r="F212" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Primary TO?</t>
         </is>
       </c>
       <c r="G212" s="4" t="inlineStr">
@@ -31694,208 +31714,8 @@
         </is>
       </c>
     </row>
-    <row r="213">
-      <c r="A213" s="4" t="inlineStr">
-        <is>
-          <t>Secondary TO</t>
-        </is>
-      </c>
-      <c r="B213" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C213" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D213" s="4" t="inlineStr"/>
-      <c r="E213" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F213" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary TO?</t>
-        </is>
-      </c>
-      <c r="G213" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H213" s="4" t="inlineStr"/>
-      <c r="I213" s="4" t="inlineStr"/>
-      <c r="J213" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" s="4" t="inlineStr">
-        <is>
-          <t>Secondary FROM</t>
-        </is>
-      </c>
-      <c r="B214" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C214" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D214" s="4" t="inlineStr"/>
-      <c r="E214" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F214" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary FROM?</t>
-        </is>
-      </c>
-      <c r="G214" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H214" s="4" t="inlineStr"/>
-      <c r="I214" s="4" t="inlineStr"/>
-      <c r="J214" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" s="4" t="inlineStr">
-        <is>
-          <t>Cross TO</t>
-        </is>
-      </c>
-      <c r="B215" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C215" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D215" s="4" t="inlineStr"/>
-      <c r="E215" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F215" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross TO?</t>
-        </is>
-      </c>
-      <c r="G215" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H215" s="4" t="inlineStr"/>
-      <c r="I215" s="4" t="inlineStr"/>
-      <c r="J215" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" s="4" t="inlineStr">
-        <is>
-          <t>Cross FROM</t>
-        </is>
-      </c>
-      <c r="B216" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C216" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D216" s="4" t="inlineStr"/>
-      <c r="E216" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F216" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross FROM?</t>
-        </is>
-      </c>
-      <c r="G216" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H216" s="4" t="inlineStr"/>
-      <c r="I216" s="4" t="inlineStr"/>
-      <c r="J216" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" s="4" t="inlineStr">
-        <is>
-          <t>Primary TO</t>
-        </is>
-      </c>
-      <c r="B217" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C217" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D217" s="4" t="inlineStr"/>
-      <c r="E217" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F217" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Primary TO?</t>
-        </is>
-      </c>
-      <c r="G217" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H217" s="4" t="inlineStr"/>
-      <c r="I217" s="4" t="inlineStr"/>
-      <c r="J217" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J217"/>
+  <autoFilter ref="A1:J212"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -32396,7 +32216,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>isBootStockable; isBranchStockable; productClass; productType; costCategory; partType; isKit; isObsolete; isExcludeFromReplenishment; purchaseLeadTimeDays; isCritical</t>
+          <t>productClass; productType; costCategory; partType; isKit; isCritical</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Enrich usage status from helpdesk calls
</commit_message>
<xml_diff>
--- a/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
+++ b/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Target Fields'!$A$1:$S$151</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Template Fields'!$A$1:$H$177</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Evidence'!$A$1:$D$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$J$212</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$J$210</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Output Objects'!$A$1:$E$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Missing Important Fields'!$A$1:$E$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'SAP Investigation Log'!$A$1:$E$10</definedName>
@@ -244,8 +244,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:J212" headerRowCount="1">
-  <autoFilter ref="A1:J212"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:J210" headerRowCount="1">
+  <autoFilter ref="A1:J210"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Field"/>
     <tableColumn id="2" name="Object"/>
@@ -18067,78 +18067,86 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="4" t="inlineStr">
+      <c r="A84" s="2" t="inlineStr">
         <is>
           <t>PartsUsage</t>
         </is>
       </c>
-      <c r="B84" s="4" t="inlineStr">
+      <c r="B84" s="2" t="inlineStr">
         <is>
           <t>orderStartDatetime</t>
         </is>
       </c>
-      <c r="C84" s="4" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr">
         <is>
           <t>DateTime</t>
         </is>
       </c>
-      <c r="D84" s="4" t="inlineStr">
+      <c r="D84" s="2" t="inlineStr">
         <is>
           <t>Canonical header from PartsUsage.xlsx</t>
         </is>
       </c>
-      <c r="E84" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F84" s="4" t="inlineStr"/>
-      <c r="G84" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H84" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>HelpDesk issue tracker Created date by unambiguous call-number match</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="4" t="inlineStr">
+      <c r="A85" s="2" t="inlineStr">
         <is>
           <t>PartsUsage</t>
         </is>
       </c>
-      <c r="B85" s="4" t="inlineStr">
+      <c r="B85" s="2" t="inlineStr">
         <is>
           <t>orderStatus</t>
         </is>
       </c>
-      <c r="C85" s="4" t="inlineStr">
+      <c r="C85" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D85" s="4" t="inlineStr">
+      <c r="D85" s="2" t="inlineStr">
         <is>
           <t>Canonical header from PartsUsage.xlsx</t>
         </is>
       </c>
-      <c r="E85" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F85" s="4" t="inlineStr"/>
-      <c r="G85" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H85" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>HelpDesk issue tracker Status by unambiguous call-number match</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -22019,7 +22027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J212"/>
+  <dimension ref="A1:J210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -29117,7 +29125,7 @@
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>orderStartDatetime</t>
+          <t>resolvedDateTime</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
@@ -29138,7 +29146,7 @@
       </c>
       <c r="F148" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStartDatetime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.resolvedDateTime?</t>
         </is>
       </c>
       <c r="G148" s="4" t="inlineStr">
@@ -29157,7 +29165,7 @@
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>orderStatus</t>
+          <t>relCompanyId</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
@@ -29178,7 +29186,7 @@
       </c>
       <c r="F149" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.relCompanyId?</t>
         </is>
       </c>
       <c r="G149" s="4" t="inlineStr">
@@ -29197,7 +29205,7 @@
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>resolvedDateTime</t>
+          <t>assignedPersonCode</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
@@ -29218,7 +29226,7 @@
       </c>
       <c r="F150" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.resolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.assignedPersonCode?</t>
         </is>
       </c>
       <c r="G150" s="4" t="inlineStr">
@@ -29237,12 +29245,12 @@
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>relCompanyId</t>
+          <t>orderNumber</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
@@ -29258,7 +29266,7 @@
       </c>
       <c r="F151" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.relCompanyId?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.orderNumber?</t>
         </is>
       </c>
       <c r="G151" s="4" t="inlineStr">
@@ -29277,12 +29285,12 @@
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>assignedPersonCode</t>
+          <t>RequestID</t>
         </is>
       </c>
       <c r="B152" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C152" s="4" t="inlineStr">
@@ -29298,7 +29306,7 @@
       </c>
       <c r="F152" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.assignedPersonCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.RequestID?</t>
         </is>
       </c>
       <c r="G152" s="4" t="inlineStr">
@@ -29317,7 +29325,7 @@
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>orderNumber</t>
+          <t>location</t>
         </is>
       </c>
       <c r="B153" s="4" t="inlineStr">
@@ -29338,7 +29346,7 @@
       </c>
       <c r="F153" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.orderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.location?</t>
         </is>
       </c>
       <c r="G153" s="4" t="inlineStr">
@@ -29357,7 +29365,7 @@
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>RequestID</t>
+          <t>eta</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
@@ -29378,7 +29386,7 @@
       </c>
       <c r="F154" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.RequestID?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.eta?</t>
         </is>
       </c>
       <c r="G154" s="4" t="inlineStr">
@@ -29397,7 +29405,7 @@
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>actualEta</t>
         </is>
       </c>
       <c r="B155" s="4" t="inlineStr">
@@ -29418,7 +29426,7 @@
       </c>
       <c r="F155" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.location?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualEta?</t>
         </is>
       </c>
       <c r="G155" s="4" t="inlineStr">
@@ -29437,7 +29445,7 @@
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>eta</t>
+          <t>actualResolveDateTime</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
@@ -29458,7 +29466,7 @@
       </c>
       <c r="F156" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.eta?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualResolveDateTime?</t>
         </is>
       </c>
       <c r="G156" s="4" t="inlineStr">
@@ -29477,7 +29485,7 @@
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>actualEta</t>
+          <t>recallDateTime</t>
         </is>
       </c>
       <c r="B157" s="4" t="inlineStr">
@@ -29498,7 +29506,7 @@
       </c>
       <c r="F157" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualEta?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.recallDateTime?</t>
         </is>
       </c>
       <c r="G157" s="4" t="inlineStr">
@@ -29517,7 +29525,7 @@
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>actualResolveDateTime</t>
+          <t>actualRecallDateTime</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
@@ -29538,7 +29546,7 @@
       </c>
       <c r="F158" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualResolveDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualRecallDateTime?</t>
         </is>
       </c>
       <c r="G158" s="4" t="inlineStr">
@@ -29557,7 +29565,7 @@
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>recallDateTime</t>
+          <t>slaEtaClock</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
@@ -29578,7 +29586,7 @@
       </c>
       <c r="F159" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.recallDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaClock?</t>
         </is>
       </c>
       <c r="G159" s="4" t="inlineStr">
@@ -29597,7 +29605,7 @@
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>actualRecallDateTime</t>
+          <t>slaResolveClock</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
@@ -29618,7 +29626,7 @@
       </c>
       <c r="F160" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualRecallDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveClock?</t>
         </is>
       </c>
       <c r="G160" s="4" t="inlineStr">
@@ -29637,7 +29645,7 @@
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>slaEtaClock</t>
+          <t>slaFailureCode</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
@@ -29658,7 +29666,7 @@
       </c>
       <c r="F161" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaClock?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaFailureCode?</t>
         </is>
       </c>
       <c r="G161" s="4" t="inlineStr">
@@ -29677,7 +29685,7 @@
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>slaResolveClock</t>
+          <t>slaEtaHit</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
@@ -29698,7 +29706,7 @@
       </c>
       <c r="F162" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveClock?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaHit?</t>
         </is>
       </c>
       <c r="G162" s="4" t="inlineStr">
@@ -29717,7 +29725,7 @@
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>slaFailureCode</t>
+          <t>slaResolveDateTime</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
@@ -29738,7 +29746,7 @@
       </c>
       <c r="F163" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaFailureCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveDateTime?</t>
         </is>
       </c>
       <c r="G163" s="4" t="inlineStr">
@@ -29757,12 +29765,12 @@
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>slaEtaHit</t>
+          <t>orderNumber</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C164" s="4" t="inlineStr">
@@ -29778,7 +29786,7 @@
       </c>
       <c r="F164" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaHit?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderNumber?</t>
         </is>
       </c>
       <c r="G164" s="4" t="inlineStr">
@@ -29797,12 +29805,12 @@
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t>slaResolveDateTime</t>
+          <t>requestId</t>
         </is>
       </c>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C165" s="4" t="inlineStr">
@@ -29818,7 +29826,7 @@
       </c>
       <c r="F165" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.requestId?</t>
         </is>
       </c>
       <c r="G165" s="4" t="inlineStr">
@@ -29837,7 +29845,7 @@
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>orderNumber</t>
+          <t>customerCompanyCode</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
@@ -29858,7 +29866,7 @@
       </c>
       <c r="F166" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.customerCompanyCode?</t>
         </is>
       </c>
       <c r="G166" s="4" t="inlineStr">
@@ -29877,7 +29885,7 @@
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>requestId</t>
+          <t>orderStatus</t>
         </is>
       </c>
       <c r="B167" s="4" t="inlineStr">
@@ -29898,7 +29906,7 @@
       </c>
       <c r="F167" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.requestId?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStatus?</t>
         </is>
       </c>
       <c r="G167" s="4" t="inlineStr">
@@ -29917,7 +29925,7 @@
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>customerCompanyCode</t>
+          <t>orderStartDatetime</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
@@ -29938,7 +29946,7 @@
       </c>
       <c r="F168" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.customerCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStartDatetime?</t>
         </is>
       </c>
       <c r="G168" s="4" t="inlineStr">
@@ -29957,7 +29965,7 @@
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>orderStatus</t>
+          <t>siteCompanyCode</t>
         </is>
       </c>
       <c r="B169" s="4" t="inlineStr">
@@ -29978,7 +29986,7 @@
       </c>
       <c r="F169" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.siteCompanyCode?</t>
         </is>
       </c>
       <c r="G169" s="4" t="inlineStr">
@@ -29997,7 +30005,7 @@
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>orderStartDatetime</t>
+          <t>repairType</t>
         </is>
       </c>
       <c r="B170" s="4" t="inlineStr">
@@ -30018,7 +30026,7 @@
       </c>
       <c r="F170" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStartDatetime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairType?</t>
         </is>
       </c>
       <c r="G170" s="4" t="inlineStr">
@@ -30037,7 +30045,7 @@
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>siteCompanyCode</t>
+          <t>partsOrderDateTime</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
@@ -30058,7 +30066,7 @@
       </c>
       <c r="F171" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.siteCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsOrderDateTime?</t>
         </is>
       </c>
       <c r="G171" s="4" t="inlineStr">
@@ -30077,7 +30085,7 @@
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>repairType</t>
+          <t>partsReceivedDateTime</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
@@ -30098,7 +30106,7 @@
       </c>
       <c r="F172" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairType?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsReceivedDateTime?</t>
         </is>
       </c>
       <c r="G172" s="4" t="inlineStr">
@@ -30117,7 +30125,7 @@
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>partsOrderDateTime</t>
+          <t>repairCode</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
@@ -30138,7 +30146,7 @@
       </c>
       <c r="F173" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsOrderDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCode?</t>
         </is>
       </c>
       <c r="G173" s="4" t="inlineStr">
@@ -30157,7 +30165,7 @@
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>partsReceivedDateTime</t>
+          <t>repairCompany</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
@@ -30178,7 +30186,7 @@
       </c>
       <c r="F174" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsReceivedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCompany?</t>
         </is>
       </c>
       <c r="G174" s="4" t="inlineStr">
@@ -30197,7 +30205,7 @@
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>repairCode</t>
+          <t>raStatus</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
@@ -30218,7 +30226,7 @@
       </c>
       <c r="F175" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.raStatus?</t>
         </is>
       </c>
       <c r="G175" s="4" t="inlineStr">
@@ -30237,7 +30245,7 @@
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>repairCompany</t>
+          <t>Warehouse</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
@@ -30258,7 +30266,7 @@
       </c>
       <c r="F176" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCompany?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.Warehouse?</t>
         </is>
       </c>
       <c r="G176" s="4" t="inlineStr">
@@ -30277,7 +30285,7 @@
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>raStatus</t>
+          <t>assignedPerson</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
@@ -30298,7 +30306,7 @@
       </c>
       <c r="F177" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.raStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.assignedPerson?</t>
         </is>
       </c>
       <c r="G177" s="4" t="inlineStr">
@@ -30317,7 +30325,7 @@
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>Warehouse</t>
+          <t>resolvedDateTime</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
@@ -30338,7 +30346,7 @@
       </c>
       <c r="F178" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.Warehouse?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.resolvedDateTime?</t>
         </is>
       </c>
       <c r="G178" s="4" t="inlineStr">
@@ -30357,7 +30365,7 @@
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>assignedPerson</t>
+          <t>serialNumber</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
@@ -30378,7 +30386,7 @@
       </c>
       <c r="F179" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.assignedPerson?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.serialNumber?</t>
         </is>
       </c>
       <c r="G179" s="4" t="inlineStr">
@@ -30397,7 +30405,7 @@
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>resolvedDateTime</t>
+          <t>quantityUsed</t>
         </is>
       </c>
       <c r="B180" s="4" t="inlineStr">
@@ -30418,7 +30426,7 @@
       </c>
       <c r="F180" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.resolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.quantityUsed?</t>
         </is>
       </c>
       <c r="G180" s="4" t="inlineStr">
@@ -30437,7 +30445,7 @@
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>serialNumber</t>
+          <t>deviceSerialNumber</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
@@ -30458,7 +30466,7 @@
       </c>
       <c r="F181" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.serialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.deviceSerialNumber?</t>
         </is>
       </c>
       <c r="G181" s="4" t="inlineStr">
@@ -30477,7 +30485,7 @@
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>quantityUsed</t>
+          <t>orderedPartId</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
@@ -30498,7 +30506,7 @@
       </c>
       <c r="F182" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.quantityUsed?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderedPartId?</t>
         </is>
       </c>
       <c r="G182" s="4" t="inlineStr">
@@ -30517,7 +30525,7 @@
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>deviceSerialNumber</t>
+          <t>actualPartId</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
@@ -30538,7 +30546,7 @@
       </c>
       <c r="F183" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.deviceSerialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.actualPartId?</t>
         </is>
       </c>
       <c r="G183" s="4" t="inlineStr">
@@ -30557,12 +30565,12 @@
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>orderedPartId</t>
+          <t>partCode</t>
         </is>
       </c>
       <c r="B184" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C184" s="4" t="inlineStr">
@@ -30578,7 +30586,7 @@
       </c>
       <c r="F184" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderedPartId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
         </is>
       </c>
       <c r="G184" s="4" t="inlineStr">
@@ -30597,12 +30605,12 @@
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>actualPartId</t>
+          <t>modelCode</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C185" s="4" t="inlineStr">
@@ -30618,7 +30626,7 @@
       </c>
       <c r="F185" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.actualPartId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
         </is>
       </c>
       <c r="G185" s="4" t="inlineStr">
@@ -30637,7 +30645,7 @@
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>partCode</t>
+          <t>modelDescription</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
@@ -30658,7 +30666,7 @@
       </c>
       <c r="F186" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
         </is>
       </c>
       <c r="G186" s="4" t="inlineStr">
@@ -30677,12 +30685,12 @@
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>modelCode</t>
+          <t>inventoryTransferImoId</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C187" s="4" t="inlineStr">
@@ -30698,7 +30706,7 @@
       </c>
       <c r="F187" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.inventoryTransferImoId?</t>
         </is>
       </c>
       <c r="G187" s="4" t="inlineStr">
@@ -30717,12 +30725,12 @@
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>modelDescription</t>
+          <t>createdDateTime</t>
         </is>
       </c>
       <c r="B188" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C188" s="4" t="inlineStr">
@@ -30738,7 +30746,7 @@
       </c>
       <c r="F188" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.createdDateTime?</t>
         </is>
       </c>
       <c r="G188" s="4" t="inlineStr">
@@ -30757,7 +30765,7 @@
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>inventoryTransferImoId</t>
+          <t>completedDateTime</t>
         </is>
       </c>
       <c r="B189" s="4" t="inlineStr">
@@ -30778,7 +30786,7 @@
       </c>
       <c r="F189" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.inventoryTransferImoId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.completedDateTime?</t>
         </is>
       </c>
       <c r="G189" s="4" t="inlineStr">
@@ -30797,7 +30805,7 @@
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>createdDateTime</t>
+          <t>fromWarehouseId</t>
         </is>
       </c>
       <c r="B190" s="4" t="inlineStr">
@@ -30818,7 +30826,7 @@
       </c>
       <c r="F190" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.createdDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.fromWarehouseId?</t>
         </is>
       </c>
       <c r="G190" s="4" t="inlineStr">
@@ -30837,7 +30845,7 @@
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>completedDateTime</t>
+          <t>toWarehouseId</t>
         </is>
       </c>
       <c r="B191" s="4" t="inlineStr">
@@ -30858,7 +30866,7 @@
       </c>
       <c r="F191" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.completedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.toWarehouseId?</t>
         </is>
       </c>
       <c r="G191" s="4" t="inlineStr">
@@ -30877,7 +30885,7 @@
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>fromWarehouseId</t>
+          <t>demandStatus</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
@@ -30898,7 +30906,7 @@
       </c>
       <c r="F192" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.fromWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.demandStatus?</t>
         </is>
       </c>
       <c r="G192" s="4" t="inlineStr">
@@ -30917,7 +30925,7 @@
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>toWarehouseId</t>
+          <t>orderStatusIsClosed</t>
         </is>
       </c>
       <c r="B193" s="4" t="inlineStr">
@@ -30938,7 +30946,7 @@
       </c>
       <c r="F193" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.toWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.orderStatusIsClosed?</t>
         </is>
       </c>
       <c r="G193" s="4" t="inlineStr">
@@ -30957,7 +30965,7 @@
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>demandStatus</t>
+          <t>movementType</t>
         </is>
       </c>
       <c r="B194" s="4" t="inlineStr">
@@ -30978,7 +30986,7 @@
       </c>
       <c r="F194" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.demandStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
         </is>
       </c>
       <c r="G194" s="4" t="inlineStr">
@@ -30997,7 +31005,7 @@
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>orderStatusIsClosed</t>
+          <t>addressId</t>
         </is>
       </c>
       <c r="B195" s="4" t="inlineStr">
@@ -31018,7 +31026,7 @@
       </c>
       <c r="F195" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.orderStatusIsClosed?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
         </is>
       </c>
       <c r="G195" s="4" t="inlineStr">
@@ -31037,7 +31045,7 @@
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>movementType</t>
+          <t>Bpart</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
@@ -31058,7 +31066,7 @@
       </c>
       <c r="F196" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.Bpart?</t>
         </is>
       </c>
       <c r="G196" s="4" t="inlineStr">
@@ -31077,7 +31085,7 @@
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>addressId</t>
+          <t>quantity</t>
         </is>
       </c>
       <c r="B197" s="4" t="inlineStr">
@@ -31098,7 +31106,7 @@
       </c>
       <c r="F197" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.quantity?</t>
         </is>
       </c>
       <c r="G197" s="4" t="inlineStr">
@@ -31117,7 +31125,7 @@
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>Bpart</t>
+          <t>shipListCode</t>
         </is>
       </c>
       <c r="B198" s="4" t="inlineStr">
@@ -31138,7 +31146,7 @@
       </c>
       <c r="F198" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.Bpart?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
         </is>
       </c>
       <c r="G198" s="4" t="inlineStr">
@@ -31155,54 +31163,54 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="4" t="inlineStr">
-        <is>
-          <t>quantity</t>
-        </is>
-      </c>
-      <c r="B199" s="4" t="inlineStr">
-        <is>
-          <t>InventoryTransfers</t>
-        </is>
-      </c>
-      <c r="C199" s="4" t="inlineStr">
+      <c r="A199" s="3" t="inlineStr">
+        <is>
+          <t>demandStatus</t>
+        </is>
+      </c>
+      <c r="B199" s="3" t="inlineStr">
+        <is>
+          <t>PurchaseOrders</t>
+        </is>
+      </c>
+      <c r="C199" s="3" t="inlineStr">
         <is>
           <t>Planning V2 template</t>
         </is>
       </c>
-      <c r="D199" s="4" t="inlineStr"/>
-      <c r="E199" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F199" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.quantity?</t>
-        </is>
-      </c>
-      <c r="G199" s="4" t="inlineStr">
+      <c r="D199" s="3" t="inlineStr"/>
+      <c r="E199" s="3" t="inlineStr">
+        <is>
+          <t>Review required</t>
+        </is>
+      </c>
+      <c r="F199" s="3" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
+        </is>
+      </c>
+      <c r="G199" s="3" t="inlineStr">
         <is>
           <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
         </is>
       </c>
-      <c r="H199" s="4" t="inlineStr"/>
-      <c r="I199" s="4" t="inlineStr"/>
-      <c r="J199" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="H199" s="3" t="inlineStr"/>
+      <c r="I199" s="3" t="inlineStr"/>
+      <c r="J199" s="3" t="inlineStr">
+        <is>
+          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.NumAtCard and part/SPL Master evidence also matches.</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>shipListCode</t>
+          <t>partType</t>
         </is>
       </c>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C200" s="4" t="inlineStr">
@@ -31218,7 +31226,7 @@
       </c>
       <c r="F200" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.partType?</t>
         </is>
       </c>
       <c r="G200" s="4" t="inlineStr">
@@ -31235,49 +31243,49 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="3" t="inlineStr">
-        <is>
-          <t>demandStatus</t>
-        </is>
-      </c>
-      <c r="B201" s="3" t="inlineStr">
-        <is>
-          <t>PurchaseOrders</t>
-        </is>
-      </c>
-      <c r="C201" s="3" t="inlineStr">
+      <c r="A201" s="4" t="inlineStr">
+        <is>
+          <t>partTypeDescription</t>
+        </is>
+      </c>
+      <c r="B201" s="4" t="inlineStr">
+        <is>
+          <t>PartTypes</t>
+        </is>
+      </c>
+      <c r="C201" s="4" t="inlineStr">
         <is>
           <t>Planning V2 template</t>
         </is>
       </c>
-      <c r="D201" s="3" t="inlineStr"/>
-      <c r="E201" s="3" t="inlineStr">
-        <is>
-          <t>Review required</t>
-        </is>
-      </c>
-      <c r="F201" s="3" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
-        </is>
-      </c>
-      <c r="G201" s="3" t="inlineStr">
+      <c r="D201" s="4" t="inlineStr"/>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F201" s="4" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeDescription?</t>
+        </is>
+      </c>
+      <c r="G201" s="4" t="inlineStr">
         <is>
           <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
         </is>
       </c>
-      <c r="H201" s="3" t="inlineStr"/>
-      <c r="I201" s="3" t="inlineStr"/>
-      <c r="J201" s="3" t="inlineStr">
-        <is>
-          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.NumAtCard and part/SPL Master evidence also matches.</t>
+      <c r="H201" s="4" t="inlineStr"/>
+      <c r="I201" s="4" t="inlineStr"/>
+      <c r="J201" s="4" t="inlineStr">
+        <is>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>partType</t>
+          <t>isReworkable</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
@@ -31298,7 +31306,7 @@
       </c>
       <c r="F202" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partType?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.isReworkable?</t>
         </is>
       </c>
       <c r="G202" s="4" t="inlineStr">
@@ -31317,12 +31325,12 @@
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>partTypeDescription</t>
+          <t>partNumber</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C203" s="4" t="inlineStr">
@@ -31338,7 +31346,7 @@
       </c>
       <c r="F203" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeDescription?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
         </is>
       </c>
       <c r="G203" s="4" t="inlineStr">
@@ -31357,12 +31365,12 @@
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>isReworkable</t>
+          <t>unitOfMeasure</t>
         </is>
       </c>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C204" s="4" t="inlineStr">
@@ -31378,7 +31386,7 @@
       </c>
       <c r="F204" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.isReworkable?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
         </is>
       </c>
       <c r="G204" s="4" t="inlineStr">
@@ -31397,7 +31405,7 @@
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>partNumber</t>
+          <t>yield</t>
         </is>
       </c>
       <c r="B205" s="4" t="inlineStr">
@@ -31418,7 +31426,7 @@
       </c>
       <c r="F205" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
         </is>
       </c>
       <c r="G205" s="4" t="inlineStr">
@@ -31437,12 +31445,12 @@
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
         <is>
-          <t>unitOfMeasure</t>
+          <t>Secondary TO</t>
         </is>
       </c>
       <c r="B206" s="4" t="inlineStr">
         <is>
-          <t>Yields</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C206" s="4" t="inlineStr">
@@ -31458,7 +31466,7 @@
       </c>
       <c r="F206" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary TO?</t>
         </is>
       </c>
       <c r="G206" s="4" t="inlineStr">
@@ -31477,12 +31485,12 @@
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>yield</t>
+          <t>Secondary FROM</t>
         </is>
       </c>
       <c r="B207" s="4" t="inlineStr">
         <is>
-          <t>Yields</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C207" s="4" t="inlineStr">
@@ -31498,7 +31506,7 @@
       </c>
       <c r="F207" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary FROM?</t>
         </is>
       </c>
       <c r="G207" s="4" t="inlineStr">
@@ -31517,7 +31525,7 @@
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
         <is>
-          <t>Secondary TO</t>
+          <t>Cross TO</t>
         </is>
       </c>
       <c r="B208" s="4" t="inlineStr">
@@ -31538,7 +31546,7 @@
       </c>
       <c r="F208" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary TO?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross TO?</t>
         </is>
       </c>
       <c r="G208" s="4" t="inlineStr">
@@ -31557,7 +31565,7 @@
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t>Secondary FROM</t>
+          <t>Cross FROM</t>
         </is>
       </c>
       <c r="B209" s="4" t="inlineStr">
@@ -31578,7 +31586,7 @@
       </c>
       <c r="F209" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary FROM?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross FROM?</t>
         </is>
       </c>
       <c r="G209" s="4" t="inlineStr">
@@ -31597,7 +31605,7 @@
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
         <is>
-          <t>Cross TO</t>
+          <t>Primary TO</t>
         </is>
       </c>
       <c r="B210" s="4" t="inlineStr">
@@ -31618,7 +31626,7 @@
       </c>
       <c r="F210" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross TO?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Primary TO?</t>
         </is>
       </c>
       <c r="G210" s="4" t="inlineStr">
@@ -31634,88 +31642,8 @@
         </is>
       </c>
     </row>
-    <row r="211">
-      <c r="A211" s="4" t="inlineStr">
-        <is>
-          <t>Cross FROM</t>
-        </is>
-      </c>
-      <c r="B211" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C211" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D211" s="4" t="inlineStr"/>
-      <c r="E211" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F211" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross FROM?</t>
-        </is>
-      </c>
-      <c r="G211" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H211" s="4" t="inlineStr"/>
-      <c r="I211" s="4" t="inlineStr"/>
-      <c r="J211" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" s="4" t="inlineStr">
-        <is>
-          <t>Primary TO</t>
-        </is>
-      </c>
-      <c r="B212" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C212" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D212" s="4" t="inlineStr"/>
-      <c r="E212" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F212" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Primary TO?</t>
-        </is>
-      </c>
-      <c r="G212" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H212" s="4" t="inlineStr"/>
-      <c r="I212" s="4" t="inlineStr"/>
-      <c r="J212" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J212"/>
+  <autoFilter ref="A1:J210"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -32343,7 +32271,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>OrderType; orderStartDatetime; orderStatus; resolvedDateTime; relCompanyId; assignedPersonCode</t>
+          <t>OrderType; resolvedDateTime; relCompanyId; assignedPersonCode</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Set service order type for usage
</commit_message>
<xml_diff>
--- a/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
+++ b/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Target Fields'!$A$1:$S$151</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Template Fields'!$A$1:$H$177</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Evidence'!$A$1:$D$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$J$210</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$J$200</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Output Objects'!$A$1:$E$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Missing Important Fields'!$A$1:$E$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'SAP Investigation Log'!$A$1:$E$10</definedName>
@@ -244,8 +244,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:J210" headerRowCount="1">
-  <autoFilter ref="A1:J210"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:J200" headerRowCount="1">
+  <autoFilter ref="A1:J200"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Field"/>
     <tableColumn id="2" name="Object"/>
@@ -15359,36 +15359,40 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Vendors</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>vendorId</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Canonical header from Vendors.xlsx</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr"/>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>SAP Service Layer SQLQueries:OPOR.CardCode</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -15427,40 +15431,44 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Vendors</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>isActive</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Boolean</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Canonical header from Vendors.xlsx</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr"/>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>SAP Service Layer SQLQueries:OCRD.validFor joined from PO vendor</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -17189,40 +17197,36 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+      <c r="A61" s="4" t="inlineStr">
         <is>
           <t>WarehouseStockOnHand</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B61" s="4" t="inlineStr">
         <is>
           <t>partNumber</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr"/>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="C61" s="4" t="inlineStr"/>
+      <c r="D61" s="4" t="inlineStr">
         <is>
           <t>Canonical header from Warehouse Stock on Hand.xlsx</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="F61" s="2" t="inlineStr">
-        <is>
-          <t>SAP Service Layer SQLQueries:OITW.ItemCode</t>
-        </is>
-      </c>
-      <c r="G61" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H61" s="2" t="inlineStr">
-        <is>
-          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr"/>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
@@ -17991,36 +17995,40 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="4" t="inlineStr">
+      <c r="A82" s="2" t="inlineStr">
         <is>
           <t>PartsUsage</t>
         </is>
       </c>
-      <c r="B82" s="4" t="inlineStr">
+      <c r="B82" s="2" t="inlineStr">
         <is>
           <t>OrderType</t>
         </is>
       </c>
-      <c r="C82" s="4" t="inlineStr"/>
-      <c r="D82" s="4" t="inlineStr">
+      <c r="C82" s="2" t="inlineStr"/>
+      <c r="D82" s="2" t="inlineStr">
         <is>
           <t>Canonical header from PartsUsage.xlsx</t>
         </is>
       </c>
-      <c r="E82" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F82" s="4" t="inlineStr"/>
-      <c r="G82" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H82" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Business rule: service_order for all CoCre8 usage</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -20117,268 +20125,296 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="4" t="inlineStr">
+      <c r="A137" s="2" t="inlineStr">
         <is>
           <t>InventoryTransfers</t>
         </is>
       </c>
-      <c r="B137" s="4" t="inlineStr">
+      <c r="B137" s="2" t="inlineStr">
         <is>
           <t>inventoryTransferImoId</t>
         </is>
       </c>
-      <c r="C137" s="4" t="inlineStr">
+      <c r="C137" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D137" s="4" t="inlineStr">
+      <c r="D137" s="2" t="inlineStr">
         <is>
           <t>Canonical header from Inventory Transfers.xlsx</t>
         </is>
       </c>
-      <c r="E137" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F137" s="4" t="inlineStr"/>
-      <c r="G137" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H137" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>Stock Audit Report.txt:Document + Item No. + absolute Quantity + pair sequence for IM rows</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="4" t="inlineStr">
+      <c r="A138" s="2" t="inlineStr">
         <is>
           <t>InventoryTransfers</t>
         </is>
       </c>
-      <c r="B138" s="4" t="inlineStr">
+      <c r="B138" s="2" t="inlineStr">
         <is>
           <t>createdDateTime</t>
         </is>
       </c>
-      <c r="C138" s="4" t="inlineStr">
+      <c r="C138" s="2" t="inlineStr">
         <is>
           <t>Datetime</t>
         </is>
       </c>
-      <c r="D138" s="4" t="inlineStr">
+      <c r="D138" s="2" t="inlineStr">
         <is>
           <t>Canonical header from Inventory Transfers.xlsx</t>
         </is>
       </c>
-      <c r="E138" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F138" s="4" t="inlineStr"/>
-      <c r="G138" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H138" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>Stock Audit Report.txt:Posting Date for paired IM rows</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="4" t="inlineStr">
+      <c r="A139" s="2" t="inlineStr">
         <is>
           <t>InventoryTransfers</t>
         </is>
       </c>
-      <c r="B139" s="4" t="inlineStr">
+      <c r="B139" s="2" t="inlineStr">
         <is>
           <t>completedDateTime</t>
         </is>
       </c>
-      <c r="C139" s="4" t="inlineStr">
+      <c r="C139" s="2" t="inlineStr">
         <is>
           <t>Datetime</t>
         </is>
       </c>
-      <c r="D139" s="4" t="inlineStr">
+      <c r="D139" s="2" t="inlineStr">
         <is>
           <t>Canonical header from Inventory Transfers.xlsx</t>
         </is>
       </c>
-      <c r="E139" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F139" s="4" t="inlineStr"/>
-      <c r="G139" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H139" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>Stock Audit Report.txt:Posting Date for paired IM rows</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="4" t="inlineStr">
+      <c r="A140" s="2" t="inlineStr">
         <is>
           <t>InventoryTransfers</t>
         </is>
       </c>
-      <c r="B140" s="4" t="inlineStr">
+      <c r="B140" s="2" t="inlineStr">
         <is>
           <t>fromWarehouseId</t>
         </is>
       </c>
-      <c r="C140" s="4" t="inlineStr">
+      <c r="C140" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D140" s="4" t="inlineStr">
+      <c r="D140" s="2" t="inlineStr">
         <is>
           <t>Canonical header from Inventory Transfers.xlsx</t>
         </is>
       </c>
-      <c r="E140" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F140" s="4" t="inlineStr"/>
-      <c r="G140" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H140" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>Stock Audit Report.txt:Whse on negative IM quantity row</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="4" t="inlineStr">
+      <c r="A141" s="2" t="inlineStr">
         <is>
           <t>InventoryTransfers</t>
         </is>
       </c>
-      <c r="B141" s="4" t="inlineStr">
+      <c r="B141" s="2" t="inlineStr">
         <is>
           <t>toWarehouseId</t>
         </is>
       </c>
-      <c r="C141" s="4" t="inlineStr">
+      <c r="C141" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D141" s="4" t="inlineStr">
+      <c r="D141" s="2" t="inlineStr">
         <is>
           <t>Canonical header from Inventory Transfers.xlsx</t>
         </is>
       </c>
-      <c r="E141" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F141" s="4" t="inlineStr"/>
-      <c r="G141" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H141" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>Stock Audit Report.txt:Whse on positive IM quantity row</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="4" t="inlineStr">
+      <c r="A142" s="2" t="inlineStr">
         <is>
           <t>InventoryTransfers</t>
         </is>
       </c>
-      <c r="B142" s="4" t="inlineStr">
+      <c r="B142" s="2" t="inlineStr">
         <is>
           <t>demandStatus</t>
         </is>
       </c>
-      <c r="C142" s="4" t="inlineStr">
+      <c r="C142" s="2" t="inlineStr">
         <is>
           <t>Enum&lt;String&gt;</t>
         </is>
       </c>
-      <c r="D142" s="4" t="inlineStr">
+      <c r="D142" s="2" t="inlineStr">
         <is>
           <t>Canonical header from Inventory Transfers.xlsx</t>
         </is>
       </c>
-      <c r="E142" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F142" s="4" t="inlineStr"/>
-      <c r="G142" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H142" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>Business rule: Fulfilled for posted paired IM rows</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="4" t="inlineStr">
+      <c r="A143" s="2" t="inlineStr">
         <is>
           <t>InventoryTransfers</t>
         </is>
       </c>
-      <c r="B143" s="4" t="inlineStr">
+      <c r="B143" s="2" t="inlineStr">
         <is>
           <t>orderStatusIsClosed</t>
         </is>
       </c>
-      <c r="C143" s="4" t="inlineStr">
+      <c r="C143" s="2" t="inlineStr">
         <is>
           <t>Boolean</t>
         </is>
       </c>
-      <c r="D143" s="4" t="inlineStr">
+      <c r="D143" s="2" t="inlineStr">
         <is>
           <t>Canonical header from Inventory Transfers.xlsx</t>
         </is>
       </c>
-      <c r="E143" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F143" s="4" t="inlineStr"/>
-      <c r="G143" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H143" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>Business rule: Y for posted paired IM rows</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -20493,40 +20529,44 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="4" t="inlineStr">
+      <c r="A147" s="2" t="inlineStr">
         <is>
           <t>InventoryTransfers</t>
         </is>
       </c>
-      <c r="B147" s="4" t="inlineStr">
+      <c r="B147" s="2" t="inlineStr">
         <is>
           <t>quantity</t>
         </is>
       </c>
-      <c r="C147" s="4" t="inlineStr">
+      <c r="C147" s="2" t="inlineStr">
         <is>
           <t>Double</t>
         </is>
       </c>
-      <c r="D147" s="4" t="inlineStr">
+      <c r="D147" s="2" t="inlineStr">
         <is>
           <t>Canonical header from Inventory Transfers.xlsx</t>
         </is>
       </c>
-      <c r="E147" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F147" s="4" t="inlineStr"/>
-      <c r="G147" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H147" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>Stock Audit Report.txt:absolute IM Quantity for paired rows</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -22027,7 +22067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J210"/>
+  <dimension ref="A1:J200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -27845,7 +27885,7 @@
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>vendorId</t>
+          <t>vendorName</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
@@ -27866,7 +27906,7 @@
       </c>
       <c r="F116" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Vendors.vendorId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Vendors.vendorName?</t>
         </is>
       </c>
       <c r="G116" s="4" t="inlineStr">
@@ -27885,12 +27925,12 @@
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>vendorName</t>
+          <t>productClass</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>Vendors</t>
+          <t>Parts</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
@@ -27901,12 +27941,12 @@
       <c r="D117" s="4" t="inlineStr"/>
       <c r="E117" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Not available in checked source</t>
         </is>
       </c>
       <c r="F117" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Vendors.vendorName?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.productClass?</t>
         </is>
       </c>
       <c r="G117" s="4" t="inlineStr">
@@ -27918,19 +27958,19 @@
       <c r="I117" s="4" t="inlineStr"/>
       <c r="J117" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. Live SAP item master check found broad ItemGroups such as FUJITSU/ACER/CHOICE and generic ItemType/ItemClass/MaterialType values, not Planning V2 class/type semantics.</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>isActive</t>
+          <t>productType</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>Vendors</t>
+          <t>Parts</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
@@ -27941,12 +27981,12 @@
       <c r="D118" s="4" t="inlineStr"/>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Not available in checked source</t>
         </is>
       </c>
       <c r="F118" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Vendors.isActive?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.productType?</t>
         </is>
       </c>
       <c r="G118" s="4" t="inlineStr">
@@ -27958,14 +27998,14 @@
       <c r="I118" s="4" t="inlineStr"/>
       <c r="J118" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. Live SAP item master check found broad ItemGroups such as FUJITSU/ACER/CHOICE and generic ItemType/ItemClass/MaterialType values, not Planning V2 class/type semantics.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>productClass</t>
+          <t>costCategory</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
@@ -27981,12 +28021,12 @@
       <c r="D119" s="4" t="inlineStr"/>
       <c r="E119" s="4" t="inlineStr">
         <is>
-          <t>Not available in checked source</t>
+          <t>Investigate SAP first</t>
         </is>
       </c>
       <c r="F119" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.productClass?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.costCategory?</t>
         </is>
       </c>
       <c r="G119" s="4" t="inlineStr">
@@ -27998,14 +28038,14 @@
       <c r="I119" s="4" t="inlineStr"/>
       <c r="J119" s="4" t="inlineStr">
         <is>
-          <t>Left blank. Live SAP item master check found broad ItemGroups such as FUJITSU/ACER/CHOICE and generic ItemType/ItemClass/MaterialType values, not Planning V2 class/type semantics.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>productType</t>
+          <t>partType</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
@@ -28026,7 +28066,7 @@
       </c>
       <c r="F120" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.productType?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.partType?</t>
         </is>
       </c>
       <c r="G120" s="4" t="inlineStr">
@@ -28045,7 +28085,7 @@
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>costCategory</t>
+          <t>isKit</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
@@ -28066,7 +28106,7 @@
       </c>
       <c r="F121" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.costCategory?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.isKit?</t>
         </is>
       </c>
       <c r="G121" s="4" t="inlineStr">
@@ -28085,7 +28125,7 @@
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>partType</t>
+          <t>isCritical</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
@@ -28101,12 +28141,12 @@
       <c r="D122" s="4" t="inlineStr"/>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>Not available in checked source</t>
+          <t>Investigate SAP first</t>
         </is>
       </c>
       <c r="F122" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.partType?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.isCritical?</t>
         </is>
       </c>
       <c r="G122" s="4" t="inlineStr">
@@ -28118,19 +28158,19 @@
       <c r="I122" s="4" t="inlineStr"/>
       <c r="J122" s="4" t="inlineStr">
         <is>
-          <t>Left blank. Live SAP item master check found broad ItemGroups such as FUJITSU/ACER/CHOICE and generic ItemType/ItemClass/MaterialType values, not Planning V2 class/type semantics.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>isKit</t>
+          <t>externalAddressId</t>
         </is>
       </c>
       <c r="B123" s="4" t="inlineStr">
         <is>
-          <t>Parts</t>
+          <t>Addresses</t>
         </is>
       </c>
       <c r="C123" s="4" t="inlineStr">
@@ -28146,7 +28186,7 @@
       </c>
       <c r="F123" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isKit?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.externalAddressId?</t>
         </is>
       </c>
       <c r="G123" s="4" t="inlineStr">
@@ -28158,19 +28198,19 @@
       <c r="I123" s="4" t="inlineStr"/>
       <c r="J123" s="4" t="inlineStr">
         <is>
-          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t>isCritical</t>
+          <t>customerExternalId</t>
         </is>
       </c>
       <c r="B124" s="4" t="inlineStr">
         <is>
-          <t>Parts</t>
+          <t>Addresses</t>
         </is>
       </c>
       <c r="C124" s="4" t="inlineStr">
@@ -28186,7 +28226,7 @@
       </c>
       <c r="F124" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isCritical?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.customerExternalId?</t>
         </is>
       </c>
       <c r="G124" s="4" t="inlineStr">
@@ -28198,14 +28238,14 @@
       <c r="I124" s="4" t="inlineStr"/>
       <c r="J124" s="4" t="inlineStr">
         <is>
-          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
         <is>
-          <t>externalAddressId</t>
+          <t>6,0</t>
         </is>
       </c>
       <c r="B125" s="4" t="inlineStr">
@@ -28226,7 +28266,7 @@
       </c>
       <c r="F125" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.externalAddressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.6,0?</t>
         </is>
       </c>
       <c r="G125" s="4" t="inlineStr">
@@ -28245,7 +28285,7 @@
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
         <is>
-          <t>customerExternalId</t>
+          <t>addressLine2</t>
         </is>
       </c>
       <c r="B126" s="4" t="inlineStr">
@@ -28266,7 +28306,7 @@
       </c>
       <c r="F126" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.customerExternalId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.addressLine2?</t>
         </is>
       </c>
       <c r="G126" s="4" t="inlineStr">
@@ -28285,7 +28325,7 @@
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
         <is>
-          <t>6,0</t>
+          <t>addressLine3</t>
         </is>
       </c>
       <c r="B127" s="4" t="inlineStr">
@@ -28306,7 +28346,7 @@
       </c>
       <c r="F127" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.6,0?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.addressLine3?</t>
         </is>
       </c>
       <c r="G127" s="4" t="inlineStr">
@@ -28325,7 +28365,7 @@
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
         <is>
-          <t>addressLine2</t>
+          <t>city</t>
         </is>
       </c>
       <c r="B128" s="4" t="inlineStr">
@@ -28346,7 +28386,7 @@
       </c>
       <c r="F128" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.addressLine2?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.city?</t>
         </is>
       </c>
       <c r="G128" s="4" t="inlineStr">
@@ -28365,7 +28405,7 @@
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t>addressLine3</t>
+          <t>stateProvince</t>
         </is>
       </c>
       <c r="B129" s="4" t="inlineStr">
@@ -28386,7 +28426,7 @@
       </c>
       <c r="F129" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.addressLine3?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.stateProvince?</t>
         </is>
       </c>
       <c r="G129" s="4" t="inlineStr">
@@ -28405,7 +28445,7 @@
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>countryCode</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
@@ -28426,7 +28466,7 @@
       </c>
       <c r="F130" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.city?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.countryCode?</t>
         </is>
       </c>
       <c r="G130" s="4" t="inlineStr">
@@ -28445,7 +28485,7 @@
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>stateProvince</t>
+          <t>latitude</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
@@ -28466,7 +28506,7 @@
       </c>
       <c r="F131" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.stateProvince?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.latitude?</t>
         </is>
       </c>
       <c r="G131" s="4" t="inlineStr">
@@ -28485,7 +28525,7 @@
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>countryCode</t>
+          <t>longitude</t>
         </is>
       </c>
       <c r="B132" s="4" t="inlineStr">
@@ -28506,7 +28546,7 @@
       </c>
       <c r="F132" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.countryCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.longitude?</t>
         </is>
       </c>
       <c r="G132" s="4" t="inlineStr">
@@ -28525,7 +28565,7 @@
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
         <is>
-          <t>latitude</t>
+          <t>timeZone</t>
         </is>
       </c>
       <c r="B133" s="4" t="inlineStr">
@@ -28546,7 +28586,7 @@
       </c>
       <c r="F133" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.latitude?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.timeZone?</t>
         </is>
       </c>
       <c r="G133" s="4" t="inlineStr">
@@ -28565,7 +28605,7 @@
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
         <is>
-          <t>longitude</t>
+          <t>nodeId</t>
         </is>
       </c>
       <c r="B134" s="4" t="inlineStr">
@@ -28586,7 +28626,7 @@
       </c>
       <c r="F134" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.longitude?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.nodeId?</t>
         </is>
       </c>
       <c r="G134" s="4" t="inlineStr">
@@ -28605,12 +28645,12 @@
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
         <is>
-          <t>timeZone</t>
+          <t>partNumber</t>
         </is>
       </c>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t>Addresses</t>
+          <t>WarehouseStockOnHand</t>
         </is>
       </c>
       <c r="C135" s="4" t="inlineStr">
@@ -28626,7 +28666,7 @@
       </c>
       <c r="F135" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.timeZone?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseStockOnHand.partNumber?</t>
         </is>
       </c>
       <c r="G135" s="4" t="inlineStr">
@@ -28645,12 +28685,12 @@
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>nodeId</t>
+          <t>personId</t>
         </is>
       </c>
       <c r="B136" s="4" t="inlineStr">
         <is>
-          <t>Addresses</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C136" s="4" t="inlineStr">
@@ -28666,7 +28706,7 @@
       </c>
       <c r="F136" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.nodeId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.personId?</t>
         </is>
       </c>
       <c r="G136" s="4" t="inlineStr">
@@ -28685,7 +28725,7 @@
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
         <is>
-          <t>personId</t>
+          <t>role</t>
         </is>
       </c>
       <c r="B137" s="4" t="inlineStr">
@@ -28706,7 +28746,7 @@
       </c>
       <c r="F137" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.personId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.role?</t>
         </is>
       </c>
       <c r="G137" s="4" t="inlineStr">
@@ -28725,7 +28765,7 @@
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>addressId</t>
         </is>
       </c>
       <c r="B138" s="4" t="inlineStr">
@@ -28746,7 +28786,7 @@
       </c>
       <c r="F138" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.role?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.addressId?</t>
         </is>
       </c>
       <c r="G138" s="4" t="inlineStr">
@@ -28765,7 +28805,7 @@
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>addressId</t>
+          <t>nodeId</t>
         </is>
       </c>
       <c r="B139" s="4" t="inlineStr">
@@ -28786,7 +28826,7 @@
       </c>
       <c r="F139" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.addressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.nodeId?</t>
         </is>
       </c>
       <c r="G139" s="4" t="inlineStr">
@@ -28805,7 +28845,7 @@
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>nodeId</t>
+          <t>firstName</t>
         </is>
       </c>
       <c r="B140" s="4" t="inlineStr">
@@ -28826,7 +28866,7 @@
       </c>
       <c r="F140" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.nodeId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.firstName?</t>
         </is>
       </c>
       <c r="G140" s="4" t="inlineStr">
@@ -28845,7 +28885,7 @@
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
         <is>
-          <t>firstName</t>
+          <t>middleName</t>
         </is>
       </c>
       <c r="B141" s="4" t="inlineStr">
@@ -28866,7 +28906,7 @@
       </c>
       <c r="F141" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.firstName?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.middleName?</t>
         </is>
       </c>
       <c r="G141" s="4" t="inlineStr">
@@ -28885,7 +28925,7 @@
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>middleName</t>
+          <t>surname</t>
         </is>
       </c>
       <c r="B142" s="4" t="inlineStr">
@@ -28906,7 +28946,7 @@
       </c>
       <c r="F142" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.middleName?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.surname?</t>
         </is>
       </c>
       <c r="G142" s="4" t="inlineStr">
@@ -28925,7 +28965,7 @@
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>surname</t>
+          <t>isActive</t>
         </is>
       </c>
       <c r="B143" s="4" t="inlineStr">
@@ -28946,7 +28986,7 @@
       </c>
       <c r="F143" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.surname?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.isActive?</t>
         </is>
       </c>
       <c r="G143" s="4" t="inlineStr">
@@ -28965,7 +29005,7 @@
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>isActive</t>
+          <t>telephoneNumber</t>
         </is>
       </c>
       <c r="B144" s="4" t="inlineStr">
@@ -28986,7 +29026,7 @@
       </c>
       <c r="F144" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.isActive?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.telephoneNumber?</t>
         </is>
       </c>
       <c r="G144" s="4" t="inlineStr">
@@ -29005,7 +29045,7 @@
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>telephoneNumber</t>
+          <t>whs id</t>
         </is>
       </c>
       <c r="B145" s="4" t="inlineStr">
@@ -29026,7 +29066,7 @@
       </c>
       <c r="F145" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.telephoneNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.whs id?</t>
         </is>
       </c>
       <c r="G145" s="4" t="inlineStr">
@@ -29045,12 +29085,12 @@
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>whs id</t>
+          <t>resolvedDateTime</t>
         </is>
       </c>
       <c r="B146" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C146" s="4" t="inlineStr">
@@ -29066,7 +29106,7 @@
       </c>
       <c r="F146" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.whs id?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.resolvedDateTime?</t>
         </is>
       </c>
       <c r="G146" s="4" t="inlineStr">
@@ -29085,7 +29125,7 @@
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>OrderType</t>
+          <t>relCompanyId</t>
         </is>
       </c>
       <c r="B147" s="4" t="inlineStr">
@@ -29106,7 +29146,7 @@
       </c>
       <c r="F147" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.OrderType?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.relCompanyId?</t>
         </is>
       </c>
       <c r="G147" s="4" t="inlineStr">
@@ -29125,7 +29165,7 @@
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>resolvedDateTime</t>
+          <t>assignedPersonCode</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
@@ -29146,7 +29186,7 @@
       </c>
       <c r="F148" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.resolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.assignedPersonCode?</t>
         </is>
       </c>
       <c r="G148" s="4" t="inlineStr">
@@ -29165,12 +29205,12 @@
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>relCompanyId</t>
+          <t>orderNumber</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">
@@ -29186,7 +29226,7 @@
       </c>
       <c r="F149" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.relCompanyId?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.orderNumber?</t>
         </is>
       </c>
       <c r="G149" s="4" t="inlineStr">
@@ -29205,12 +29245,12 @@
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>assignedPersonCode</t>
+          <t>RequestID</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C150" s="4" t="inlineStr">
@@ -29226,7 +29266,7 @@
       </c>
       <c r="F150" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.assignedPersonCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.RequestID?</t>
         </is>
       </c>
       <c r="G150" s="4" t="inlineStr">
@@ -29245,7 +29285,7 @@
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>orderNumber</t>
+          <t>location</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
@@ -29266,7 +29306,7 @@
       </c>
       <c r="F151" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.orderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.location?</t>
         </is>
       </c>
       <c r="G151" s="4" t="inlineStr">
@@ -29285,7 +29325,7 @@
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>RequestID</t>
+          <t>eta</t>
         </is>
       </c>
       <c r="B152" s="4" t="inlineStr">
@@ -29306,7 +29346,7 @@
       </c>
       <c r="F152" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.RequestID?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.eta?</t>
         </is>
       </c>
       <c r="G152" s="4" t="inlineStr">
@@ -29325,7 +29365,7 @@
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>actualEta</t>
         </is>
       </c>
       <c r="B153" s="4" t="inlineStr">
@@ -29346,7 +29386,7 @@
       </c>
       <c r="F153" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.location?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualEta?</t>
         </is>
       </c>
       <c r="G153" s="4" t="inlineStr">
@@ -29365,7 +29405,7 @@
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>eta</t>
+          <t>actualResolveDateTime</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
@@ -29386,7 +29426,7 @@
       </c>
       <c r="F154" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.eta?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualResolveDateTime?</t>
         </is>
       </c>
       <c r="G154" s="4" t="inlineStr">
@@ -29405,7 +29445,7 @@
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>actualEta</t>
+          <t>recallDateTime</t>
         </is>
       </c>
       <c r="B155" s="4" t="inlineStr">
@@ -29426,7 +29466,7 @@
       </c>
       <c r="F155" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualEta?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.recallDateTime?</t>
         </is>
       </c>
       <c r="G155" s="4" t="inlineStr">
@@ -29445,7 +29485,7 @@
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>actualResolveDateTime</t>
+          <t>actualRecallDateTime</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
@@ -29466,7 +29506,7 @@
       </c>
       <c r="F156" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualResolveDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualRecallDateTime?</t>
         </is>
       </c>
       <c r="G156" s="4" t="inlineStr">
@@ -29485,7 +29525,7 @@
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>recallDateTime</t>
+          <t>slaEtaClock</t>
         </is>
       </c>
       <c r="B157" s="4" t="inlineStr">
@@ -29506,7 +29546,7 @@
       </c>
       <c r="F157" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.recallDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaClock?</t>
         </is>
       </c>
       <c r="G157" s="4" t="inlineStr">
@@ -29525,7 +29565,7 @@
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>actualRecallDateTime</t>
+          <t>slaResolveClock</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
@@ -29546,7 +29586,7 @@
       </c>
       <c r="F158" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualRecallDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveClock?</t>
         </is>
       </c>
       <c r="G158" s="4" t="inlineStr">
@@ -29565,7 +29605,7 @@
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>slaEtaClock</t>
+          <t>slaFailureCode</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
@@ -29586,7 +29626,7 @@
       </c>
       <c r="F159" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaClock?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaFailureCode?</t>
         </is>
       </c>
       <c r="G159" s="4" t="inlineStr">
@@ -29605,7 +29645,7 @@
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>slaResolveClock</t>
+          <t>slaEtaHit</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
@@ -29626,7 +29666,7 @@
       </c>
       <c r="F160" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveClock?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaHit?</t>
         </is>
       </c>
       <c r="G160" s="4" t="inlineStr">
@@ -29645,7 +29685,7 @@
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>slaFailureCode</t>
+          <t>slaResolveDateTime</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
@@ -29666,7 +29706,7 @@
       </c>
       <c r="F161" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaFailureCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveDateTime?</t>
         </is>
       </c>
       <c r="G161" s="4" t="inlineStr">
@@ -29685,12 +29725,12 @@
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>slaEtaHit</t>
+          <t>orderNumber</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C162" s="4" t="inlineStr">
@@ -29706,7 +29746,7 @@
       </c>
       <c r="F162" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaHit?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderNumber?</t>
         </is>
       </c>
       <c r="G162" s="4" t="inlineStr">
@@ -29725,12 +29765,12 @@
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>slaResolveDateTime</t>
+          <t>requestId</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C163" s="4" t="inlineStr">
@@ -29746,7 +29786,7 @@
       </c>
       <c r="F163" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.requestId?</t>
         </is>
       </c>
       <c r="G163" s="4" t="inlineStr">
@@ -29765,7 +29805,7 @@
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>orderNumber</t>
+          <t>customerCompanyCode</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
@@ -29786,7 +29826,7 @@
       </c>
       <c r="F164" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.customerCompanyCode?</t>
         </is>
       </c>
       <c r="G164" s="4" t="inlineStr">
@@ -29805,7 +29845,7 @@
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t>requestId</t>
+          <t>orderStatus</t>
         </is>
       </c>
       <c r="B165" s="4" t="inlineStr">
@@ -29826,7 +29866,7 @@
       </c>
       <c r="F165" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.requestId?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStatus?</t>
         </is>
       </c>
       <c r="G165" s="4" t="inlineStr">
@@ -29845,7 +29885,7 @@
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>customerCompanyCode</t>
+          <t>orderStartDatetime</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
@@ -29866,7 +29906,7 @@
       </c>
       <c r="F166" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.customerCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStartDatetime?</t>
         </is>
       </c>
       <c r="G166" s="4" t="inlineStr">
@@ -29885,7 +29925,7 @@
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>orderStatus</t>
+          <t>siteCompanyCode</t>
         </is>
       </c>
       <c r="B167" s="4" t="inlineStr">
@@ -29906,7 +29946,7 @@
       </c>
       <c r="F167" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.siteCompanyCode?</t>
         </is>
       </c>
       <c r="G167" s="4" t="inlineStr">
@@ -29925,7 +29965,7 @@
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>orderStartDatetime</t>
+          <t>repairType</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
@@ -29946,7 +29986,7 @@
       </c>
       <c r="F168" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStartDatetime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairType?</t>
         </is>
       </c>
       <c r="G168" s="4" t="inlineStr">
@@ -29965,7 +30005,7 @@
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>siteCompanyCode</t>
+          <t>partsOrderDateTime</t>
         </is>
       </c>
       <c r="B169" s="4" t="inlineStr">
@@ -29986,7 +30026,7 @@
       </c>
       <c r="F169" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.siteCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsOrderDateTime?</t>
         </is>
       </c>
       <c r="G169" s="4" t="inlineStr">
@@ -30005,7 +30045,7 @@
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>repairType</t>
+          <t>partsReceivedDateTime</t>
         </is>
       </c>
       <c r="B170" s="4" t="inlineStr">
@@ -30026,7 +30066,7 @@
       </c>
       <c r="F170" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairType?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsReceivedDateTime?</t>
         </is>
       </c>
       <c r="G170" s="4" t="inlineStr">
@@ -30045,7 +30085,7 @@
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>partsOrderDateTime</t>
+          <t>repairCode</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
@@ -30066,7 +30106,7 @@
       </c>
       <c r="F171" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsOrderDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCode?</t>
         </is>
       </c>
       <c r="G171" s="4" t="inlineStr">
@@ -30085,7 +30125,7 @@
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>partsReceivedDateTime</t>
+          <t>repairCompany</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
@@ -30106,7 +30146,7 @@
       </c>
       <c r="F172" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsReceivedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCompany?</t>
         </is>
       </c>
       <c r="G172" s="4" t="inlineStr">
@@ -30125,7 +30165,7 @@
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>repairCode</t>
+          <t>raStatus</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
@@ -30146,7 +30186,7 @@
       </c>
       <c r="F173" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.raStatus?</t>
         </is>
       </c>
       <c r="G173" s="4" t="inlineStr">
@@ -30165,7 +30205,7 @@
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>repairCompany</t>
+          <t>Warehouse</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
@@ -30186,7 +30226,7 @@
       </c>
       <c r="F174" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCompany?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.Warehouse?</t>
         </is>
       </c>
       <c r="G174" s="4" t="inlineStr">
@@ -30205,7 +30245,7 @@
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>raStatus</t>
+          <t>assignedPerson</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
@@ -30226,7 +30266,7 @@
       </c>
       <c r="F175" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.raStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.assignedPerson?</t>
         </is>
       </c>
       <c r="G175" s="4" t="inlineStr">
@@ -30245,7 +30285,7 @@
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>Warehouse</t>
+          <t>resolvedDateTime</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
@@ -30266,7 +30306,7 @@
       </c>
       <c r="F176" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.Warehouse?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.resolvedDateTime?</t>
         </is>
       </c>
       <c r="G176" s="4" t="inlineStr">
@@ -30285,7 +30325,7 @@
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>assignedPerson</t>
+          <t>serialNumber</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
@@ -30306,7 +30346,7 @@
       </c>
       <c r="F177" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.assignedPerson?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.serialNumber?</t>
         </is>
       </c>
       <c r="G177" s="4" t="inlineStr">
@@ -30325,7 +30365,7 @@
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>resolvedDateTime</t>
+          <t>quantityUsed</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
@@ -30346,7 +30386,7 @@
       </c>
       <c r="F178" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.resolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.quantityUsed?</t>
         </is>
       </c>
       <c r="G178" s="4" t="inlineStr">
@@ -30365,7 +30405,7 @@
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>serialNumber</t>
+          <t>deviceSerialNumber</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
@@ -30386,7 +30426,7 @@
       </c>
       <c r="F179" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.serialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.deviceSerialNumber?</t>
         </is>
       </c>
       <c r="G179" s="4" t="inlineStr">
@@ -30405,7 +30445,7 @@
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>quantityUsed</t>
+          <t>orderedPartId</t>
         </is>
       </c>
       <c r="B180" s="4" t="inlineStr">
@@ -30426,7 +30466,7 @@
       </c>
       <c r="F180" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.quantityUsed?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderedPartId?</t>
         </is>
       </c>
       <c r="G180" s="4" t="inlineStr">
@@ -30445,7 +30485,7 @@
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>deviceSerialNumber</t>
+          <t>actualPartId</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
@@ -30466,7 +30506,7 @@
       </c>
       <c r="F181" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.deviceSerialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.actualPartId?</t>
         </is>
       </c>
       <c r="G181" s="4" t="inlineStr">
@@ -30485,12 +30525,12 @@
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>orderedPartId</t>
+          <t>partCode</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C182" s="4" t="inlineStr">
@@ -30506,7 +30546,7 @@
       </c>
       <c r="F182" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderedPartId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
         </is>
       </c>
       <c r="G182" s="4" t="inlineStr">
@@ -30525,12 +30565,12 @@
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>actualPartId</t>
+          <t>modelCode</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C183" s="4" t="inlineStr">
@@ -30546,7 +30586,7 @@
       </c>
       <c r="F183" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.actualPartId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
         </is>
       </c>
       <c r="G183" s="4" t="inlineStr">
@@ -30565,7 +30605,7 @@
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>partCode</t>
+          <t>modelDescription</t>
         </is>
       </c>
       <c r="B184" s="4" t="inlineStr">
@@ -30586,7 +30626,7 @@
       </c>
       <c r="F184" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
         </is>
       </c>
       <c r="G184" s="4" t="inlineStr">
@@ -30605,12 +30645,12 @@
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>modelCode</t>
+          <t>movementType</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C185" s="4" t="inlineStr">
@@ -30626,7 +30666,7 @@
       </c>
       <c r="F185" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
         </is>
       </c>
       <c r="G185" s="4" t="inlineStr">
@@ -30645,12 +30685,12 @@
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>modelDescription</t>
+          <t>addressId</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C186" s="4" t="inlineStr">
@@ -30666,7 +30706,7 @@
       </c>
       <c r="F186" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
         </is>
       </c>
       <c r="G186" s="4" t="inlineStr">
@@ -30685,7 +30725,7 @@
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>inventoryTransferImoId</t>
+          <t>Bpart</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
@@ -30706,7 +30746,7 @@
       </c>
       <c r="F187" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.inventoryTransferImoId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.Bpart?</t>
         </is>
       </c>
       <c r="G187" s="4" t="inlineStr">
@@ -30725,7 +30765,7 @@
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>createdDateTime</t>
+          <t>shipListCode</t>
         </is>
       </c>
       <c r="B188" s="4" t="inlineStr">
@@ -30746,7 +30786,7 @@
       </c>
       <c r="F188" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.createdDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
         </is>
       </c>
       <c r="G188" s="4" t="inlineStr">
@@ -30763,54 +30803,54 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="4" t="inlineStr">
-        <is>
-          <t>completedDateTime</t>
-        </is>
-      </c>
-      <c r="B189" s="4" t="inlineStr">
-        <is>
-          <t>InventoryTransfers</t>
-        </is>
-      </c>
-      <c r="C189" s="4" t="inlineStr">
+      <c r="A189" s="3" t="inlineStr">
+        <is>
+          <t>demandStatus</t>
+        </is>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>PurchaseOrders</t>
+        </is>
+      </c>
+      <c r="C189" s="3" t="inlineStr">
         <is>
           <t>Planning V2 template</t>
         </is>
       </c>
-      <c r="D189" s="4" t="inlineStr"/>
-      <c r="E189" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F189" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.completedDateTime?</t>
-        </is>
-      </c>
-      <c r="G189" s="4" t="inlineStr">
+      <c r="D189" s="3" t="inlineStr"/>
+      <c r="E189" s="3" t="inlineStr">
+        <is>
+          <t>Review required</t>
+        </is>
+      </c>
+      <c r="F189" s="3" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
+        </is>
+      </c>
+      <c r="G189" s="3" t="inlineStr">
         <is>
           <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
         </is>
       </c>
-      <c r="H189" s="4" t="inlineStr"/>
-      <c r="I189" s="4" t="inlineStr"/>
-      <c r="J189" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="H189" s="3" t="inlineStr"/>
+      <c r="I189" s="3" t="inlineStr"/>
+      <c r="J189" s="3" t="inlineStr">
+        <is>
+          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.NumAtCard and part/SPL Master evidence also matches.</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>fromWarehouseId</t>
+          <t>partType</t>
         </is>
       </c>
       <c r="B190" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C190" s="4" t="inlineStr">
@@ -30826,7 +30866,7 @@
       </c>
       <c r="F190" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.fromWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.partType?</t>
         </is>
       </c>
       <c r="G190" s="4" t="inlineStr">
@@ -30845,12 +30885,12 @@
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>toWarehouseId</t>
+          <t>partTypeDescription</t>
         </is>
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr">
@@ -30866,7 +30906,7 @@
       </c>
       <c r="F191" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.toWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeDescription?</t>
         </is>
       </c>
       <c r="G191" s="4" t="inlineStr">
@@ -30885,12 +30925,12 @@
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>demandStatus</t>
+          <t>isReworkable</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C192" s="4" t="inlineStr">
@@ -30906,7 +30946,7 @@
       </c>
       <c r="F192" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.demandStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.isReworkable?</t>
         </is>
       </c>
       <c r="G192" s="4" t="inlineStr">
@@ -30925,12 +30965,12 @@
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>orderStatusIsClosed</t>
+          <t>partNumber</t>
         </is>
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C193" s="4" t="inlineStr">
@@ -30946,7 +30986,7 @@
       </c>
       <c r="F193" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.orderStatusIsClosed?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
         </is>
       </c>
       <c r="G193" s="4" t="inlineStr">
@@ -30965,12 +31005,12 @@
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>movementType</t>
+          <t>unitOfMeasure</t>
         </is>
       </c>
       <c r="B194" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C194" s="4" t="inlineStr">
@@ -30986,7 +31026,7 @@
       </c>
       <c r="F194" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
         </is>
       </c>
       <c r="G194" s="4" t="inlineStr">
@@ -31005,12 +31045,12 @@
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>addressId</t>
+          <t>yield</t>
         </is>
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
@@ -31026,7 +31066,7 @@
       </c>
       <c r="F195" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
         </is>
       </c>
       <c r="G195" s="4" t="inlineStr">
@@ -31045,12 +31085,12 @@
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>Bpart</t>
+          <t>Secondary TO</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C196" s="4" t="inlineStr">
@@ -31066,7 +31106,7 @@
       </c>
       <c r="F196" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.Bpart?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary TO?</t>
         </is>
       </c>
       <c r="G196" s="4" t="inlineStr">
@@ -31085,12 +31125,12 @@
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>Secondary FROM</t>
         </is>
       </c>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr">
@@ -31106,7 +31146,7 @@
       </c>
       <c r="F197" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.quantity?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary FROM?</t>
         </is>
       </c>
       <c r="G197" s="4" t="inlineStr">
@@ -31125,12 +31165,12 @@
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>shipListCode</t>
+          <t>Cross TO</t>
         </is>
       </c>
       <c r="B198" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C198" s="4" t="inlineStr">
@@ -31146,7 +31186,7 @@
       </c>
       <c r="F198" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross TO?</t>
         </is>
       </c>
       <c r="G198" s="4" t="inlineStr">
@@ -31163,54 +31203,54 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="3" t="inlineStr">
-        <is>
-          <t>demandStatus</t>
-        </is>
-      </c>
-      <c r="B199" s="3" t="inlineStr">
-        <is>
-          <t>PurchaseOrders</t>
-        </is>
-      </c>
-      <c r="C199" s="3" t="inlineStr">
+      <c r="A199" s="4" t="inlineStr">
+        <is>
+          <t>Cross FROM</t>
+        </is>
+      </c>
+      <c r="B199" s="4" t="inlineStr">
+        <is>
+          <t>WarehouseExclusions</t>
+        </is>
+      </c>
+      <c r="C199" s="4" t="inlineStr">
         <is>
           <t>Planning V2 template</t>
         </is>
       </c>
-      <c r="D199" s="3" t="inlineStr"/>
-      <c r="E199" s="3" t="inlineStr">
-        <is>
-          <t>Review required</t>
-        </is>
-      </c>
-      <c r="F199" s="3" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
-        </is>
-      </c>
-      <c r="G199" s="3" t="inlineStr">
+      <c r="D199" s="4" t="inlineStr"/>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>Investigate SAP first</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="inlineStr">
+        <is>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross FROM?</t>
+        </is>
+      </c>
+      <c r="G199" s="4" t="inlineStr">
         <is>
           <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
         </is>
       </c>
-      <c r="H199" s="3" t="inlineStr"/>
-      <c r="I199" s="3" t="inlineStr"/>
-      <c r="J199" s="3" t="inlineStr">
-        <is>
-          <t>Conditional HelpDesk enrichment. Use ReplenishStatus only when PurchaseOrder filename stem matches SAP OPOR.NumAtCard and part/SPL Master evidence also matches.</t>
+      <c r="H199" s="4" t="inlineStr"/>
+      <c r="I199" s="4" t="inlineStr"/>
+      <c r="J199" s="4" t="inlineStr">
+        <is>
+          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>partType</t>
+          <t>Primary TO</t>
         </is>
       </c>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C200" s="4" t="inlineStr">
@@ -31226,7 +31266,7 @@
       </c>
       <c r="F200" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partType?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Primary TO?</t>
         </is>
       </c>
       <c r="G200" s="4" t="inlineStr">
@@ -31242,408 +31282,8 @@
         </is>
       </c>
     </row>
-    <row r="201">
-      <c r="A201" s="4" t="inlineStr">
-        <is>
-          <t>partTypeDescription</t>
-        </is>
-      </c>
-      <c r="B201" s="4" t="inlineStr">
-        <is>
-          <t>PartTypes</t>
-        </is>
-      </c>
-      <c r="C201" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D201" s="4" t="inlineStr"/>
-      <c r="E201" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F201" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeDescription?</t>
-        </is>
-      </c>
-      <c r="G201" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H201" s="4" t="inlineStr"/>
-      <c r="I201" s="4" t="inlineStr"/>
-      <c r="J201" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" s="4" t="inlineStr">
-        <is>
-          <t>isReworkable</t>
-        </is>
-      </c>
-      <c r="B202" s="4" t="inlineStr">
-        <is>
-          <t>PartTypes</t>
-        </is>
-      </c>
-      <c r="C202" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D202" s="4" t="inlineStr"/>
-      <c r="E202" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F202" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.isReworkable?</t>
-        </is>
-      </c>
-      <c r="G202" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H202" s="4" t="inlineStr"/>
-      <c r="I202" s="4" t="inlineStr"/>
-      <c r="J202" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" s="4" t="inlineStr">
-        <is>
-          <t>partNumber</t>
-        </is>
-      </c>
-      <c r="B203" s="4" t="inlineStr">
-        <is>
-          <t>Yields</t>
-        </is>
-      </c>
-      <c r="C203" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D203" s="4" t="inlineStr"/>
-      <c r="E203" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F203" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
-        </is>
-      </c>
-      <c r="G203" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H203" s="4" t="inlineStr"/>
-      <c r="I203" s="4" t="inlineStr"/>
-      <c r="J203" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" s="4" t="inlineStr">
-        <is>
-          <t>unitOfMeasure</t>
-        </is>
-      </c>
-      <c r="B204" s="4" t="inlineStr">
-        <is>
-          <t>Yields</t>
-        </is>
-      </c>
-      <c r="C204" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D204" s="4" t="inlineStr"/>
-      <c r="E204" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F204" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
-        </is>
-      </c>
-      <c r="G204" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H204" s="4" t="inlineStr"/>
-      <c r="I204" s="4" t="inlineStr"/>
-      <c r="J204" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" s="4" t="inlineStr">
-        <is>
-          <t>yield</t>
-        </is>
-      </c>
-      <c r="B205" s="4" t="inlineStr">
-        <is>
-          <t>Yields</t>
-        </is>
-      </c>
-      <c r="C205" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D205" s="4" t="inlineStr"/>
-      <c r="E205" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F205" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
-        </is>
-      </c>
-      <c r="G205" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H205" s="4" t="inlineStr"/>
-      <c r="I205" s="4" t="inlineStr"/>
-      <c r="J205" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" s="4" t="inlineStr">
-        <is>
-          <t>Secondary TO</t>
-        </is>
-      </c>
-      <c r="B206" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C206" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D206" s="4" t="inlineStr"/>
-      <c r="E206" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F206" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary TO?</t>
-        </is>
-      </c>
-      <c r="G206" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H206" s="4" t="inlineStr"/>
-      <c r="I206" s="4" t="inlineStr"/>
-      <c r="J206" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" s="4" t="inlineStr">
-        <is>
-          <t>Secondary FROM</t>
-        </is>
-      </c>
-      <c r="B207" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C207" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D207" s="4" t="inlineStr"/>
-      <c r="E207" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F207" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Secondary FROM?</t>
-        </is>
-      </c>
-      <c r="G207" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H207" s="4" t="inlineStr"/>
-      <c r="I207" s="4" t="inlineStr"/>
-      <c r="J207" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" s="4" t="inlineStr">
-        <is>
-          <t>Cross TO</t>
-        </is>
-      </c>
-      <c r="B208" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C208" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D208" s="4" t="inlineStr"/>
-      <c r="E208" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F208" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross TO?</t>
-        </is>
-      </c>
-      <c r="G208" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H208" s="4" t="inlineStr"/>
-      <c r="I208" s="4" t="inlineStr"/>
-      <c r="J208" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" s="4" t="inlineStr">
-        <is>
-          <t>Cross FROM</t>
-        </is>
-      </c>
-      <c r="B209" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C209" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D209" s="4" t="inlineStr"/>
-      <c r="E209" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F209" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Cross FROM?</t>
-        </is>
-      </c>
-      <c r="G209" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H209" s="4" t="inlineStr"/>
-      <c r="I209" s="4" t="inlineStr"/>
-      <c r="J209" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" s="4" t="inlineStr">
-        <is>
-          <t>Primary TO</t>
-        </is>
-      </c>
-      <c r="B210" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C210" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D210" s="4" t="inlineStr"/>
-      <c r="E210" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F210" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.Primary TO?</t>
-        </is>
-      </c>
-      <c r="G210" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H210" s="4" t="inlineStr"/>
-      <c r="I210" s="4" t="inlineStr"/>
-      <c r="J210" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J210"/>
+  <autoFilter ref="A1:J200"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -32095,29 +31735,29 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Vendors</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Vendors.csv</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Pending/header only</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>vendorId, vendorName, isActive</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>vendorId; vendorName; isActive</t>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>vendorName</t>
         </is>
       </c>
     </row>
@@ -32199,27 +31839,31 @@
       <c r="E21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>WarehouseStockOnHand</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>WarehouseStockOnHand.csv</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>partNumber, warehouseCode, quantityAllocated, quantityOnHand, quantityInbound, uniqueId</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>partNumber</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -32271,7 +31915,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>OrderType; resolvedDateTime; relCompanyId; assignedPersonCode</t>
+          <t>resolvedDateTime; relCompanyId; assignedPersonCode</t>
         </is>
       </c>
     </row>
@@ -32380,29 +32024,29 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>InventoryTransfers</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>InventoryTransfers.csv</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Pending/header only</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>inventoryTransferImoId, createdDateTime, completedDateTime, fromWarehouseId, toWarehouseId, demandStatus, orderStatusIsClosed, movementType, addressId, Bpart, quantity, shipListCode</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>inventoryTransferImoId; createdDateTime; completedDateTime; fromWarehouseId; toWarehouseId; demandStatus; orderStatusIsClosed; movementType; addressId; Bpart; quantity; shipListCode</t>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>movementType; addressId; Bpart; shipListCode</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Altsgen part type enrichment
</commit_message>
<xml_diff>
--- a/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
+++ b/docs/field-map/CoCre8_PlanningV2_Field_Map.xlsx
@@ -20978,70 +20978,78 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="4" t="inlineStr">
+      <c r="A161" s="2" t="inlineStr">
         <is>
           <t>PartTypes</t>
         </is>
       </c>
-      <c r="B161" s="4" t="inlineStr">
+      <c r="B161" s="2" t="inlineStr">
         <is>
           <t>partType</t>
         </is>
       </c>
-      <c r="C161" s="4" t="inlineStr"/>
-      <c r="D161" s="4" t="inlineStr">
+      <c r="C161" s="2" t="inlineStr"/>
+      <c r="D161" s="2" t="inlineStr">
         <is>
           <t>Canonical header from partTypes.xlsx</t>
         </is>
       </c>
-      <c r="E161" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F161" s="4" t="inlineStr"/>
-      <c r="G161" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H161" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E161" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F161" s="2" t="inlineStr">
+        <is>
+          <t>Hosted Altsgen batch API:commodity_type for CoCre8 parts</t>
+        </is>
+      </c>
+      <c r="G161" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H161" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="4" t="inlineStr">
+      <c r="A162" s="2" t="inlineStr">
         <is>
           <t>PartTypes</t>
         </is>
       </c>
-      <c r="B162" s="4" t="inlineStr">
+      <c r="B162" s="2" t="inlineStr">
         <is>
           <t>partTypeDescription</t>
         </is>
       </c>
-      <c r="C162" s="4" t="inlineStr"/>
-      <c r="D162" s="4" t="inlineStr">
+      <c r="C162" s="2" t="inlineStr"/>
+      <c r="D162" s="2" t="inlineStr">
         <is>
           <t>Canonical header from partTypes.xlsx</t>
         </is>
       </c>
-      <c r="E162" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F162" s="4" t="inlineStr"/>
-      <c r="G162" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H162" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>Hosted Altsgen batch API:spec_summary.description or humanized commodity_type</t>
+        </is>
+      </c>
+      <c r="G162" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H162" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -21948,7 +21956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J153"/>
+  <dimension ref="A1:J151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -29166,7 +29174,7 @@
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>partType</t>
+          <t>isReworkable</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
@@ -29187,7 +29195,7 @@
       </c>
       <c r="F151" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partType?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.isReworkable?</t>
         </is>
       </c>
       <c r="G151" s="4" t="inlineStr">
@@ -29198,86 +29206,6 @@
       <c r="H151" s="4" t="inlineStr"/>
       <c r="I151" s="4" t="inlineStr"/>
       <c r="J151" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="4" t="inlineStr">
-        <is>
-          <t>partTypeDescription</t>
-        </is>
-      </c>
-      <c r="B152" s="4" t="inlineStr">
-        <is>
-          <t>PartTypes</t>
-        </is>
-      </c>
-      <c r="C152" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D152" s="4" t="inlineStr"/>
-      <c r="E152" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F152" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeDescription?</t>
-        </is>
-      </c>
-      <c r="G152" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H152" s="4" t="inlineStr"/>
-      <c r="I152" s="4" t="inlineStr"/>
-      <c r="J152" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="4" t="inlineStr">
-        <is>
-          <t>isReworkable</t>
-        </is>
-      </c>
-      <c r="B153" s="4" t="inlineStr">
-        <is>
-          <t>PartTypes</t>
-        </is>
-      </c>
-      <c r="C153" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D153" s="4" t="inlineStr"/>
-      <c r="E153" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F153" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.isReworkable?</t>
-        </is>
-      </c>
-      <c r="G153" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="H153" s="4" t="inlineStr"/>
-      <c r="I153" s="4" t="inlineStr"/>
-      <c r="J153" s="4" t="inlineStr">
         <is>
           <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
         </is>
@@ -30075,29 +30003,29 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>PartTypes</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>PartTypes.csv</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Pending/header only</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>partType, partTypeDescription, isReworkable</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>partType; partTypeDescription; isReworkable</t>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>isReworkable</t>
         </is>
       </c>
     </row>

</xml_diff>